<commit_message>
Implemented PID and DriveController
</commit_message>
<xml_diff>
--- a/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
+++ b/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_Software\electrical_hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC50C2D5-55A5-427D-A053-BD29FB099B66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFE2FBE8-47B0-4669-9FD4-62BD20041242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2370" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Layout" sheetId="1" r:id="rId1"/>
@@ -926,15 +926,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1001,7 +992,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1014,9 +1004,6 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1029,9 +1016,6 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1044,6 +1028,15 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1080,15 +1073,22 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1372,737 +1372,740 @@
   <dimension ref="B2:S25"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
+    <col min="2" max="2" width="4.19921875" customWidth="1"/>
     <col min="3" max="3" width="6.1328125" customWidth="1"/>
     <col min="4" max="4" width="3.59765625" customWidth="1"/>
     <col min="5" max="16" width="13.19921875" customWidth="1"/>
     <col min="17" max="17" width="3.796875" customWidth="1"/>
+    <col min="18" max="18" width="3.3984375" customWidth="1"/>
+    <col min="19" max="19" width="3.265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:19" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="83"/>
-      <c r="I2" s="83"/>
-      <c r="J2" s="83"/>
-      <c r="K2" s="83"/>
-      <c r="L2" s="83"/>
-      <c r="M2" s="83"/>
-      <c r="N2" s="83"/>
-      <c r="O2" s="83"/>
-      <c r="P2" s="83"/>
-      <c r="Q2" s="83"/>
-      <c r="R2" s="83"/>
-      <c r="S2" s="83"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
+      <c r="Q2" s="59"/>
+      <c r="R2" s="59"/>
+      <c r="S2" s="59"/>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B3" s="9"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="11"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
+      <c r="J3" s="83"/>
+      <c r="K3" s="83"/>
+      <c r="L3" s="83"/>
+      <c r="M3" s="83"/>
+      <c r="N3" s="83"/>
+      <c r="O3" s="83"/>
+      <c r="P3" s="83"/>
+      <c r="Q3" s="83"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="79"/>
     </row>
     <row r="4" spans="2:19" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B4" s="12"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="65" t="s">
+      <c r="B4" s="72"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="53" t="s">
         <v>102</v>
       </c>
-      <c r="F4" s="66" t="s">
+      <c r="F4" s="54" t="s">
         <v>103</v>
       </c>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="54"/>
-      <c r="O4" s="54"/>
-      <c r="P4" s="66" t="s">
+      <c r="G4" s="82"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="82"/>
+      <c r="J4" s="82"/>
+      <c r="K4" s="82"/>
+      <c r="L4" s="82"/>
+      <c r="M4" s="82"/>
+      <c r="N4" s="82"/>
+      <c r="O4" s="82"/>
+      <c r="P4" s="54" t="s">
         <v>108</v>
       </c>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="14"/>
+      <c r="Q4" s="73"/>
+      <c r="R4" s="73"/>
+      <c r="S4" s="74"/>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B5" s="12"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="55" t="s">
+      <c r="B5" s="72"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="55" t="s">
+      <c r="F5" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="55" t="s">
+      <c r="G5" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="55" t="s">
+      <c r="H5" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="55" t="s">
+      <c r="I5" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="55" t="s">
+      <c r="J5" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="K5" s="55" t="s">
+      <c r="K5" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="L5" s="55" t="s">
+      <c r="L5" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="M5" s="55" t="s">
+      <c r="M5" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="N5" s="55" t="s">
+      <c r="N5" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="O5" s="55" t="s">
+      <c r="O5" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="P5" s="55" t="s">
+      <c r="P5" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="13"/>
-      <c r="S5" s="14"/>
+      <c r="Q5" s="79"/>
+      <c r="R5" s="73"/>
+      <c r="S5" s="74"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B6" s="12"/>
-      <c r="C6" s="22" t="s">
+      <c r="B6" s="72"/>
+      <c r="C6" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="81" t="s">
+      <c r="E6" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="81"/>
-      <c r="G6" s="81"/>
-      <c r="H6" s="81"/>
-      <c r="I6" s="81"/>
-      <c r="J6" s="81"/>
-      <c r="K6" s="81"/>
-      <c r="L6" s="81"/>
-      <c r="M6" s="81"/>
-      <c r="N6" s="81"/>
-      <c r="O6" s="81"/>
-      <c r="P6" s="81"/>
-      <c r="Q6" s="19" t="s">
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="57"/>
+      <c r="J6" s="57"/>
+      <c r="K6" s="57"/>
+      <c r="L6" s="57"/>
+      <c r="M6" s="57"/>
+      <c r="N6" s="57"/>
+      <c r="O6" s="57"/>
+      <c r="P6" s="57"/>
+      <c r="Q6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="R6" s="13"/>
-      <c r="S6" s="14"/>
+      <c r="R6" s="73"/>
+      <c r="S6" s="74"/>
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B7" s="12"/>
-      <c r="C7" s="23" t="s">
+      <c r="B7" s="72"/>
+      <c r="C7" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="81"/>
-      <c r="F7" s="81"/>
-      <c r="G7" s="81"/>
-      <c r="H7" s="81"/>
-      <c r="I7" s="81"/>
-      <c r="J7" s="81"/>
-      <c r="K7" s="81"/>
-      <c r="L7" s="81"/>
-      <c r="M7" s="81"/>
-      <c r="N7" s="81"/>
-      <c r="O7" s="81"/>
-      <c r="P7" s="81"/>
-      <c r="Q7" s="19" t="s">
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="57"/>
+      <c r="H7" s="57"/>
+      <c r="I7" s="57"/>
+      <c r="J7" s="57"/>
+      <c r="K7" s="57"/>
+      <c r="L7" s="57"/>
+      <c r="M7" s="57"/>
+      <c r="N7" s="57"/>
+      <c r="O7" s="57"/>
+      <c r="P7" s="57"/>
+      <c r="Q7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="R7" s="13"/>
-      <c r="S7" s="14"/>
+      <c r="R7" s="73"/>
+      <c r="S7" s="74"/>
     </row>
     <row r="8" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="56" t="s">
+      <c r="B8" s="72"/>
+      <c r="C8" s="73"/>
+      <c r="D8" s="75"/>
+      <c r="E8" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="F8" s="56" t="s">
+      <c r="F8" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="G8" s="56" t="s">
+      <c r="G8" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="H8" s="56" t="s">
+      <c r="H8" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="I8" s="56" t="s">
+      <c r="I8" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="J8" s="56" t="s">
+      <c r="J8" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="K8" s="56" t="s">
+      <c r="K8" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="L8" s="56" t="s">
+      <c r="L8" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="M8" s="56" t="s">
+      <c r="M8" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="N8" s="56" t="s">
+      <c r="N8" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="O8" s="56" t="s">
+      <c r="O8" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="P8" s="56" t="s">
+      <c r="P8" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="Q8" s="17"/>
-      <c r="R8" s="13"/>
-      <c r="S8" s="14"/>
+      <c r="Q8" s="77"/>
+      <c r="R8" s="73"/>
+      <c r="S8" s="74"/>
     </row>
     <row r="9" spans="2:19" ht="38.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="12"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="67" t="s">
+      <c r="B9" s="72"/>
+      <c r="C9" s="73"/>
+      <c r="D9" s="73"/>
+      <c r="E9" s="55" t="s">
         <v>104</v>
       </c>
-      <c r="F9" s="68" t="s">
+      <c r="F9" s="56" t="s">
         <v>105</v>
       </c>
-      <c r="G9" s="57" t="s">
+      <c r="G9" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="58" t="s">
+      <c r="H9" s="48" t="s">
         <v>32</v>
       </c>
-      <c r="I9" s="57" t="s">
+      <c r="I9" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="58" t="s">
+      <c r="J9" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="K9" s="57" t="s">
+      <c r="K9" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="L9" s="58" t="s">
+      <c r="L9" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="M9" s="57" t="s">
+      <c r="M9" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="N9" s="58" t="s">
+      <c r="N9" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="O9" s="59"/>
-      <c r="P9" s="59"/>
-      <c r="Q9" s="13"/>
-      <c r="R9" s="13"/>
-      <c r="S9" s="14"/>
+      <c r="O9" s="78"/>
+      <c r="P9" s="78"/>
+      <c r="Q9" s="73"/>
+      <c r="R9" s="73"/>
+      <c r="S9" s="74"/>
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="13"/>
-      <c r="R10" s="13"/>
-      <c r="S10" s="14"/>
+      <c r="B10" s="72"/>
+      <c r="C10" s="73"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="73"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="73"/>
+      <c r="H10" s="73"/>
+      <c r="I10" s="73"/>
+      <c r="J10" s="73"/>
+      <c r="K10" s="73"/>
+      <c r="L10" s="73"/>
+      <c r="M10" s="73"/>
+      <c r="N10" s="73"/>
+      <c r="O10" s="73"/>
+      <c r="P10" s="73"/>
+      <c r="Q10" s="73"/>
+      <c r="R10" s="73"/>
+      <c r="S10" s="74"/>
     </row>
     <row r="11" spans="2:19" ht="29.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B11" s="12"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
-      <c r="I11" s="54"/>
-      <c r="J11" s="54"/>
-      <c r="K11" s="54"/>
-      <c r="L11" s="54"/>
-      <c r="M11" s="54"/>
-      <c r="N11" s="54"/>
-      <c r="O11" s="54"/>
-      <c r="P11" s="54"/>
-      <c r="Q11" s="13"/>
-      <c r="R11" s="13"/>
-      <c r="S11" s="14"/>
+      <c r="B11" s="72"/>
+      <c r="C11" s="73"/>
+      <c r="D11" s="73"/>
+      <c r="E11" s="82"/>
+      <c r="F11" s="82"/>
+      <c r="G11" s="82"/>
+      <c r="H11" s="82"/>
+      <c r="I11" s="82"/>
+      <c r="J11" s="82"/>
+      <c r="K11" s="82"/>
+      <c r="L11" s="82"/>
+      <c r="M11" s="82"/>
+      <c r="N11" s="82"/>
+      <c r="O11" s="82"/>
+      <c r="P11" s="82"/>
+      <c r="Q11" s="73"/>
+      <c r="R11" s="73"/>
+      <c r="S11" s="74"/>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B12" s="12"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="60" t="s">
+      <c r="B12" s="72"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="60" t="s">
+      <c r="F12" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="60" t="s">
+      <c r="G12" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="60" t="s">
+      <c r="H12" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="60" t="s">
+      <c r="I12" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="J12" s="60" t="s">
+      <c r="J12" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="K12" s="60" t="s">
+      <c r="K12" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="L12" s="60" t="s">
+      <c r="L12" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="M12" s="60" t="s">
+      <c r="M12" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="60" t="s">
+      <c r="N12" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="O12" s="60" t="s">
+      <c r="O12" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="P12" s="60" t="s">
+      <c r="P12" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="13"/>
-      <c r="S12" s="14"/>
+      <c r="Q12" s="79"/>
+      <c r="R12" s="73"/>
+      <c r="S12" s="74"/>
     </row>
     <row r="13" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B13" s="12"/>
-      <c r="C13" s="22" t="s">
+      <c r="B13" s="72"/>
+      <c r="C13" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="D13" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="82" t="s">
+      <c r="E13" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="82"/>
-      <c r="G13" s="82"/>
-      <c r="H13" s="82"/>
-      <c r="I13" s="82"/>
-      <c r="J13" s="82"/>
-      <c r="K13" s="82"/>
-      <c r="L13" s="82"/>
-      <c r="M13" s="82"/>
-      <c r="N13" s="82"/>
-      <c r="O13" s="82"/>
-      <c r="P13" s="82"/>
-      <c r="Q13" s="20" t="s">
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
+      <c r="H13" s="58"/>
+      <c r="I13" s="58"/>
+      <c r="J13" s="58"/>
+      <c r="K13" s="58"/>
+      <c r="L13" s="58"/>
+      <c r="M13" s="58"/>
+      <c r="N13" s="58"/>
+      <c r="O13" s="58"/>
+      <c r="P13" s="58"/>
+      <c r="Q13" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="R13" s="13"/>
-      <c r="S13" s="14"/>
+      <c r="R13" s="73"/>
+      <c r="S13" s="74"/>
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B14" s="12"/>
-      <c r="C14" s="23" t="s">
+      <c r="B14" s="72"/>
+      <c r="C14" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="82"/>
-      <c r="F14" s="82"/>
-      <c r="G14" s="82"/>
-      <c r="H14" s="82"/>
-      <c r="I14" s="82"/>
-      <c r="J14" s="82"/>
-      <c r="K14" s="82"/>
-      <c r="L14" s="82"/>
-      <c r="M14" s="82"/>
-      <c r="N14" s="82"/>
-      <c r="O14" s="82"/>
-      <c r="P14" s="82"/>
-      <c r="Q14" s="20" t="s">
+      <c r="E14" s="58"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="58"/>
+      <c r="I14" s="58"/>
+      <c r="J14" s="58"/>
+      <c r="K14" s="58"/>
+      <c r="L14" s="58"/>
+      <c r="M14" s="58"/>
+      <c r="N14" s="58"/>
+      <c r="O14" s="58"/>
+      <c r="P14" s="58"/>
+      <c r="Q14" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="R14" s="13"/>
-      <c r="S14" s="14"/>
+      <c r="R14" s="73"/>
+      <c r="S14" s="74"/>
     </row>
     <row r="15" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B15" s="12"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="61" t="s">
+      <c r="B15" s="72"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="F15" s="61" t="s">
+      <c r="F15" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="G15" s="61" t="s">
+      <c r="G15" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="H15" s="61" t="s">
+      <c r="H15" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="I15" s="61" t="s">
+      <c r="I15" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="J15" s="61" t="s">
+      <c r="J15" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="K15" s="61" t="s">
+      <c r="K15" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="L15" s="61" t="s">
+      <c r="L15" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="M15" s="61" t="s">
+      <c r="M15" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="N15" s="61" t="s">
+      <c r="N15" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="O15" s="61" t="s">
+      <c r="O15" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="P15" s="61" t="s">
+      <c r="P15" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="Q15" s="17"/>
-      <c r="R15" s="13"/>
-      <c r="S15" s="14"/>
+      <c r="Q15" s="77"/>
+      <c r="R15" s="73"/>
+      <c r="S15" s="74"/>
     </row>
     <row r="16" spans="2:19" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B16" s="12"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="57" t="s">
+      <c r="B16" s="72"/>
+      <c r="C16" s="73"/>
+      <c r="D16" s="73"/>
+      <c r="E16" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="58" t="s">
+      <c r="F16" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="59"/>
-      <c r="H16" s="58" t="s">
+      <c r="G16" s="78"/>
+      <c r="H16" s="48" t="s">
         <v>106</v>
       </c>
-      <c r="I16" s="59"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="59"/>
-      <c r="L16" s="59"/>
-      <c r="M16" s="59"/>
-      <c r="N16" s="59"/>
-      <c r="O16" s="57" t="s">
+      <c r="I16" s="78"/>
+      <c r="J16" s="78"/>
+      <c r="K16" s="78"/>
+      <c r="L16" s="78"/>
+      <c r="M16" s="78"/>
+      <c r="N16" s="78"/>
+      <c r="O16" s="47" t="s">
         <v>41</v>
       </c>
-      <c r="P16" s="58" t="s">
+      <c r="P16" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="Q16" s="13"/>
-      <c r="R16" s="13"/>
-      <c r="S16" s="14"/>
+      <c r="Q16" s="73"/>
+      <c r="R16" s="73"/>
+      <c r="S16" s="74"/>
     </row>
     <row r="17" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="13"/>
-      <c r="R17" s="13"/>
-      <c r="S17" s="14"/>
+      <c r="B17" s="72"/>
+      <c r="C17" s="73"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="73"/>
+      <c r="F17" s="73"/>
+      <c r="G17" s="73"/>
+      <c r="H17" s="73"/>
+      <c r="I17" s="73"/>
+      <c r="J17" s="73"/>
+      <c r="K17" s="73"/>
+      <c r="L17" s="73"/>
+      <c r="M17" s="73"/>
+      <c r="N17" s="73"/>
+      <c r="O17" s="73"/>
+      <c r="P17" s="73"/>
+      <c r="Q17" s="73"/>
+      <c r="R17" s="73"/>
+      <c r="S17" s="74"/>
     </row>
     <row r="18" spans="2:19" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="12"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="62" t="s">
+      <c r="B18" s="72"/>
+      <c r="C18" s="73"/>
+      <c r="D18" s="73"/>
+      <c r="E18" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="F18" s="63" t="s">
+      <c r="F18" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="G18" s="64"/>
-      <c r="H18" s="63" t="s">
+      <c r="G18" s="81"/>
+      <c r="H18" s="52" t="s">
         <v>107</v>
       </c>
-      <c r="I18" s="64"/>
-      <c r="J18" s="64"/>
-      <c r="K18" s="64"/>
-      <c r="L18" s="64"/>
-      <c r="M18" s="62" t="s">
+      <c r="I18" s="81"/>
+      <c r="J18" s="81"/>
+      <c r="K18" s="81"/>
+      <c r="L18" s="81"/>
+      <c r="M18" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="N18" s="63" t="s">
+      <c r="N18" s="52" t="s">
         <v>109</v>
       </c>
-      <c r="O18" s="62" t="s">
+      <c r="O18" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="P18" s="63" t="s">
+      <c r="P18" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="Q18" s="13"/>
-      <c r="R18" s="13"/>
-      <c r="S18" s="14"/>
+      <c r="Q18" s="73"/>
+      <c r="R18" s="73"/>
+      <c r="S18" s="74"/>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B19" s="12"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="60" t="s">
+      <c r="B19" s="72"/>
+      <c r="C19" s="73"/>
+      <c r="D19" s="80"/>
+      <c r="E19" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="F19" s="60" t="s">
+      <c r="F19" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="G19" s="60" t="s">
+      <c r="G19" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="H19" s="60" t="s">
+      <c r="H19" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="I19" s="60" t="s">
+      <c r="I19" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="J19" s="60" t="s">
+      <c r="J19" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="K19" s="60" t="s">
+      <c r="K19" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="L19" s="60" t="s">
+      <c r="L19" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="M19" s="60" t="s">
+      <c r="M19" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="N19" s="60" t="s">
+      <c r="N19" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="O19" s="60" t="s">
+      <c r="O19" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="P19" s="60" t="s">
+      <c r="P19" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="13"/>
-      <c r="S19" s="14"/>
+      <c r="Q19" s="79"/>
+      <c r="R19" s="73"/>
+      <c r="S19" s="74"/>
     </row>
     <row r="20" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B20" s="12"/>
-      <c r="C20" s="22" t="s">
+      <c r="B20" s="72"/>
+      <c r="C20" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="82" t="s">
+      <c r="E20" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="82"/>
-      <c r="G20" s="82"/>
-      <c r="H20" s="82"/>
-      <c r="I20" s="82"/>
-      <c r="J20" s="82"/>
-      <c r="K20" s="82"/>
-      <c r="L20" s="82"/>
-      <c r="M20" s="82"/>
-      <c r="N20" s="82"/>
-      <c r="O20" s="82"/>
-      <c r="P20" s="82"/>
-      <c r="Q20" s="20" t="s">
+      <c r="F20" s="58"/>
+      <c r="G20" s="58"/>
+      <c r="H20" s="58"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="58"/>
+      <c r="K20" s="58"/>
+      <c r="L20" s="58"/>
+      <c r="M20" s="58"/>
+      <c r="N20" s="58"/>
+      <c r="O20" s="58"/>
+      <c r="P20" s="58"/>
+      <c r="Q20" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="R20" s="13"/>
-      <c r="S20" s="14"/>
+      <c r="R20" s="73"/>
+      <c r="S20" s="74"/>
     </row>
     <row r="21" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B21" s="12"/>
-      <c r="C21" s="23" t="s">
+      <c r="B21" s="72"/>
+      <c r="C21" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="D21" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="82"/>
-      <c r="F21" s="82"/>
-      <c r="G21" s="82"/>
-      <c r="H21" s="82"/>
-      <c r="I21" s="82"/>
-      <c r="J21" s="82"/>
-      <c r="K21" s="82"/>
-      <c r="L21" s="82"/>
-      <c r="M21" s="82"/>
-      <c r="N21" s="82"/>
-      <c r="O21" s="82"/>
-      <c r="P21" s="82"/>
-      <c r="Q21" s="20" t="s">
+      <c r="E21" s="58"/>
+      <c r="F21" s="58"/>
+      <c r="G21" s="58"/>
+      <c r="H21" s="58"/>
+      <c r="I21" s="58"/>
+      <c r="J21" s="58"/>
+      <c r="K21" s="58"/>
+      <c r="L21" s="58"/>
+      <c r="M21" s="58"/>
+      <c r="N21" s="58"/>
+      <c r="O21" s="58"/>
+      <c r="P21" s="58"/>
+      <c r="Q21" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="R21" s="13"/>
-      <c r="S21" s="14"/>
+      <c r="R21" s="73"/>
+      <c r="S21" s="74"/>
     </row>
     <row r="22" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B22" s="12"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="61" t="s">
+      <c r="B22" s="72"/>
+      <c r="C22" s="73"/>
+      <c r="D22" s="75"/>
+      <c r="E22" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="F22" s="61" t="s">
+      <c r="F22" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="G22" s="61" t="s">
+      <c r="G22" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="H22" s="61" t="s">
+      <c r="H22" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="I22" s="61" t="s">
+      <c r="I22" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="J22" s="61" t="s">
+      <c r="J22" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="K22" s="61" t="s">
+      <c r="K22" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="L22" s="61" t="s">
+      <c r="L22" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="M22" s="61" t="s">
+      <c r="M22" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="N22" s="61" t="s">
+      <c r="N22" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="O22" s="61" t="s">
+      <c r="O22" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="P22" s="61" t="s">
+      <c r="P22" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="Q22" s="17"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="14"/>
+      <c r="Q22" s="77"/>
+      <c r="R22" s="73"/>
+      <c r="S22" s="74"/>
     </row>
     <row r="23" spans="2:19" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B23" s="12"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="57" t="s">
+      <c r="B23" s="72"/>
+      <c r="C23" s="73"/>
+      <c r="D23" s="73"/>
+      <c r="E23" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="F23" s="58" t="s">
+      <c r="F23" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="G23" s="59"/>
-      <c r="H23" s="59"/>
-      <c r="I23" s="59"/>
-      <c r="J23" s="59"/>
-      <c r="K23" s="59"/>
-      <c r="L23" s="59"/>
-      <c r="M23" s="59"/>
-      <c r="N23" s="59"/>
-      <c r="O23" s="57" t="s">
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
+      <c r="I23" s="78"/>
+      <c r="J23" s="78"/>
+      <c r="K23" s="78"/>
+      <c r="L23" s="78"/>
+      <c r="M23" s="78"/>
+      <c r="N23" s="78"/>
+      <c r="O23" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="P23" s="58" t="s">
+      <c r="P23" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="14"/>
+      <c r="Q23" s="73"/>
+      <c r="R23" s="73"/>
+      <c r="S23" s="74"/>
     </row>
     <row r="24" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B24" s="12"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="13"/>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="13"/>
-      <c r="R24" s="13"/>
-      <c r="S24" s="14"/>
+      <c r="B24" s="72"/>
+      <c r="C24" s="73"/>
+      <c r="D24" s="73"/>
+      <c r="E24" s="73"/>
+      <c r="F24" s="73"/>
+      <c r="G24" s="73"/>
+      <c r="H24" s="73"/>
+      <c r="I24" s="73"/>
+      <c r="J24" s="73"/>
+      <c r="K24" s="73"/>
+      <c r="L24" s="73"/>
+      <c r="M24" s="73"/>
+      <c r="N24" s="73"/>
+      <c r="O24" s="73"/>
+      <c r="P24" s="73"/>
+      <c r="Q24" s="73"/>
+      <c r="R24" s="73"/>
+      <c r="S24" s="74"/>
     </row>
     <row r="25" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B25" s="15"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="16"/>
-      <c r="Q25" s="16"/>
-      <c r="R25" s="16"/>
-      <c r="S25" s="17"/>
+      <c r="B25" s="75"/>
+      <c r="C25" s="76"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="76"/>
+      <c r="I25" s="76"/>
+      <c r="J25" s="76"/>
+      <c r="K25" s="76"/>
+      <c r="L25" s="76"/>
+      <c r="M25" s="76"/>
+      <c r="N25" s="76"/>
+      <c r="O25" s="76"/>
+      <c r="P25" s="76"/>
+      <c r="Q25" s="76"/>
+      <c r="R25" s="76"/>
+      <c r="S25" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2122,60 +2125,66 @@
   <dimension ref="B2:AP28"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
+    <col min="2" max="2" width="4.796875" customWidth="1"/>
     <col min="3" max="3" width="11.19921875" customWidth="1"/>
     <col min="4" max="4" width="11.1328125" customWidth="1"/>
     <col min="5" max="8" width="12.265625" customWidth="1"/>
     <col min="9" max="9" width="11.1328125" customWidth="1"/>
     <col min="10" max="10" width="11.19921875" customWidth="1"/>
+    <col min="11" max="11" width="5.33203125" customWidth="1"/>
+    <col min="12" max="13" width="3.59765625" customWidth="1"/>
+    <col min="26" max="27" width="3.59765625" customWidth="1"/>
+    <col min="28" max="28" width="2.9296875" customWidth="1"/>
+    <col min="36" max="36" width="3.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:42" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B3" s="72" t="s">
+      <c r="B3" s="63" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="73"/>
-      <c r="I3" s="73"/>
-      <c r="J3" s="73"/>
-      <c r="K3" s="74"/>
-      <c r="M3" s="72" t="s">
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="65"/>
+      <c r="M3" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="N3" s="73"/>
-      <c r="O3" s="73"/>
-      <c r="P3" s="73"/>
-      <c r="Q3" s="73"/>
-      <c r="R3" s="73"/>
-      <c r="S3" s="73"/>
-      <c r="T3" s="73"/>
-      <c r="U3" s="73"/>
-      <c r="V3" s="73"/>
-      <c r="W3" s="73"/>
-      <c r="X3" s="73"/>
-      <c r="Y3" s="73"/>
-      <c r="Z3" s="74"/>
-      <c r="AB3" s="72" t="s">
+      <c r="N3" s="64"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
+      <c r="X3" s="64"/>
+      <c r="Y3" s="64"/>
+      <c r="Z3" s="65"/>
+      <c r="AB3" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="AC3" s="73"/>
-      <c r="AD3" s="73"/>
-      <c r="AE3" s="73"/>
-      <c r="AF3" s="73"/>
-      <c r="AG3" s="73"/>
-      <c r="AH3" s="73"/>
-      <c r="AI3" s="73"/>
-      <c r="AJ3" s="74"/>
-      <c r="AK3" s="42"/>
-      <c r="AL3" s="42"/>
-      <c r="AM3" s="42"/>
-      <c r="AN3" s="42"/>
-      <c r="AO3" s="42"/>
-      <c r="AP3" s="42"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
+      <c r="AJ3" s="65"/>
+      <c r="AK3" s="33"/>
+      <c r="AL3" s="33"/>
+      <c r="AM3" s="33"/>
+      <c r="AN3" s="33"/>
+      <c r="AO3" s="33"/>
+      <c r="AP3" s="33"/>
     </row>
     <row r="4" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="1"/>
@@ -2214,169 +2223,169 @@
     </row>
     <row r="5" spans="2:42" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="4"/>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="69" t="s">
+      <c r="E5" s="60" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="69"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="69"/>
-      <c r="I5" s="24" t="s">
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="15" t="s">
         <v>59</v>
       </c>
       <c r="K5" s="5"/>
       <c r="M5" s="4"/>
-      <c r="N5" s="40" t="s">
+      <c r="N5" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="O5" s="34" t="s">
+      <c r="O5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="P5" s="78" t="s">
+      <c r="P5" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="Q5" s="78"/>
-      <c r="R5" s="78"/>
-      <c r="S5" s="78"/>
-      <c r="T5" s="78"/>
-      <c r="U5" s="78"/>
-      <c r="V5" s="78"/>
-      <c r="W5" s="78"/>
-      <c r="X5" s="35" t="s">
+      <c r="Q5" s="69"/>
+      <c r="R5" s="69"/>
+      <c r="S5" s="69"/>
+      <c r="T5" s="69"/>
+      <c r="U5" s="69"/>
+      <c r="V5" s="69"/>
+      <c r="W5" s="69"/>
+      <c r="X5" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="Y5" s="29" t="s">
+      <c r="Y5" s="20" t="s">
         <v>81</v>
       </c>
       <c r="Z5" s="5"/>
       <c r="AB5" s="4"/>
-      <c r="AC5" s="52" t="s">
+      <c r="AC5" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AD5" s="43" t="s">
+      <c r="AD5" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="AE5" s="75" t="s">
+      <c r="AE5" s="66" t="s">
         <v>93</v>
       </c>
-      <c r="AF5" s="75"/>
-      <c r="AG5" s="75"/>
-      <c r="AH5" s="44" t="s">
+      <c r="AF5" s="66"/>
+      <c r="AG5" s="66"/>
+      <c r="AH5" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="AI5" s="49" t="s">
+      <c r="AI5" s="40" t="s">
         <v>112</v>
       </c>
       <c r="AJ5" s="5"/>
     </row>
     <row r="6" spans="2:42" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B6" s="4"/>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="70"/>
-      <c r="H6" s="70"/>
-      <c r="I6" s="25" t="s">
+      <c r="E6" s="61"/>
+      <c r="F6" s="61"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="61"/>
+      <c r="I6" s="16" t="s">
         <v>60</v>
       </c>
       <c r="K6" s="5"/>
       <c r="M6" s="4"/>
-      <c r="O6" s="36"/>
-      <c r="P6" s="79"/>
-      <c r="Q6" s="79"/>
-      <c r="R6" s="79"/>
-      <c r="S6" s="79"/>
-      <c r="T6" s="79"/>
-      <c r="U6" s="79"/>
-      <c r="V6" s="79"/>
-      <c r="W6" s="79"/>
-      <c r="X6" s="37"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="70"/>
+      <c r="Q6" s="70"/>
+      <c r="R6" s="70"/>
+      <c r="S6" s="70"/>
+      <c r="T6" s="70"/>
+      <c r="U6" s="70"/>
+      <c r="V6" s="70"/>
+      <c r="W6" s="70"/>
+      <c r="X6" s="28"/>
       <c r="Z6" s="5"/>
       <c r="AB6" s="4"/>
-      <c r="AC6" s="51"/>
-      <c r="AD6" s="45"/>
-      <c r="AE6" s="76"/>
-      <c r="AF6" s="76"/>
-      <c r="AG6" s="76"/>
-      <c r="AH6" s="46"/>
-      <c r="AI6" s="50"/>
+      <c r="AC6" s="42"/>
+      <c r="AD6" s="36"/>
+      <c r="AE6" s="67"/>
+      <c r="AF6" s="67"/>
+      <c r="AG6" s="67"/>
+      <c r="AH6" s="37"/>
+      <c r="AI6" s="41"/>
       <c r="AJ6" s="5"/>
     </row>
     <row r="7" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="4"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="70"/>
-      <c r="G7" s="70"/>
-      <c r="H7" s="70"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="61"/>
+      <c r="H7" s="61"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
       <c r="M7" s="4"/>
-      <c r="N7" s="41" t="s">
+      <c r="N7" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O7" s="38" t="s">
+      <c r="O7" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P7" s="80"/>
-      <c r="Q7" s="80"/>
-      <c r="R7" s="80"/>
-      <c r="S7" s="80"/>
-      <c r="T7" s="80"/>
-      <c r="U7" s="80"/>
-      <c r="V7" s="80"/>
-      <c r="W7" s="80"/>
-      <c r="X7" s="39" t="s">
+      <c r="P7" s="71"/>
+      <c r="Q7" s="71"/>
+      <c r="R7" s="71"/>
+      <c r="S7" s="71"/>
+      <c r="T7" s="71"/>
+      <c r="U7" s="71"/>
+      <c r="V7" s="71"/>
+      <c r="W7" s="71"/>
+      <c r="X7" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="Y7" s="29" t="s">
+      <c r="Y7" s="20" t="s">
         <v>85</v>
       </c>
       <c r="Z7" s="5"/>
       <c r="AB7" s="4"/>
-      <c r="AC7" s="52" t="s">
+      <c r="AC7" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="AD7" s="47" t="s">
+      <c r="AD7" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="AE7" s="77"/>
-      <c r="AF7" s="77"/>
-      <c r="AG7" s="77"/>
-      <c r="AH7" s="48" t="s">
+      <c r="AE7" s="68"/>
+      <c r="AF7" s="68"/>
+      <c r="AG7" s="68"/>
+      <c r="AH7" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="AI7" s="49" t="s">
+      <c r="AI7" s="40" t="s">
         <v>111</v>
       </c>
       <c r="AJ7" s="5"/>
     </row>
     <row r="8" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="4"/>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E8" s="70"/>
-      <c r="F8" s="70"/>
-      <c r="G8" s="70"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="26" t="s">
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
+      <c r="I8" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="J8" s="29" t="s">
+      <c r="J8" s="20" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="5"/>
@@ -2387,44 +2396,44 @@
     </row>
     <row r="9" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B9" s="4"/>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E9" s="71"/>
-      <c r="F9" s="71"/>
-      <c r="G9" s="71"/>
-      <c r="H9" s="71"/>
-      <c r="I9" s="27" t="s">
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="62"/>
+      <c r="I9" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="J9" s="29" t="s">
+      <c r="J9" s="20" t="s">
         <v>65</v>
       </c>
       <c r="K9" s="5"/>
       <c r="M9" s="4"/>
-      <c r="N9" s="40" t="s">
+      <c r="N9" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="O9" s="34" t="s">
+      <c r="O9" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="P9" s="78" t="s">
+      <c r="P9" s="69" t="s">
         <v>83</v>
       </c>
-      <c r="Q9" s="78"/>
-      <c r="R9" s="78"/>
-      <c r="S9" s="78"/>
-      <c r="T9" s="78"/>
-      <c r="U9" s="78"/>
-      <c r="V9" s="78"/>
-      <c r="W9" s="78"/>
-      <c r="X9" s="35" t="s">
+      <c r="Q9" s="69"/>
+      <c r="R9" s="69"/>
+      <c r="S9" s="69"/>
+      <c r="T9" s="69"/>
+      <c r="U9" s="69"/>
+      <c r="V9" s="69"/>
+      <c r="W9" s="69"/>
+      <c r="X9" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="Y9" s="29" t="s">
+      <c r="Y9" s="20" t="s">
         <v>84</v>
       </c>
       <c r="Z9" s="5"/>
@@ -2435,57 +2444,57 @@
       <c r="B10" s="4"/>
       <c r="K10" s="5"/>
       <c r="M10" s="4"/>
-      <c r="O10" s="36"/>
-      <c r="P10" s="79"/>
-      <c r="Q10" s="79"/>
-      <c r="R10" s="79"/>
-      <c r="S10" s="79"/>
-      <c r="T10" s="79"/>
-      <c r="U10" s="79"/>
-      <c r="V10" s="79"/>
-      <c r="W10" s="79"/>
-      <c r="X10" s="37"/>
+      <c r="O10" s="27"/>
+      <c r="P10" s="70"/>
+      <c r="Q10" s="70"/>
+      <c r="R10" s="70"/>
+      <c r="S10" s="70"/>
+      <c r="T10" s="70"/>
+      <c r="U10" s="70"/>
+      <c r="V10" s="70"/>
+      <c r="W10" s="70"/>
+      <c r="X10" s="28"/>
       <c r="Z10" s="5"/>
       <c r="AB10" s="4"/>
       <c r="AJ10" s="5"/>
     </row>
     <row r="11" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="4"/>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="30" t="s">
+      <c r="D11" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="69" t="s">
+      <c r="E11" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="F11" s="69"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="69"/>
-      <c r="I11" s="24" t="s">
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
+      <c r="H11" s="60"/>
+      <c r="I11" s="15" t="s">
         <v>59</v>
       </c>
       <c r="K11" s="5"/>
       <c r="M11" s="4"/>
-      <c r="N11" s="41" t="s">
+      <c r="N11" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O11" s="38" t="s">
+      <c r="O11" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P11" s="80"/>
-      <c r="Q11" s="80"/>
-      <c r="R11" s="80"/>
-      <c r="S11" s="80"/>
-      <c r="T11" s="80"/>
-      <c r="U11" s="80"/>
-      <c r="V11" s="80"/>
-      <c r="W11" s="80"/>
-      <c r="X11" s="39" t="s">
+      <c r="P11" s="71"/>
+      <c r="Q11" s="71"/>
+      <c r="R11" s="71"/>
+      <c r="S11" s="71"/>
+      <c r="T11" s="71"/>
+      <c r="U11" s="71"/>
+      <c r="V11" s="71"/>
+      <c r="W11" s="71"/>
+      <c r="X11" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="Y11" s="29" t="s">
+      <c r="Y11" s="20" t="s">
         <v>82</v>
       </c>
       <c r="Z11" s="5"/>
@@ -2494,17 +2503,17 @@
     </row>
     <row r="12" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B12" s="4"/>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="31" t="s">
+      <c r="D12" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E12" s="70"/>
-      <c r="F12" s="70"/>
-      <c r="G12" s="70"/>
-      <c r="H12" s="70"/>
-      <c r="I12" s="25" t="s">
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="16" t="s">
         <v>60</v>
       </c>
       <c r="K12" s="5"/>
@@ -2516,33 +2525,33 @@
     <row r="13" spans="2:42" x14ac:dyDescent="0.45">
       <c r="B13" s="4"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="70"/>
-      <c r="F13" s="70"/>
-      <c r="G13" s="70"/>
-      <c r="H13" s="70"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="61"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
       <c r="M13" s="4"/>
-      <c r="N13" s="40" t="s">
+      <c r="N13" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="O13" s="34" t="s">
+      <c r="O13" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="P13" s="78" t="s">
+      <c r="P13" s="69" t="s">
         <v>86</v>
       </c>
-      <c r="Q13" s="78"/>
-      <c r="R13" s="78"/>
-      <c r="S13" s="78"/>
-      <c r="T13" s="78"/>
-      <c r="U13" s="78"/>
-      <c r="V13" s="78"/>
-      <c r="W13" s="78"/>
-      <c r="X13" s="35" t="s">
+      <c r="Q13" s="69"/>
+      <c r="R13" s="69"/>
+      <c r="S13" s="69"/>
+      <c r="T13" s="69"/>
+      <c r="U13" s="69"/>
+      <c r="V13" s="69"/>
+      <c r="W13" s="69"/>
+      <c r="X13" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="Y13" s="29" t="s">
+      <c r="Y13" s="20" t="s">
         <v>88</v>
       </c>
       <c r="Z13" s="5"/>
@@ -2551,76 +2560,76 @@
     </row>
     <row r="14" spans="2:42" x14ac:dyDescent="0.45">
       <c r="B14" s="4"/>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E14" s="70"/>
-      <c r="F14" s="70"/>
-      <c r="G14" s="70"/>
-      <c r="H14" s="70"/>
-      <c r="I14" s="26" t="s">
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="J14" s="29" t="s">
+      <c r="J14" s="20" t="s">
         <v>69</v>
       </c>
       <c r="K14" s="5"/>
       <c r="M14" s="4"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="79"/>
-      <c r="Q14" s="79"/>
-      <c r="R14" s="79"/>
-      <c r="S14" s="79"/>
-      <c r="T14" s="79"/>
-      <c r="U14" s="79"/>
-      <c r="V14" s="79"/>
-      <c r="W14" s="79"/>
-      <c r="X14" s="37"/>
+      <c r="O14" s="27"/>
+      <c r="P14" s="70"/>
+      <c r="Q14" s="70"/>
+      <c r="R14" s="70"/>
+      <c r="S14" s="70"/>
+      <c r="T14" s="70"/>
+      <c r="U14" s="70"/>
+      <c r="V14" s="70"/>
+      <c r="W14" s="70"/>
+      <c r="X14" s="28"/>
       <c r="Z14" s="5"/>
       <c r="AB14" s="4"/>
       <c r="AJ14" s="5"/>
     </row>
     <row r="15" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="4"/>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="33" t="s">
+      <c r="D15" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E15" s="71"/>
-      <c r="F15" s="71"/>
-      <c r="G15" s="71"/>
-      <c r="H15" s="71"/>
-      <c r="I15" s="27" t="s">
+      <c r="E15" s="62"/>
+      <c r="F15" s="62"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="62"/>
+      <c r="I15" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="J15" s="29" t="s">
+      <c r="J15" s="20" t="s">
         <v>68</v>
       </c>
       <c r="K15" s="5"/>
       <c r="M15" s="4"/>
-      <c r="N15" s="41" t="s">
+      <c r="N15" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O15" s="38" t="s">
+      <c r="O15" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P15" s="80"/>
-      <c r="Q15" s="80"/>
-      <c r="R15" s="80"/>
-      <c r="S15" s="80"/>
-      <c r="T15" s="80"/>
-      <c r="U15" s="80"/>
-      <c r="V15" s="80"/>
-      <c r="W15" s="80"/>
-      <c r="X15" s="39" t="s">
+      <c r="P15" s="71"/>
+      <c r="Q15" s="71"/>
+      <c r="R15" s="71"/>
+      <c r="S15" s="71"/>
+      <c r="T15" s="71"/>
+      <c r="U15" s="71"/>
+      <c r="V15" s="71"/>
+      <c r="W15" s="71"/>
+      <c r="X15" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="Y15" s="29" t="s">
+      <c r="Y15" s="20" t="s">
         <v>89</v>
       </c>
       <c r="Z15" s="5"/>
@@ -2644,115 +2653,115 @@
     </row>
     <row r="17" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B17" s="4"/>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="30" t="s">
+      <c r="D17" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E17" s="69" t="s">
+      <c r="E17" s="60" t="s">
         <v>70</v>
       </c>
-      <c r="F17" s="69"/>
-      <c r="G17" s="69"/>
-      <c r="H17" s="69"/>
-      <c r="I17" s="24" t="s">
+      <c r="F17" s="60"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
+      <c r="I17" s="15" t="s">
         <v>59</v>
       </c>
       <c r="K17" s="5"/>
       <c r="M17" s="4"/>
-      <c r="N17" s="40" t="s">
+      <c r="N17" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="O17" s="34" t="s">
+      <c r="O17" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="P17" s="78" t="s">
+      <c r="P17" s="69" t="s">
         <v>87</v>
       </c>
-      <c r="Q17" s="78"/>
-      <c r="R17" s="78"/>
-      <c r="S17" s="78"/>
-      <c r="T17" s="78"/>
-      <c r="U17" s="78"/>
-      <c r="V17" s="78"/>
-      <c r="W17" s="78"/>
-      <c r="X17" s="35" t="s">
+      <c r="Q17" s="69"/>
+      <c r="R17" s="69"/>
+      <c r="S17" s="69"/>
+      <c r="T17" s="69"/>
+      <c r="U17" s="69"/>
+      <c r="V17" s="69"/>
+      <c r="W17" s="69"/>
+      <c r="X17" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="Y17" s="29" t="s">
+      <c r="Y17" s="20" t="s">
         <v>90</v>
       </c>
       <c r="Z17" s="5"/>
     </row>
     <row r="18" spans="2:36" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B18" s="4"/>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="31" t="s">
+      <c r="D18" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E18" s="70"/>
-      <c r="F18" s="70"/>
-      <c r="G18" s="70"/>
-      <c r="H18" s="70"/>
-      <c r="I18" s="25" t="s">
+      <c r="E18" s="61"/>
+      <c r="F18" s="61"/>
+      <c r="G18" s="61"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="16" t="s">
         <v>60</v>
       </c>
       <c r="K18" s="5"/>
       <c r="M18" s="4"/>
-      <c r="O18" s="36"/>
-      <c r="P18" s="79"/>
-      <c r="Q18" s="79"/>
-      <c r="R18" s="79"/>
-      <c r="S18" s="79"/>
-      <c r="T18" s="79"/>
-      <c r="U18" s="79"/>
-      <c r="V18" s="79"/>
-      <c r="W18" s="79"/>
-      <c r="X18" s="37"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="70"/>
+      <c r="Q18" s="70"/>
+      <c r="R18" s="70"/>
+      <c r="S18" s="70"/>
+      <c r="T18" s="70"/>
+      <c r="U18" s="70"/>
+      <c r="V18" s="70"/>
+      <c r="W18" s="70"/>
+      <c r="X18" s="28"/>
       <c r="Z18" s="5"/>
-      <c r="AB18" s="72" t="s">
+      <c r="AB18" s="63" t="s">
         <v>101</v>
       </c>
-      <c r="AC18" s="73"/>
-      <c r="AD18" s="73"/>
-      <c r="AE18" s="73"/>
-      <c r="AF18" s="73"/>
-      <c r="AG18" s="73"/>
-      <c r="AH18" s="73"/>
-      <c r="AI18" s="73"/>
-      <c r="AJ18" s="74"/>
+      <c r="AC18" s="64"/>
+      <c r="AD18" s="64"/>
+      <c r="AE18" s="64"/>
+      <c r="AF18" s="64"/>
+      <c r="AG18" s="64"/>
+      <c r="AH18" s="64"/>
+      <c r="AI18" s="64"/>
+      <c r="AJ18" s="65"/>
     </row>
     <row r="19" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="4"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="70"/>
-      <c r="F19" s="70"/>
-      <c r="G19" s="70"/>
-      <c r="H19" s="70"/>
+      <c r="E19" s="61"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="61"/>
+      <c r="H19" s="61"/>
       <c r="I19" s="5"/>
       <c r="K19" s="5"/>
       <c r="M19" s="4"/>
-      <c r="N19" s="41" t="s">
+      <c r="N19" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O19" s="38" t="s">
+      <c r="O19" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P19" s="80"/>
-      <c r="Q19" s="80"/>
-      <c r="R19" s="80"/>
-      <c r="S19" s="80"/>
-      <c r="T19" s="80"/>
-      <c r="U19" s="80"/>
-      <c r="V19" s="80"/>
-      <c r="W19" s="80"/>
-      <c r="X19" s="39" t="s">
+      <c r="P19" s="71"/>
+      <c r="Q19" s="71"/>
+      <c r="R19" s="71"/>
+      <c r="S19" s="71"/>
+      <c r="T19" s="71"/>
+      <c r="U19" s="71"/>
+      <c r="V19" s="71"/>
+      <c r="W19" s="71"/>
+      <c r="X19" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="Y19" s="29" t="s">
+      <c r="Y19" s="20" t="s">
         <v>91</v>
       </c>
       <c r="Z19" s="5"/>
@@ -2768,71 +2777,71 @@
     </row>
     <row r="20" spans="2:36" x14ac:dyDescent="0.45">
       <c r="B20" s="4"/>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D20" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E20" s="70"/>
-      <c r="F20" s="70"/>
-      <c r="G20" s="70"/>
-      <c r="H20" s="70"/>
-      <c r="I20" s="26" t="s">
+      <c r="E20" s="61"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="61"/>
+      <c r="H20" s="61"/>
+      <c r="I20" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="J20" s="29" t="s">
+      <c r="J20" s="20" t="s">
         <v>72</v>
       </c>
       <c r="K20" s="5"/>
       <c r="M20" s="4"/>
       <c r="Z20" s="5"/>
       <c r="AB20" s="4"/>
-      <c r="AC20" s="52" t="s">
+      <c r="AC20" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AD20" s="43" t="s">
+      <c r="AD20" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="AE20" s="75" t="s">
+      <c r="AE20" s="66" t="s">
         <v>97</v>
       </c>
-      <c r="AF20" s="75"/>
-      <c r="AG20" s="75"/>
+      <c r="AF20" s="66"/>
+      <c r="AG20" s="66"/>
       <c r="AH20" s="3"/>
       <c r="AJ20" s="5"/>
     </row>
     <row r="21" spans="2:36" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B21" s="4"/>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="33" t="s">
+      <c r="D21" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E21" s="71"/>
-      <c r="F21" s="71"/>
-      <c r="G21" s="71"/>
-      <c r="H21" s="71"/>
-      <c r="I21" s="27" t="s">
+      <c r="E21" s="62"/>
+      <c r="F21" s="62"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="62"/>
+      <c r="I21" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="J21" s="29" t="s">
+      <c r="J21" s="20" t="s">
         <v>71</v>
       </c>
       <c r="K21" s="5"/>
       <c r="M21" s="4"/>
       <c r="Z21" s="5"/>
       <c r="AB21" s="4"/>
-      <c r="AC21" s="51"/>
-      <c r="AD21" s="45"/>
-      <c r="AE21" s="76"/>
-      <c r="AF21" s="76"/>
-      <c r="AG21" s="76"/>
-      <c r="AH21" s="53" t="s">
+      <c r="AC21" s="42"/>
+      <c r="AD21" s="36"/>
+      <c r="AE21" s="67"/>
+      <c r="AF21" s="67"/>
+      <c r="AG21" s="67"/>
+      <c r="AH21" s="44" t="s">
         <v>99</v>
       </c>
-      <c r="AI21" s="49" t="s">
+      <c r="AI21" s="40" t="s">
         <v>100</v>
       </c>
       <c r="AJ21" s="5"/>
@@ -2843,33 +2852,33 @@
       <c r="M22" s="4"/>
       <c r="Z22" s="5"/>
       <c r="AB22" s="4"/>
-      <c r="AC22" s="52" t="s">
+      <c r="AC22" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="AD22" s="47" t="s">
+      <c r="AD22" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="AE22" s="77"/>
-      <c r="AF22" s="77"/>
-      <c r="AG22" s="77"/>
+      <c r="AE22" s="68"/>
+      <c r="AF22" s="68"/>
+      <c r="AG22" s="68"/>
       <c r="AH22" s="8"/>
       <c r="AJ22" s="5"/>
     </row>
     <row r="23" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B23" s="4"/>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="30" t="s">
+      <c r="D23" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E23" s="69" t="s">
+      <c r="E23" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="F23" s="69"/>
-      <c r="G23" s="69"/>
-      <c r="H23" s="69"/>
-      <c r="I23" s="24" t="s">
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="15" t="s">
         <v>59</v>
       </c>
       <c r="K23" s="5"/>
@@ -2880,112 +2889,112 @@
     </row>
     <row r="24" spans="2:36" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B24" s="4"/>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="31" t="s">
+      <c r="D24" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="70"/>
-      <c r="F24" s="70"/>
-      <c r="G24" s="70"/>
-      <c r="H24" s="70"/>
-      <c r="I24" s="25" t="s">
+      <c r="E24" s="61"/>
+      <c r="F24" s="61"/>
+      <c r="G24" s="61"/>
+      <c r="H24" s="61"/>
+      <c r="I24" s="16" t="s">
         <v>60</v>
       </c>
       <c r="K24" s="5"/>
       <c r="M24" s="4"/>
       <c r="Z24" s="5"/>
       <c r="AB24" s="4"/>
-      <c r="AC24" s="52" t="s">
+      <c r="AC24" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AD24" s="43" t="s">
+      <c r="AD24" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="AE24" s="75" t="s">
+      <c r="AE24" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="AF24" s="75"/>
-      <c r="AG24" s="75"/>
+      <c r="AF24" s="66"/>
+      <c r="AG24" s="66"/>
       <c r="AH24" s="3"/>
       <c r="AJ24" s="5"/>
     </row>
     <row r="25" spans="2:36" ht="19.5" x14ac:dyDescent="0.6">
       <c r="B25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="70"/>
-      <c r="F25" s="70"/>
-      <c r="G25" s="70"/>
-      <c r="H25" s="70"/>
+      <c r="E25" s="61"/>
+      <c r="F25" s="61"/>
+      <c r="G25" s="61"/>
+      <c r="H25" s="61"/>
       <c r="I25" s="5"/>
       <c r="K25" s="5"/>
       <c r="M25" s="4"/>
       <c r="Z25" s="5"/>
       <c r="AB25" s="4"/>
-      <c r="AC25" s="51"/>
-      <c r="AD25" s="45"/>
-      <c r="AE25" s="76"/>
-      <c r="AF25" s="76"/>
-      <c r="AG25" s="76"/>
-      <c r="AH25" s="53" t="s">
+      <c r="AC25" s="42"/>
+      <c r="AD25" s="36"/>
+      <c r="AE25" s="67"/>
+      <c r="AF25" s="67"/>
+      <c r="AG25" s="67"/>
+      <c r="AH25" s="44" t="s">
         <v>99</v>
       </c>
-      <c r="AI25" s="49" t="s">
+      <c r="AI25" s="40" t="s">
         <v>1</v>
       </c>
       <c r="AJ25" s="5"/>
     </row>
     <row r="26" spans="2:36" ht="14.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B26" s="4"/>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="32" t="s">
+      <c r="D26" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E26" s="70"/>
-      <c r="F26" s="70"/>
-      <c r="G26" s="70"/>
-      <c r="H26" s="70"/>
-      <c r="I26" s="26" t="s">
+      <c r="E26" s="61"/>
+      <c r="F26" s="61"/>
+      <c r="G26" s="61"/>
+      <c r="H26" s="61"/>
+      <c r="I26" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="J26" s="29" t="s">
+      <c r="J26" s="20" t="s">
         <v>75</v>
       </c>
       <c r="K26" s="5"/>
       <c r="M26" s="4"/>
       <c r="Z26" s="5"/>
       <c r="AB26" s="4"/>
-      <c r="AC26" s="52" t="s">
+      <c r="AC26" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="AD26" s="47" t="s">
+      <c r="AD26" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="AE26" s="77"/>
-      <c r="AF26" s="77"/>
-      <c r="AG26" s="77"/>
+      <c r="AE26" s="68"/>
+      <c r="AF26" s="68"/>
+      <c r="AG26" s="68"/>
       <c r="AH26" s="8"/>
       <c r="AJ26" s="5"/>
     </row>
     <row r="27" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B27" s="4"/>
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E27" s="71"/>
-      <c r="F27" s="71"/>
-      <c r="G27" s="71"/>
-      <c r="H27" s="71"/>
-      <c r="I27" s="27" t="s">
+      <c r="E27" s="62"/>
+      <c r="F27" s="62"/>
+      <c r="G27" s="62"/>
+      <c r="H27" s="62"/>
+      <c r="I27" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="J27" s="29" t="s">
+      <c r="J27" s="20" t="s">
         <v>74</v>
       </c>
       <c r="K27" s="5"/>

</xml_diff>

<commit_message>
Fixed some drive train issues
</commit_message>
<xml_diff>
--- a/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
+++ b/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_Software\electrical_hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFE2FBE8-47B0-4669-9FD4-62BD20041242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A406F8DC-A6C9-4FAB-BE16-7D4F81268323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Layout" sheetId="1" r:id="rId1"/>
@@ -916,7 +916,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1028,6 +1028,13 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1073,22 +1080,27 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1382,77 +1394,72 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:19" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="62" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="Q2" s="59"/>
-      <c r="R2" s="59"/>
-      <c r="S2" s="59"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B3" s="80"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
-      <c r="J3" s="83"/>
-      <c r="K3" s="83"/>
-      <c r="L3" s="83"/>
-      <c r="M3" s="83"/>
-      <c r="N3" s="83"/>
-      <c r="O3" s="83"/>
-      <c r="P3" s="83"/>
-      <c r="Q3" s="83"/>
-      <c r="R3" s="83"/>
-      <c r="S3" s="79"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="3"/>
     </row>
     <row r="4" spans="2:19" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B4" s="72"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
+      <c r="B4" s="4"/>
       <c r="E4" s="53" t="s">
         <v>102</v>
       </c>
       <c r="F4" s="54" t="s">
         <v>103</v>
       </c>
-      <c r="G4" s="82"/>
-      <c r="H4" s="82"/>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82"/>
-      <c r="K4" s="82"/>
-      <c r="L4" s="82"/>
-      <c r="M4" s="82"/>
-      <c r="N4" s="82"/>
-      <c r="O4" s="82"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="59"/>
+      <c r="O4" s="59"/>
       <c r="P4" s="54" t="s">
         <v>108</v>
       </c>
-      <c r="Q4" s="73"/>
-      <c r="R4" s="73"/>
-      <c r="S4" s="74"/>
+      <c r="S4" s="5"/>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B5" s="72"/>
-      <c r="C5" s="73"/>
-      <c r="D5" s="80"/>
+      <c r="B5" s="4"/>
+      <c r="D5" s="1"/>
       <c r="E5" s="45" t="s">
         <v>13</v>
       </c>
@@ -1489,68 +1496,64 @@
       <c r="P5" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="Q5" s="79"/>
-      <c r="R5" s="73"/>
-      <c r="S5" s="74"/>
+      <c r="Q5" s="3"/>
+      <c r="S5" s="5"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B6" s="72"/>
+      <c r="B6" s="4"/>
       <c r="C6" s="13" t="s">
         <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="57" t="s">
+      <c r="E6" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
-      <c r="I6" s="57"/>
-      <c r="J6" s="57"/>
-      <c r="K6" s="57"/>
-      <c r="L6" s="57"/>
-      <c r="M6" s="57"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="57"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="60"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="60"/>
+      <c r="L6" s="60"/>
+      <c r="M6" s="60"/>
+      <c r="N6" s="60"/>
+      <c r="O6" s="60"/>
+      <c r="P6" s="60"/>
       <c r="Q6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="R6" s="73"/>
-      <c r="S6" s="74"/>
+      <c r="S6" s="5"/>
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B7" s="72"/>
+      <c r="B7" s="4"/>
       <c r="C7" s="14" t="s">
         <v>40</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="57"/>
-      <c r="H7" s="57"/>
-      <c r="I7" s="57"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="57"/>
-      <c r="L7" s="57"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
-      <c r="P7" s="57"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="60"/>
+      <c r="G7" s="60"/>
+      <c r="H7" s="60"/>
+      <c r="I7" s="60"/>
+      <c r="J7" s="60"/>
+      <c r="K7" s="60"/>
+      <c r="L7" s="60"/>
+      <c r="M7" s="60"/>
+      <c r="N7" s="60"/>
+      <c r="O7" s="60"/>
+      <c r="P7" s="60"/>
       <c r="Q7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="R7" s="73"/>
-      <c r="S7" s="74"/>
+      <c r="S7" s="5"/>
     </row>
     <row r="8" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B8" s="72"/>
-      <c r="C8" s="73"/>
-      <c r="D8" s="75"/>
+      <c r="B8" s="4"/>
+      <c r="D8" s="6"/>
       <c r="E8" s="46" t="s">
         <v>1</v>
       </c>
@@ -1587,14 +1590,11 @@
       <c r="P8" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="Q8" s="77"/>
-      <c r="R8" s="73"/>
-      <c r="S8" s="74"/>
+      <c r="Q8" s="8"/>
+      <c r="S8" s="5"/>
     </row>
     <row r="9" spans="2:19" ht="38.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="72"/>
-      <c r="C9" s="73"/>
-      <c r="D9" s="73"/>
+      <c r="B9" s="4"/>
       <c r="E9" s="55" t="s">
         <v>104</v>
       </c>
@@ -1625,56 +1625,33 @@
       <c r="N9" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="O9" s="78"/>
-      <c r="P9" s="78"/>
-      <c r="Q9" s="73"/>
-      <c r="R9" s="73"/>
-      <c r="S9" s="74"/>
+      <c r="O9" s="57"/>
+      <c r="P9" s="57"/>
+      <c r="S9" s="5"/>
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B10" s="72"/>
-      <c r="C10" s="73"/>
-      <c r="D10" s="73"/>
-      <c r="E10" s="73"/>
-      <c r="F10" s="73"/>
-      <c r="G10" s="73"/>
-      <c r="H10" s="73"/>
-      <c r="I10" s="73"/>
-      <c r="J10" s="73"/>
-      <c r="K10" s="73"/>
-      <c r="L10" s="73"/>
-      <c r="M10" s="73"/>
-      <c r="N10" s="73"/>
-      <c r="O10" s="73"/>
-      <c r="P10" s="73"/>
-      <c r="Q10" s="73"/>
-      <c r="R10" s="73"/>
-      <c r="S10" s="74"/>
+      <c r="B10" s="4"/>
+      <c r="S10" s="5"/>
     </row>
     <row r="11" spans="2:19" ht="29.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B11" s="72"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="82"/>
-      <c r="F11" s="82"/>
-      <c r="G11" s="82"/>
-      <c r="H11" s="82"/>
-      <c r="I11" s="82"/>
-      <c r="J11" s="82"/>
-      <c r="K11" s="82"/>
-      <c r="L11" s="82"/>
-      <c r="M11" s="82"/>
-      <c r="N11" s="82"/>
-      <c r="O11" s="82"/>
-      <c r="P11" s="82"/>
-      <c r="Q11" s="73"/>
-      <c r="R11" s="73"/>
-      <c r="S11" s="74"/>
+      <c r="B11" s="4"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="59"/>
+      <c r="K11" s="59"/>
+      <c r="L11" s="59"/>
+      <c r="M11" s="59"/>
+      <c r="N11" s="59"/>
+      <c r="O11" s="59"/>
+      <c r="P11" s="59"/>
+      <c r="S11" s="5"/>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B12" s="72"/>
-      <c r="C12" s="73"/>
-      <c r="D12" s="80"/>
+      <c r="B12" s="4"/>
+      <c r="D12" s="1"/>
       <c r="E12" s="49" t="s">
         <v>13</v>
       </c>
@@ -1711,68 +1688,64 @@
       <c r="P12" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="Q12" s="79"/>
-      <c r="R12" s="73"/>
-      <c r="S12" s="74"/>
+      <c r="Q12" s="3"/>
+      <c r="S12" s="5"/>
     </row>
     <row r="13" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B13" s="72"/>
+      <c r="B13" s="4"/>
       <c r="C13" s="13" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="58" t="s">
+      <c r="E13" s="61" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="58"/>
-      <c r="G13" s="58"/>
-      <c r="H13" s="58"/>
-      <c r="I13" s="58"/>
-      <c r="J13" s="58"/>
-      <c r="K13" s="58"/>
-      <c r="L13" s="58"/>
-      <c r="M13" s="58"/>
-      <c r="N13" s="58"/>
-      <c r="O13" s="58"/>
-      <c r="P13" s="58"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="61"/>
+      <c r="I13" s="61"/>
+      <c r="J13" s="61"/>
+      <c r="K13" s="61"/>
+      <c r="L13" s="61"/>
+      <c r="M13" s="61"/>
+      <c r="N13" s="61"/>
+      <c r="O13" s="61"/>
+      <c r="P13" s="61"/>
       <c r="Q13" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="R13" s="73"/>
-      <c r="S13" s="74"/>
+      <c r="S13" s="5"/>
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B14" s="72"/>
+      <c r="B14" s="4"/>
       <c r="C14" s="14" t="s">
         <v>30</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="58"/>
-      <c r="F14" s="58"/>
-      <c r="G14" s="58"/>
-      <c r="H14" s="58"/>
-      <c r="I14" s="58"/>
-      <c r="J14" s="58"/>
-      <c r="K14" s="58"/>
-      <c r="L14" s="58"/>
-      <c r="M14" s="58"/>
-      <c r="N14" s="58"/>
-      <c r="O14" s="58"/>
-      <c r="P14" s="58"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="61"/>
+      <c r="L14" s="61"/>
+      <c r="M14" s="61"/>
+      <c r="N14" s="61"/>
+      <c r="O14" s="61"/>
+      <c r="P14" s="61"/>
       <c r="Q14" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="R14" s="73"/>
-      <c r="S14" s="74"/>
+      <c r="S14" s="5"/>
     </row>
     <row r="15" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B15" s="72"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="75"/>
+      <c r="B15" s="4"/>
+      <c r="D15" s="6"/>
       <c r="E15" s="50" t="s">
         <v>1</v>
       </c>
@@ -1809,78 +1782,55 @@
       <c r="P15" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="Q15" s="77"/>
-      <c r="R15" s="73"/>
-      <c r="S15" s="74"/>
+      <c r="Q15" s="8"/>
+      <c r="S15" s="5"/>
     </row>
     <row r="16" spans="2:19" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B16" s="72"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="73"/>
+      <c r="B16" s="4"/>
       <c r="E16" s="47" t="s">
         <v>43</v>
       </c>
       <c r="F16" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="78"/>
+      <c r="G16" s="57"/>
       <c r="H16" s="48" t="s">
         <v>106</v>
       </c>
-      <c r="I16" s="78"/>
-      <c r="J16" s="78"/>
-      <c r="K16" s="78"/>
-      <c r="L16" s="78"/>
-      <c r="M16" s="78"/>
-      <c r="N16" s="78"/>
+      <c r="I16" s="57"/>
+      <c r="J16" s="57"/>
+      <c r="K16" s="57"/>
+      <c r="L16" s="57"/>
+      <c r="M16" s="57"/>
+      <c r="N16" s="57"/>
       <c r="O16" s="47" t="s">
         <v>41</v>
       </c>
       <c r="P16" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="Q16" s="73"/>
-      <c r="R16" s="73"/>
-      <c r="S16" s="74"/>
+      <c r="S16" s="5"/>
     </row>
     <row r="17" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B17" s="72"/>
-      <c r="C17" s="73"/>
-      <c r="D17" s="73"/>
-      <c r="E17" s="73"/>
-      <c r="F17" s="73"/>
-      <c r="G17" s="73"/>
-      <c r="H17" s="73"/>
-      <c r="I17" s="73"/>
-      <c r="J17" s="73"/>
-      <c r="K17" s="73"/>
-      <c r="L17" s="73"/>
-      <c r="M17" s="73"/>
-      <c r="N17" s="73"/>
-      <c r="O17" s="73"/>
-      <c r="P17" s="73"/>
-      <c r="Q17" s="73"/>
-      <c r="R17" s="73"/>
-      <c r="S17" s="74"/>
+      <c r="B17" s="4"/>
+      <c r="S17" s="5"/>
     </row>
     <row r="18" spans="2:19" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="72"/>
-      <c r="C18" s="73"/>
-      <c r="D18" s="73"/>
-      <c r="E18" s="51" t="s">
+      <c r="B18" s="4"/>
+      <c r="E18" s="59"/>
+      <c r="F18" s="59"/>
+      <c r="G18" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="F18" s="52" t="s">
+      <c r="H18" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="G18" s="81"/>
-      <c r="H18" s="52" t="s">
+      <c r="I18" s="52" t="s">
         <v>107</v>
       </c>
-      <c r="I18" s="81"/>
-      <c r="J18" s="81"/>
-      <c r="K18" s="81"/>
-      <c r="L18" s="81"/>
+      <c r="J18" s="58"/>
+      <c r="K18" s="58"/>
+      <c r="L18" s="58"/>
       <c r="M18" s="51" t="s">
         <v>110</v>
       </c>
@@ -1893,15 +1843,12 @@
       <c r="P18" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="Q18" s="73"/>
-      <c r="R18" s="73"/>
-      <c r="S18" s="74"/>
+      <c r="S18" s="5"/>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B19" s="72"/>
-      <c r="C19" s="73"/>
-      <c r="D19" s="80"/>
-      <c r="E19" s="49" t="s">
+      <c r="B19" s="4"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="75" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="49" t="s">
@@ -1934,72 +1881,68 @@
       <c r="O19" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="P19" s="49" t="s">
+      <c r="P19" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="Q19" s="79"/>
-      <c r="R19" s="73"/>
-      <c r="S19" s="74"/>
+      <c r="Q19" s="3"/>
+      <c r="S19" s="5"/>
     </row>
     <row r="20" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B20" s="72"/>
+      <c r="B20" s="4"/>
       <c r="C20" s="13" t="s">
         <v>29</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="58" t="s">
+      <c r="E20" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="58"/>
-      <c r="G20" s="58"/>
-      <c r="H20" s="58"/>
-      <c r="I20" s="58"/>
-      <c r="J20" s="58"/>
-      <c r="K20" s="58"/>
-      <c r="L20" s="58"/>
-      <c r="M20" s="58"/>
-      <c r="N20" s="58"/>
-      <c r="O20" s="58"/>
-      <c r="P20" s="58"/>
+      <c r="F20" s="78"/>
+      <c r="G20" s="78"/>
+      <c r="H20" s="78"/>
+      <c r="I20" s="78"/>
+      <c r="J20" s="78"/>
+      <c r="K20" s="78"/>
+      <c r="L20" s="78"/>
+      <c r="M20" s="78"/>
+      <c r="N20" s="78"/>
+      <c r="O20" s="78"/>
+      <c r="P20" s="79"/>
       <c r="Q20" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="R20" s="73"/>
-      <c r="S20" s="74"/>
+      <c r="S20" s="5"/>
     </row>
     <row r="21" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B21" s="72"/>
+      <c r="B21" s="4"/>
       <c r="C21" s="14" t="s">
         <v>30</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="58"/>
-      <c r="F21" s="58"/>
-      <c r="G21" s="58"/>
-      <c r="H21" s="58"/>
-      <c r="I21" s="58"/>
-      <c r="J21" s="58"/>
-      <c r="K21" s="58"/>
-      <c r="L21" s="58"/>
-      <c r="M21" s="58"/>
-      <c r="N21" s="58"/>
-      <c r="O21" s="58"/>
-      <c r="P21" s="58"/>
+      <c r="E21" s="77"/>
+      <c r="F21" s="78"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="78"/>
+      <c r="I21" s="78"/>
+      <c r="J21" s="78"/>
+      <c r="K21" s="78"/>
+      <c r="L21" s="78"/>
+      <c r="M21" s="78"/>
+      <c r="N21" s="78"/>
+      <c r="O21" s="78"/>
+      <c r="P21" s="79"/>
       <c r="Q21" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="R21" s="73"/>
-      <c r="S21" s="74"/>
+      <c r="S21" s="5"/>
     </row>
     <row r="22" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B22" s="72"/>
-      <c r="C22" s="73"/>
-      <c r="D22" s="75"/>
-      <c r="E22" s="50" t="s">
+      <c r="B22" s="4"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="80" t="s">
         <v>1</v>
       </c>
       <c r="F22" s="50" t="s">
@@ -2032,80 +1975,59 @@
       <c r="O22" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="P22" s="50" t="s">
+      <c r="P22" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="Q22" s="77"/>
-      <c r="R22" s="73"/>
-      <c r="S22" s="74"/>
+      <c r="Q22" s="8"/>
+      <c r="S22" s="5"/>
     </row>
     <row r="23" spans="2:19" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B23" s="72"/>
-      <c r="C23" s="73"/>
-      <c r="D23" s="73"/>
+      <c r="B23" s="4"/>
       <c r="E23" s="47" t="s">
         <v>49</v>
       </c>
       <c r="F23" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="G23" s="78"/>
-      <c r="H23" s="78"/>
-      <c r="I23" s="78"/>
-      <c r="J23" s="78"/>
-      <c r="K23" s="78"/>
-      <c r="L23" s="78"/>
-      <c r="M23" s="78"/>
-      <c r="N23" s="78"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="57"/>
+      <c r="J23" s="57"/>
+      <c r="K23" s="57"/>
+      <c r="L23" s="57"/>
+      <c r="M23" s="57"/>
+      <c r="N23" s="57"/>
       <c r="O23" s="47" t="s">
         <v>45</v>
       </c>
       <c r="P23" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="Q23" s="73"/>
-      <c r="R23" s="73"/>
-      <c r="S23" s="74"/>
+      <c r="S23" s="5"/>
     </row>
     <row r="24" spans="2:19" x14ac:dyDescent="0.45">
-      <c r="B24" s="72"/>
-      <c r="C24" s="73"/>
-      <c r="D24" s="73"/>
-      <c r="E24" s="73"/>
-      <c r="F24" s="73"/>
-      <c r="G24" s="73"/>
-      <c r="H24" s="73"/>
-      <c r="I24" s="73"/>
-      <c r="J24" s="73"/>
-      <c r="K24" s="73"/>
-      <c r="L24" s="73"/>
-      <c r="M24" s="73"/>
-      <c r="N24" s="73"/>
-      <c r="O24" s="73"/>
-      <c r="P24" s="73"/>
-      <c r="Q24" s="73"/>
-      <c r="R24" s="73"/>
-      <c r="S24" s="74"/>
+      <c r="B24" s="4"/>
+      <c r="S24" s="5"/>
     </row>
     <row r="25" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B25" s="75"/>
-      <c r="C25" s="76"/>
-      <c r="D25" s="76"/>
-      <c r="E25" s="76"/>
-      <c r="F25" s="76"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="76"/>
-      <c r="I25" s="76"/>
-      <c r="J25" s="76"/>
-      <c r="K25" s="76"/>
-      <c r="L25" s="76"/>
-      <c r="M25" s="76"/>
-      <c r="N25" s="76"/>
-      <c r="O25" s="76"/>
-      <c r="P25" s="76"/>
-      <c r="Q25" s="76"/>
-      <c r="R25" s="76"/>
-      <c r="S25" s="77"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
+      <c r="P25" s="7"/>
+      <c r="Q25" s="7"/>
+      <c r="R25" s="7"/>
+      <c r="S25" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2140,45 +2062,45 @@
   <sheetData>
     <row r="2" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:42" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B3" s="63" t="s">
+      <c r="B3" s="66" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="65"/>
-      <c r="M3" s="63" t="s">
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="68"/>
+      <c r="M3" s="66" t="s">
         <v>76</v>
       </c>
-      <c r="N3" s="64"/>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
-      <c r="X3" s="64"/>
-      <c r="Y3" s="64"/>
-      <c r="Z3" s="65"/>
-      <c r="AB3" s="63" t="s">
+      <c r="N3" s="67"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
+      <c r="X3" s="67"/>
+      <c r="Y3" s="67"/>
+      <c r="Z3" s="68"/>
+      <c r="AB3" s="66" t="s">
         <v>93</v>
       </c>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
-      <c r="AJ3" s="65"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
+      <c r="AJ3" s="68"/>
       <c r="AK3" s="33"/>
       <c r="AL3" s="33"/>
       <c r="AM3" s="33"/>
@@ -2229,12 +2151,12 @@
       <c r="D5" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="60" t="s">
+      <c r="E5" s="63" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="60"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
       <c r="I5" s="15" t="s">
         <v>59</v>
       </c>
@@ -2246,16 +2168,16 @@
       <c r="O5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="P5" s="69" t="s">
+      <c r="P5" s="72" t="s">
         <v>80</v>
       </c>
-      <c r="Q5" s="69"/>
-      <c r="R5" s="69"/>
-      <c r="S5" s="69"/>
-      <c r="T5" s="69"/>
-      <c r="U5" s="69"/>
-      <c r="V5" s="69"/>
-      <c r="W5" s="69"/>
+      <c r="Q5" s="72"/>
+      <c r="R5" s="72"/>
+      <c r="S5" s="72"/>
+      <c r="T5" s="72"/>
+      <c r="U5" s="72"/>
+      <c r="V5" s="72"/>
+      <c r="W5" s="72"/>
       <c r="X5" s="26" t="s">
         <v>78</v>
       </c>
@@ -2270,11 +2192,11 @@
       <c r="AD5" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="AE5" s="66" t="s">
+      <c r="AE5" s="69" t="s">
         <v>93</v>
       </c>
-      <c r="AF5" s="66"/>
-      <c r="AG5" s="66"/>
+      <c r="AF5" s="69"/>
+      <c r="AG5" s="69"/>
       <c r="AH5" s="35" t="s">
         <v>95</v>
       </c>
@@ -2291,32 +2213,32 @@
       <c r="D6" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
-      <c r="G6" s="61"/>
-      <c r="H6" s="61"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
       <c r="I6" s="16" t="s">
         <v>60</v>
       </c>
       <c r="K6" s="5"/>
       <c r="M6" s="4"/>
       <c r="O6" s="27"/>
-      <c r="P6" s="70"/>
-      <c r="Q6" s="70"/>
-      <c r="R6" s="70"/>
-      <c r="S6" s="70"/>
-      <c r="T6" s="70"/>
-      <c r="U6" s="70"/>
-      <c r="V6" s="70"/>
-      <c r="W6" s="70"/>
+      <c r="P6" s="73"/>
+      <c r="Q6" s="73"/>
+      <c r="R6" s="73"/>
+      <c r="S6" s="73"/>
+      <c r="T6" s="73"/>
+      <c r="U6" s="73"/>
+      <c r="V6" s="73"/>
+      <c r="W6" s="73"/>
       <c r="X6" s="28"/>
       <c r="Z6" s="5"/>
       <c r="AB6" s="4"/>
       <c r="AC6" s="42"/>
       <c r="AD6" s="36"/>
-      <c r="AE6" s="67"/>
-      <c r="AF6" s="67"/>
-      <c r="AG6" s="67"/>
+      <c r="AE6" s="70"/>
+      <c r="AF6" s="70"/>
+      <c r="AG6" s="70"/>
       <c r="AH6" s="37"/>
       <c r="AI6" s="41"/>
       <c r="AJ6" s="5"/>
@@ -2324,10 +2246,10 @@
     <row r="7" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="4"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="61"/>
-      <c r="F7" s="61"/>
-      <c r="G7" s="61"/>
-      <c r="H7" s="61"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
       <c r="M7" s="4"/>
@@ -2337,14 +2259,14 @@
       <c r="O7" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P7" s="71"/>
-      <c r="Q7" s="71"/>
-      <c r="R7" s="71"/>
-      <c r="S7" s="71"/>
-      <c r="T7" s="71"/>
-      <c r="U7" s="71"/>
-      <c r="V7" s="71"/>
-      <c r="W7" s="71"/>
+      <c r="P7" s="74"/>
+      <c r="Q7" s="74"/>
+      <c r="R7" s="74"/>
+      <c r="S7" s="74"/>
+      <c r="T7" s="74"/>
+      <c r="U7" s="74"/>
+      <c r="V7" s="74"/>
+      <c r="W7" s="74"/>
       <c r="X7" s="30" t="s">
         <v>79</v>
       </c>
@@ -2359,9 +2281,9 @@
       <c r="AD7" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="AE7" s="68"/>
-      <c r="AF7" s="68"/>
-      <c r="AG7" s="68"/>
+      <c r="AE7" s="71"/>
+      <c r="AF7" s="71"/>
+      <c r="AG7" s="71"/>
       <c r="AH7" s="39" t="s">
         <v>96</v>
       </c>
@@ -2378,10 +2300,10 @@
       <c r="D8" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
+      <c r="G8" s="64"/>
+      <c r="H8" s="64"/>
       <c r="I8" s="17" t="s">
         <v>61</v>
       </c>
@@ -2402,10 +2324,10 @@
       <c r="D9" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E9" s="62"/>
-      <c r="F9" s="62"/>
-      <c r="G9" s="62"/>
-      <c r="H9" s="62"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="65"/>
       <c r="I9" s="18" t="s">
         <v>62</v>
       </c>
@@ -2420,16 +2342,16 @@
       <c r="O9" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="P9" s="69" t="s">
+      <c r="P9" s="72" t="s">
         <v>83</v>
       </c>
-      <c r="Q9" s="69"/>
-      <c r="R9" s="69"/>
-      <c r="S9" s="69"/>
-      <c r="T9" s="69"/>
-      <c r="U9" s="69"/>
-      <c r="V9" s="69"/>
-      <c r="W9" s="69"/>
+      <c r="Q9" s="72"/>
+      <c r="R9" s="72"/>
+      <c r="S9" s="72"/>
+      <c r="T9" s="72"/>
+      <c r="U9" s="72"/>
+      <c r="V9" s="72"/>
+      <c r="W9" s="72"/>
       <c r="X9" s="26" t="s">
         <v>78</v>
       </c>
@@ -2445,14 +2367,14 @@
       <c r="K10" s="5"/>
       <c r="M10" s="4"/>
       <c r="O10" s="27"/>
-      <c r="P10" s="70"/>
-      <c r="Q10" s="70"/>
-      <c r="R10" s="70"/>
-      <c r="S10" s="70"/>
-      <c r="T10" s="70"/>
-      <c r="U10" s="70"/>
-      <c r="V10" s="70"/>
-      <c r="W10" s="70"/>
+      <c r="P10" s="73"/>
+      <c r="Q10" s="73"/>
+      <c r="R10" s="73"/>
+      <c r="S10" s="73"/>
+      <c r="T10" s="73"/>
+      <c r="U10" s="73"/>
+      <c r="V10" s="73"/>
+      <c r="W10" s="73"/>
       <c r="X10" s="28"/>
       <c r="Z10" s="5"/>
       <c r="AB10" s="4"/>
@@ -2466,12 +2388,12 @@
       <c r="D11" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="60" t="s">
+      <c r="E11" s="63" t="s">
         <v>67</v>
       </c>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
       <c r="I11" s="15" t="s">
         <v>59</v>
       </c>
@@ -2483,14 +2405,14 @@
       <c r="O11" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P11" s="71"/>
-      <c r="Q11" s="71"/>
-      <c r="R11" s="71"/>
-      <c r="S11" s="71"/>
-      <c r="T11" s="71"/>
-      <c r="U11" s="71"/>
-      <c r="V11" s="71"/>
-      <c r="W11" s="71"/>
+      <c r="P11" s="74"/>
+      <c r="Q11" s="74"/>
+      <c r="R11" s="74"/>
+      <c r="S11" s="74"/>
+      <c r="T11" s="74"/>
+      <c r="U11" s="74"/>
+      <c r="V11" s="74"/>
+      <c r="W11" s="74"/>
       <c r="X11" s="30" t="s">
         <v>79</v>
       </c>
@@ -2509,10 +2431,10 @@
       <c r="D12" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="64"/>
+      <c r="H12" s="64"/>
       <c r="I12" s="16" t="s">
         <v>60</v>
       </c>
@@ -2525,10 +2447,10 @@
     <row r="13" spans="2:42" x14ac:dyDescent="0.45">
       <c r="B13" s="4"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="61"/>
-      <c r="F13" s="61"/>
-      <c r="G13" s="61"/>
-      <c r="H13" s="61"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="64"/>
+      <c r="H13" s="64"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
       <c r="M13" s="4"/>
@@ -2538,16 +2460,16 @@
       <c r="O13" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="P13" s="69" t="s">
+      <c r="P13" s="72" t="s">
         <v>86</v>
       </c>
-      <c r="Q13" s="69"/>
-      <c r="R13" s="69"/>
-      <c r="S13" s="69"/>
-      <c r="T13" s="69"/>
-      <c r="U13" s="69"/>
-      <c r="V13" s="69"/>
-      <c r="W13" s="69"/>
+      <c r="Q13" s="72"/>
+      <c r="R13" s="72"/>
+      <c r="S13" s="72"/>
+      <c r="T13" s="72"/>
+      <c r="U13" s="72"/>
+      <c r="V13" s="72"/>
+      <c r="W13" s="72"/>
       <c r="X13" s="26" t="s">
         <v>78</v>
       </c>
@@ -2566,10 +2488,10 @@
       <c r="D14" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E14" s="61"/>
-      <c r="F14" s="61"/>
-      <c r="G14" s="61"/>
-      <c r="H14" s="61"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="64"/>
+      <c r="H14" s="64"/>
       <c r="I14" s="17" t="s">
         <v>61</v>
       </c>
@@ -2579,14 +2501,14 @@
       <c r="K14" s="5"/>
       <c r="M14" s="4"/>
       <c r="O14" s="27"/>
-      <c r="P14" s="70"/>
-      <c r="Q14" s="70"/>
-      <c r="R14" s="70"/>
-      <c r="S14" s="70"/>
-      <c r="T14" s="70"/>
-      <c r="U14" s="70"/>
-      <c r="V14" s="70"/>
-      <c r="W14" s="70"/>
+      <c r="P14" s="73"/>
+      <c r="Q14" s="73"/>
+      <c r="R14" s="73"/>
+      <c r="S14" s="73"/>
+      <c r="T14" s="73"/>
+      <c r="U14" s="73"/>
+      <c r="V14" s="73"/>
+      <c r="W14" s="73"/>
       <c r="X14" s="28"/>
       <c r="Z14" s="5"/>
       <c r="AB14" s="4"/>
@@ -2600,10 +2522,10 @@
       <c r="D15" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E15" s="62"/>
-      <c r="F15" s="62"/>
-      <c r="G15" s="62"/>
-      <c r="H15" s="62"/>
+      <c r="E15" s="65"/>
+      <c r="F15" s="65"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="65"/>
       <c r="I15" s="18" t="s">
         <v>62</v>
       </c>
@@ -2618,14 +2540,14 @@
       <c r="O15" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P15" s="71"/>
-      <c r="Q15" s="71"/>
-      <c r="R15" s="71"/>
-      <c r="S15" s="71"/>
-      <c r="T15" s="71"/>
-      <c r="U15" s="71"/>
-      <c r="V15" s="71"/>
-      <c r="W15" s="71"/>
+      <c r="P15" s="74"/>
+      <c r="Q15" s="74"/>
+      <c r="R15" s="74"/>
+      <c r="S15" s="74"/>
+      <c r="T15" s="74"/>
+      <c r="U15" s="74"/>
+      <c r="V15" s="74"/>
+      <c r="W15" s="74"/>
       <c r="X15" s="30" t="s">
         <v>79</v>
       </c>
@@ -2659,12 +2581,12 @@
       <c r="D17" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E17" s="60" t="s">
+      <c r="E17" s="63" t="s">
         <v>70</v>
       </c>
-      <c r="F17" s="60"/>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
+      <c r="F17" s="63"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="63"/>
       <c r="I17" s="15" t="s">
         <v>59</v>
       </c>
@@ -2676,16 +2598,16 @@
       <c r="O17" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="P17" s="69" t="s">
+      <c r="P17" s="72" t="s">
         <v>87</v>
       </c>
-      <c r="Q17" s="69"/>
-      <c r="R17" s="69"/>
-      <c r="S17" s="69"/>
-      <c r="T17" s="69"/>
-      <c r="U17" s="69"/>
-      <c r="V17" s="69"/>
-      <c r="W17" s="69"/>
+      <c r="Q17" s="72"/>
+      <c r="R17" s="72"/>
+      <c r="S17" s="72"/>
+      <c r="T17" s="72"/>
+      <c r="U17" s="72"/>
+      <c r="V17" s="72"/>
+      <c r="W17" s="72"/>
       <c r="X17" s="26" t="s">
         <v>78</v>
       </c>
@@ -2702,45 +2624,45 @@
       <c r="D18" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E18" s="61"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="64"/>
+      <c r="H18" s="64"/>
       <c r="I18" s="16" t="s">
         <v>60</v>
       </c>
       <c r="K18" s="5"/>
       <c r="M18" s="4"/>
       <c r="O18" s="27"/>
-      <c r="P18" s="70"/>
-      <c r="Q18" s="70"/>
-      <c r="R18" s="70"/>
-      <c r="S18" s="70"/>
-      <c r="T18" s="70"/>
-      <c r="U18" s="70"/>
-      <c r="V18" s="70"/>
-      <c r="W18" s="70"/>
+      <c r="P18" s="73"/>
+      <c r="Q18" s="73"/>
+      <c r="R18" s="73"/>
+      <c r="S18" s="73"/>
+      <c r="T18" s="73"/>
+      <c r="U18" s="73"/>
+      <c r="V18" s="73"/>
+      <c r="W18" s="73"/>
       <c r="X18" s="28"/>
       <c r="Z18" s="5"/>
-      <c r="AB18" s="63" t="s">
+      <c r="AB18" s="66" t="s">
         <v>101</v>
       </c>
-      <c r="AC18" s="64"/>
-      <c r="AD18" s="64"/>
-      <c r="AE18" s="64"/>
-      <c r="AF18" s="64"/>
-      <c r="AG18" s="64"/>
-      <c r="AH18" s="64"/>
-      <c r="AI18" s="64"/>
-      <c r="AJ18" s="65"/>
+      <c r="AC18" s="67"/>
+      <c r="AD18" s="67"/>
+      <c r="AE18" s="67"/>
+      <c r="AF18" s="67"/>
+      <c r="AG18" s="67"/>
+      <c r="AH18" s="67"/>
+      <c r="AI18" s="67"/>
+      <c r="AJ18" s="68"/>
     </row>
     <row r="19" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="4"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="61"/>
-      <c r="F19" s="61"/>
-      <c r="G19" s="61"/>
-      <c r="H19" s="61"/>
+      <c r="E19" s="64"/>
+      <c r="F19" s="64"/>
+      <c r="G19" s="64"/>
+      <c r="H19" s="64"/>
       <c r="I19" s="5"/>
       <c r="K19" s="5"/>
       <c r="M19" s="4"/>
@@ -2750,14 +2672,14 @@
       <c r="O19" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P19" s="71"/>
-      <c r="Q19" s="71"/>
-      <c r="R19" s="71"/>
-      <c r="S19" s="71"/>
-      <c r="T19" s="71"/>
-      <c r="U19" s="71"/>
-      <c r="V19" s="71"/>
-      <c r="W19" s="71"/>
+      <c r="P19" s="74"/>
+      <c r="Q19" s="74"/>
+      <c r="R19" s="74"/>
+      <c r="S19" s="74"/>
+      <c r="T19" s="74"/>
+      <c r="U19" s="74"/>
+      <c r="V19" s="74"/>
+      <c r="W19" s="74"/>
       <c r="X19" s="30" t="s">
         <v>79</v>
       </c>
@@ -2783,10 +2705,10 @@
       <c r="D20" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="61"/>
-      <c r="H20" s="61"/>
+      <c r="E20" s="64"/>
+      <c r="F20" s="64"/>
+      <c r="G20" s="64"/>
+      <c r="H20" s="64"/>
       <c r="I20" s="17" t="s">
         <v>61</v>
       </c>
@@ -2803,11 +2725,11 @@
       <c r="AD20" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="AE20" s="66" t="s">
+      <c r="AE20" s="69" t="s">
         <v>97</v>
       </c>
-      <c r="AF20" s="66"/>
-      <c r="AG20" s="66"/>
+      <c r="AF20" s="69"/>
+      <c r="AG20" s="69"/>
       <c r="AH20" s="3"/>
       <c r="AJ20" s="5"/>
     </row>
@@ -2819,10 +2741,10 @@
       <c r="D21" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E21" s="62"/>
-      <c r="F21" s="62"/>
-      <c r="G21" s="62"/>
-      <c r="H21" s="62"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="65"/>
+      <c r="G21" s="65"/>
+      <c r="H21" s="65"/>
       <c r="I21" s="18" t="s">
         <v>62</v>
       </c>
@@ -2835,9 +2757,9 @@
       <c r="AB21" s="4"/>
       <c r="AC21" s="42"/>
       <c r="AD21" s="36"/>
-      <c r="AE21" s="67"/>
-      <c r="AF21" s="67"/>
-      <c r="AG21" s="67"/>
+      <c r="AE21" s="70"/>
+      <c r="AF21" s="70"/>
+      <c r="AG21" s="70"/>
       <c r="AH21" s="44" t="s">
         <v>99</v>
       </c>
@@ -2858,9 +2780,9 @@
       <c r="AD22" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="AE22" s="68"/>
-      <c r="AF22" s="68"/>
-      <c r="AG22" s="68"/>
+      <c r="AE22" s="71"/>
+      <c r="AF22" s="71"/>
+      <c r="AG22" s="71"/>
       <c r="AH22" s="8"/>
       <c r="AJ22" s="5"/>
     </row>
@@ -2872,12 +2794,12 @@
       <c r="D23" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E23" s="60" t="s">
+      <c r="E23" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
+      <c r="F23" s="63"/>
+      <c r="G23" s="63"/>
+      <c r="H23" s="63"/>
       <c r="I23" s="15" t="s">
         <v>59</v>
       </c>
@@ -2895,10 +2817,10 @@
       <c r="D24" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="61"/>
-      <c r="F24" s="61"/>
-      <c r="G24" s="61"/>
-      <c r="H24" s="61"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
+      <c r="G24" s="64"/>
+      <c r="H24" s="64"/>
       <c r="I24" s="16" t="s">
         <v>60</v>
       </c>
@@ -2912,21 +2834,21 @@
       <c r="AD24" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="AE24" s="66" t="s">
+      <c r="AE24" s="69" t="s">
         <v>98</v>
       </c>
-      <c r="AF24" s="66"/>
-      <c r="AG24" s="66"/>
+      <c r="AF24" s="69"/>
+      <c r="AG24" s="69"/>
       <c r="AH24" s="3"/>
       <c r="AJ24" s="5"/>
     </row>
     <row r="25" spans="2:36" ht="19.5" x14ac:dyDescent="0.6">
       <c r="B25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="61"/>
-      <c r="F25" s="61"/>
-      <c r="G25" s="61"/>
-      <c r="H25" s="61"/>
+      <c r="E25" s="64"/>
+      <c r="F25" s="64"/>
+      <c r="G25" s="64"/>
+      <c r="H25" s="64"/>
       <c r="I25" s="5"/>
       <c r="K25" s="5"/>
       <c r="M25" s="4"/>
@@ -2934,9 +2856,9 @@
       <c r="AB25" s="4"/>
       <c r="AC25" s="42"/>
       <c r="AD25" s="36"/>
-      <c r="AE25" s="67"/>
-      <c r="AF25" s="67"/>
-      <c r="AG25" s="67"/>
+      <c r="AE25" s="70"/>
+      <c r="AF25" s="70"/>
+      <c r="AG25" s="70"/>
       <c r="AH25" s="44" t="s">
         <v>99</v>
       </c>
@@ -2953,10 +2875,10 @@
       <c r="D26" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E26" s="61"/>
-      <c r="F26" s="61"/>
-      <c r="G26" s="61"/>
-      <c r="H26" s="61"/>
+      <c r="E26" s="64"/>
+      <c r="F26" s="64"/>
+      <c r="G26" s="64"/>
+      <c r="H26" s="64"/>
       <c r="I26" s="17" t="s">
         <v>61</v>
       </c>
@@ -2973,9 +2895,9 @@
       <c r="AD26" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="AE26" s="68"/>
-      <c r="AF26" s="68"/>
-      <c r="AG26" s="68"/>
+      <c r="AE26" s="71"/>
+      <c r="AF26" s="71"/>
+      <c r="AG26" s="71"/>
       <c r="AH26" s="8"/>
       <c r="AJ26" s="5"/>
     </row>
@@ -2987,10 +2909,10 @@
       <c r="D27" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E27" s="62"/>
-      <c r="F27" s="62"/>
-      <c r="G27" s="62"/>
-      <c r="H27" s="62"/>
+      <c r="E27" s="65"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="65"/>
+      <c r="H27" s="65"/>
       <c r="I27" s="18" t="s">
         <v>62</v>
       </c>

</xml_diff>

<commit_message>
Added Sweeper control thorugh mechanism controller
</commit_message>
<xml_diff>
--- a/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
+++ b/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_Software\electrical_hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0620D91B-6A3C-490C-A3D9-BEF36FDD429A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20ECBA8-3ADF-47F8-A074-073F4E5230E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Layout" sheetId="1" r:id="rId1"/>
@@ -1059,6 +1059,38 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1077,15 +1109,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1095,29 +1118,6 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1411,26 +1411,26 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:19" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="81" t="s">
+      <c r="B2" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81"/>
-      <c r="I2" s="81"/>
-      <c r="J2" s="81"/>
-      <c r="K2" s="81"/>
-      <c r="L2" s="81"/>
-      <c r="M2" s="81"/>
-      <c r="N2" s="81"/>
-      <c r="O2" s="81"/>
-      <c r="P2" s="81"/>
-      <c r="Q2" s="81"/>
-      <c r="R2" s="81"/>
-      <c r="S2" s="81"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
+      <c r="P2" s="73"/>
+      <c r="Q2" s="73"/>
+      <c r="R2" s="73"/>
+      <c r="S2" s="73"/>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B3" s="1"/>
@@ -1524,20 +1524,20 @@
       <c r="D6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="77" t="s">
+      <c r="E6" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="77"/>
-      <c r="G6" s="77"/>
-      <c r="H6" s="77"/>
-      <c r="I6" s="77"/>
-      <c r="J6" s="77"/>
-      <c r="K6" s="77"/>
-      <c r="L6" s="77"/>
-      <c r="M6" s="77"/>
-      <c r="N6" s="77"/>
-      <c r="O6" s="77"/>
-      <c r="P6" s="77"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="69"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="69"/>
+      <c r="N6" s="69"/>
+      <c r="O6" s="69"/>
+      <c r="P6" s="69"/>
       <c r="Q6" s="10" t="s">
         <v>25</v>
       </c>
@@ -1551,18 +1551,18 @@
       <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="77"/>
-      <c r="F7" s="77"/>
-      <c r="G7" s="77"/>
-      <c r="H7" s="77"/>
-      <c r="I7" s="77"/>
-      <c r="J7" s="77"/>
-      <c r="K7" s="77"/>
-      <c r="L7" s="77"/>
-      <c r="M7" s="77"/>
-      <c r="N7" s="77"/>
-      <c r="O7" s="77"/>
-      <c r="P7" s="77"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="69"/>
+      <c r="H7" s="69"/>
+      <c r="I7" s="69"/>
+      <c r="J7" s="69"/>
+      <c r="K7" s="69"/>
+      <c r="L7" s="69"/>
+      <c r="M7" s="69"/>
+      <c r="N7" s="69"/>
+      <c r="O7" s="69"/>
+      <c r="P7" s="69"/>
       <c r="Q7" s="10" t="s">
         <v>26</v>
       </c>
@@ -1720,20 +1720,20 @@
       <c r="D13" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="78" t="s">
+      <c r="E13" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="78"/>
-      <c r="G13" s="78"/>
-      <c r="H13" s="78"/>
-      <c r="I13" s="78"/>
-      <c r="J13" s="78"/>
-      <c r="K13" s="78"/>
-      <c r="L13" s="78"/>
-      <c r="M13" s="78"/>
-      <c r="N13" s="78"/>
-      <c r="O13" s="78"/>
-      <c r="P13" s="78"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="70"/>
+      <c r="H13" s="70"/>
+      <c r="I13" s="70"/>
+      <c r="J13" s="70"/>
+      <c r="K13" s="70"/>
+      <c r="L13" s="70"/>
+      <c r="M13" s="70"/>
+      <c r="N13" s="70"/>
+      <c r="O13" s="70"/>
+      <c r="P13" s="70"/>
       <c r="Q13" s="11" t="s">
         <v>25</v>
       </c>
@@ -1747,18 +1747,18 @@
       <c r="D14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="78"/>
-      <c r="F14" s="78"/>
-      <c r="G14" s="78"/>
-      <c r="H14" s="78"/>
-      <c r="I14" s="78"/>
-      <c r="J14" s="78"/>
-      <c r="K14" s="78"/>
-      <c r="L14" s="78"/>
-      <c r="M14" s="78"/>
-      <c r="N14" s="78"/>
-      <c r="O14" s="78"/>
-      <c r="P14" s="78"/>
+      <c r="E14" s="70"/>
+      <c r="F14" s="70"/>
+      <c r="G14" s="70"/>
+      <c r="H14" s="70"/>
+      <c r="I14" s="70"/>
+      <c r="J14" s="70"/>
+      <c r="K14" s="70"/>
+      <c r="L14" s="70"/>
+      <c r="M14" s="70"/>
+      <c r="N14" s="70"/>
+      <c r="O14" s="70"/>
+      <c r="P14" s="70"/>
       <c r="Q14" s="11" t="s">
         <v>26</v>
       </c>
@@ -1916,20 +1916,20 @@
       <c r="D20" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="79" t="s">
+      <c r="E20" s="71" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="78"/>
-      <c r="G20" s="78"/>
-      <c r="H20" s="78"/>
-      <c r="I20" s="78"/>
-      <c r="J20" s="78"/>
-      <c r="K20" s="78"/>
-      <c r="L20" s="78"/>
-      <c r="M20" s="78"/>
-      <c r="N20" s="78"/>
-      <c r="O20" s="78"/>
-      <c r="P20" s="80"/>
+      <c r="F20" s="70"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="70"/>
+      <c r="I20" s="70"/>
+      <c r="J20" s="70"/>
+      <c r="K20" s="70"/>
+      <c r="L20" s="70"/>
+      <c r="M20" s="70"/>
+      <c r="N20" s="70"/>
+      <c r="O20" s="70"/>
+      <c r="P20" s="72"/>
       <c r="Q20" s="11" t="s">
         <v>25</v>
       </c>
@@ -1943,18 +1943,18 @@
       <c r="D21" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="79"/>
-      <c r="F21" s="78"/>
-      <c r="G21" s="78"/>
-      <c r="H21" s="78"/>
-      <c r="I21" s="78"/>
-      <c r="J21" s="78"/>
-      <c r="K21" s="78"/>
-      <c r="L21" s="78"/>
-      <c r="M21" s="78"/>
-      <c r="N21" s="78"/>
-      <c r="O21" s="78"/>
-      <c r="P21" s="80"/>
+      <c r="E21" s="71"/>
+      <c r="F21" s="70"/>
+      <c r="G21" s="70"/>
+      <c r="H21" s="70"/>
+      <c r="I21" s="70"/>
+      <c r="J21" s="70"/>
+      <c r="K21" s="70"/>
+      <c r="L21" s="70"/>
+      <c r="M21" s="70"/>
+      <c r="N21" s="70"/>
+      <c r="O21" s="70"/>
+      <c r="P21" s="72"/>
       <c r="Q21" s="11" t="s">
         <v>26</v>
       </c>
@@ -2083,45 +2083,45 @@
   <sheetData>
     <row r="2" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:42" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="80" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="J3" s="69"/>
-      <c r="K3" s="70"/>
-      <c r="M3" s="68" t="s">
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="82"/>
+      <c r="M3" s="80" t="s">
         <v>74</v>
       </c>
-      <c r="N3" s="69"/>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="69"/>
-      <c r="S3" s="69"/>
-      <c r="T3" s="69"/>
-      <c r="U3" s="69"/>
-      <c r="V3" s="69"/>
-      <c r="W3" s="69"/>
-      <c r="X3" s="69"/>
-      <c r="Y3" s="69"/>
-      <c r="Z3" s="70"/>
-      <c r="AB3" s="68" t="s">
+      <c r="N3" s="81"/>
+      <c r="O3" s="81"/>
+      <c r="P3" s="81"/>
+      <c r="Q3" s="81"/>
+      <c r="R3" s="81"/>
+      <c r="S3" s="81"/>
+      <c r="T3" s="81"/>
+      <c r="U3" s="81"/>
+      <c r="V3" s="81"/>
+      <c r="W3" s="81"/>
+      <c r="X3" s="81"/>
+      <c r="Y3" s="81"/>
+      <c r="Z3" s="82"/>
+      <c r="AB3" s="80" t="s">
         <v>91</v>
       </c>
-      <c r="AC3" s="69"/>
-      <c r="AD3" s="69"/>
-      <c r="AE3" s="69"/>
-      <c r="AF3" s="69"/>
-      <c r="AG3" s="69"/>
-      <c r="AH3" s="69"/>
-      <c r="AI3" s="69"/>
-      <c r="AJ3" s="70"/>
+      <c r="AC3" s="81"/>
+      <c r="AD3" s="81"/>
+      <c r="AE3" s="81"/>
+      <c r="AF3" s="81"/>
+      <c r="AG3" s="81"/>
+      <c r="AH3" s="81"/>
+      <c r="AI3" s="81"/>
+      <c r="AJ3" s="82"/>
       <c r="AK3" s="33"/>
       <c r="AL3" s="33"/>
       <c r="AM3" s="33"/>
@@ -2172,12 +2172,12 @@
       <c r="D5" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="65" t="s">
+      <c r="E5" s="77" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="65"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
       <c r="I5" s="15" t="s">
         <v>57</v>
       </c>
@@ -2189,16 +2189,16 @@
       <c r="O5" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P5" s="74" t="s">
+      <c r="P5" s="83" t="s">
         <v>78</v>
       </c>
-      <c r="Q5" s="74"/>
-      <c r="R5" s="74"/>
-      <c r="S5" s="74"/>
-      <c r="T5" s="74"/>
-      <c r="U5" s="74"/>
-      <c r="V5" s="74"/>
-      <c r="W5" s="74"/>
+      <c r="Q5" s="83"/>
+      <c r="R5" s="83"/>
+      <c r="S5" s="83"/>
+      <c r="T5" s="83"/>
+      <c r="U5" s="83"/>
+      <c r="V5" s="83"/>
+      <c r="W5" s="83"/>
       <c r="X5" s="26" t="s">
         <v>76</v>
       </c>
@@ -2213,11 +2213,11 @@
       <c r="AD5" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AE5" s="71" t="s">
+      <c r="AE5" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="AF5" s="71"/>
-      <c r="AG5" s="71"/>
+      <c r="AF5" s="74"/>
+      <c r="AG5" s="74"/>
       <c r="AH5" s="35" t="s">
         <v>93</v>
       </c>
@@ -2234,32 +2234,32 @@
       <c r="D6" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
+      <c r="E6" s="78"/>
+      <c r="F6" s="78"/>
+      <c r="G6" s="78"/>
+      <c r="H6" s="78"/>
       <c r="I6" s="16" t="s">
         <v>58</v>
       </c>
       <c r="K6" s="5"/>
       <c r="M6" s="4"/>
       <c r="O6" s="27"/>
-      <c r="P6" s="75"/>
-      <c r="Q6" s="75"/>
-      <c r="R6" s="75"/>
-      <c r="S6" s="75"/>
-      <c r="T6" s="75"/>
-      <c r="U6" s="75"/>
-      <c r="V6" s="75"/>
-      <c r="W6" s="75"/>
+      <c r="P6" s="84"/>
+      <c r="Q6" s="84"/>
+      <c r="R6" s="84"/>
+      <c r="S6" s="84"/>
+      <c r="T6" s="84"/>
+      <c r="U6" s="84"/>
+      <c r="V6" s="84"/>
+      <c r="W6" s="84"/>
       <c r="X6" s="28"/>
       <c r="Z6" s="5"/>
       <c r="AB6" s="4"/>
       <c r="AC6" s="42"/>
       <c r="AD6" s="36"/>
-      <c r="AE6" s="72"/>
-      <c r="AF6" s="72"/>
-      <c r="AG6" s="72"/>
+      <c r="AE6" s="75"/>
+      <c r="AF6" s="75"/>
+      <c r="AG6" s="75"/>
       <c r="AH6" s="37"/>
       <c r="AI6" s="41"/>
       <c r="AJ6" s="5"/>
@@ -2267,10 +2267,10 @@
     <row r="7" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="4"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="66"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="66"/>
-      <c r="H7" s="66"/>
+      <c r="E7" s="78"/>
+      <c r="F7" s="78"/>
+      <c r="G7" s="78"/>
+      <c r="H7" s="78"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
       <c r="M7" s="4"/>
@@ -2280,14 +2280,14 @@
       <c r="O7" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P7" s="76"/>
-      <c r="Q7" s="76"/>
-      <c r="R7" s="76"/>
-      <c r="S7" s="76"/>
-      <c r="T7" s="76"/>
-      <c r="U7" s="76"/>
-      <c r="V7" s="76"/>
-      <c r="W7" s="76"/>
+      <c r="P7" s="85"/>
+      <c r="Q7" s="85"/>
+      <c r="R7" s="85"/>
+      <c r="S7" s="85"/>
+      <c r="T7" s="85"/>
+      <c r="U7" s="85"/>
+      <c r="V7" s="85"/>
+      <c r="W7" s="85"/>
       <c r="X7" s="30" t="s">
         <v>77</v>
       </c>
@@ -2302,9 +2302,9 @@
       <c r="AD7" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="AE7" s="73"/>
-      <c r="AF7" s="73"/>
-      <c r="AG7" s="73"/>
+      <c r="AE7" s="76"/>
+      <c r="AF7" s="76"/>
+      <c r="AG7" s="76"/>
       <c r="AH7" s="39" t="s">
         <v>94</v>
       </c>
@@ -2321,10 +2321,10 @@
       <c r="D8" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="66"/>
-      <c r="F8" s="66"/>
-      <c r="G8" s="66"/>
-      <c r="H8" s="66"/>
+      <c r="E8" s="78"/>
+      <c r="F8" s="78"/>
+      <c r="G8" s="78"/>
+      <c r="H8" s="78"/>
       <c r="I8" s="17" t="s">
         <v>59</v>
       </c>
@@ -2345,10 +2345,10 @@
       <c r="D9" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="67"/>
-      <c r="F9" s="67"/>
-      <c r="G9" s="67"/>
-      <c r="H9" s="67"/>
+      <c r="E9" s="79"/>
+      <c r="F9" s="79"/>
+      <c r="G9" s="79"/>
+      <c r="H9" s="79"/>
       <c r="I9" s="18" t="s">
         <v>60</v>
       </c>
@@ -2363,16 +2363,16 @@
       <c r="O9" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P9" s="74" t="s">
+      <c r="P9" s="83" t="s">
         <v>81</v>
       </c>
-      <c r="Q9" s="74"/>
-      <c r="R9" s="74"/>
-      <c r="S9" s="74"/>
-      <c r="T9" s="74"/>
-      <c r="U9" s="74"/>
-      <c r="V9" s="74"/>
-      <c r="W9" s="74"/>
+      <c r="Q9" s="83"/>
+      <c r="R9" s="83"/>
+      <c r="S9" s="83"/>
+      <c r="T9" s="83"/>
+      <c r="U9" s="83"/>
+      <c r="V9" s="83"/>
+      <c r="W9" s="83"/>
       <c r="X9" s="26" t="s">
         <v>76</v>
       </c>
@@ -2388,14 +2388,14 @@
       <c r="K10" s="5"/>
       <c r="M10" s="4"/>
       <c r="O10" s="27"/>
-      <c r="P10" s="75"/>
-      <c r="Q10" s="75"/>
-      <c r="R10" s="75"/>
-      <c r="S10" s="75"/>
-      <c r="T10" s="75"/>
-      <c r="U10" s="75"/>
-      <c r="V10" s="75"/>
-      <c r="W10" s="75"/>
+      <c r="P10" s="84"/>
+      <c r="Q10" s="84"/>
+      <c r="R10" s="84"/>
+      <c r="S10" s="84"/>
+      <c r="T10" s="84"/>
+      <c r="U10" s="84"/>
+      <c r="V10" s="84"/>
+      <c r="W10" s="84"/>
       <c r="X10" s="28"/>
       <c r="Z10" s="5"/>
       <c r="AB10" s="4"/>
@@ -2409,12 +2409,12 @@
       <c r="D11" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="65" t="s">
+      <c r="E11" s="77" t="s">
         <v>65</v>
       </c>
-      <c r="F11" s="65"/>
-      <c r="G11" s="65"/>
-      <c r="H11" s="65"/>
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
       <c r="I11" s="15" t="s">
         <v>57</v>
       </c>
@@ -2426,14 +2426,14 @@
       <c r="O11" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P11" s="76"/>
-      <c r="Q11" s="76"/>
-      <c r="R11" s="76"/>
-      <c r="S11" s="76"/>
-      <c r="T11" s="76"/>
-      <c r="U11" s="76"/>
-      <c r="V11" s="76"/>
-      <c r="W11" s="76"/>
+      <c r="P11" s="85"/>
+      <c r="Q11" s="85"/>
+      <c r="R11" s="85"/>
+      <c r="S11" s="85"/>
+      <c r="T11" s="85"/>
+      <c r="U11" s="85"/>
+      <c r="V11" s="85"/>
+      <c r="W11" s="85"/>
       <c r="X11" s="30" t="s">
         <v>77</v>
       </c>
@@ -2452,10 +2452,10 @@
       <c r="D12" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="66"/>
-      <c r="F12" s="66"/>
-      <c r="G12" s="66"/>
-      <c r="H12" s="66"/>
+      <c r="E12" s="78"/>
+      <c r="F12" s="78"/>
+      <c r="G12" s="78"/>
+      <c r="H12" s="78"/>
       <c r="I12" s="16" t="s">
         <v>58</v>
       </c>
@@ -2468,10 +2468,10 @@
     <row r="13" spans="2:42" x14ac:dyDescent="0.45">
       <c r="B13" s="4"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="66"/>
-      <c r="F13" s="66"/>
-      <c r="G13" s="66"/>
-      <c r="H13" s="66"/>
+      <c r="E13" s="78"/>
+      <c r="F13" s="78"/>
+      <c r="G13" s="78"/>
+      <c r="H13" s="78"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
       <c r="M13" s="4"/>
@@ -2481,16 +2481,16 @@
       <c r="O13" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P13" s="74" t="s">
+      <c r="P13" s="83" t="s">
         <v>84</v>
       </c>
-      <c r="Q13" s="74"/>
-      <c r="R13" s="74"/>
-      <c r="S13" s="74"/>
-      <c r="T13" s="74"/>
-      <c r="U13" s="74"/>
-      <c r="V13" s="74"/>
-      <c r="W13" s="74"/>
+      <c r="Q13" s="83"/>
+      <c r="R13" s="83"/>
+      <c r="S13" s="83"/>
+      <c r="T13" s="83"/>
+      <c r="U13" s="83"/>
+      <c r="V13" s="83"/>
+      <c r="W13" s="83"/>
       <c r="X13" s="26" t="s">
         <v>76</v>
       </c>
@@ -2509,10 +2509,10 @@
       <c r="D14" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="66"/>
-      <c r="H14" s="66"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="78"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="78"/>
       <c r="I14" s="17" t="s">
         <v>59</v>
       </c>
@@ -2522,14 +2522,14 @@
       <c r="K14" s="5"/>
       <c r="M14" s="4"/>
       <c r="O14" s="27"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="75"/>
-      <c r="R14" s="75"/>
-      <c r="S14" s="75"/>
-      <c r="T14" s="75"/>
-      <c r="U14" s="75"/>
-      <c r="V14" s="75"/>
-      <c r="W14" s="75"/>
+      <c r="P14" s="84"/>
+      <c r="Q14" s="84"/>
+      <c r="R14" s="84"/>
+      <c r="S14" s="84"/>
+      <c r="T14" s="84"/>
+      <c r="U14" s="84"/>
+      <c r="V14" s="84"/>
+      <c r="W14" s="84"/>
       <c r="X14" s="28"/>
       <c r="Z14" s="5"/>
       <c r="AB14" s="4"/>
@@ -2543,10 +2543,10 @@
       <c r="D15" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="67"/>
+      <c r="E15" s="79"/>
+      <c r="F15" s="79"/>
+      <c r="G15" s="79"/>
+      <c r="H15" s="79"/>
       <c r="I15" s="18" t="s">
         <v>60</v>
       </c>
@@ -2561,14 +2561,14 @@
       <c r="O15" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P15" s="76"/>
-      <c r="Q15" s="76"/>
-      <c r="R15" s="76"/>
-      <c r="S15" s="76"/>
-      <c r="T15" s="76"/>
-      <c r="U15" s="76"/>
-      <c r="V15" s="76"/>
-      <c r="W15" s="76"/>
+      <c r="P15" s="85"/>
+      <c r="Q15" s="85"/>
+      <c r="R15" s="85"/>
+      <c r="S15" s="85"/>
+      <c r="T15" s="85"/>
+      <c r="U15" s="85"/>
+      <c r="V15" s="85"/>
+      <c r="W15" s="85"/>
       <c r="X15" s="30" t="s">
         <v>77</v>
       </c>
@@ -2602,12 +2602,12 @@
       <c r="D17" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="65" t="s">
+      <c r="E17" s="77" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="65"/>
-      <c r="G17" s="65"/>
-      <c r="H17" s="65"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
       <c r="I17" s="15" t="s">
         <v>57</v>
       </c>
@@ -2619,16 +2619,16 @@
       <c r="O17" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P17" s="74" t="s">
+      <c r="P17" s="83" t="s">
         <v>85</v>
       </c>
-      <c r="Q17" s="74"/>
-      <c r="R17" s="74"/>
-      <c r="S17" s="74"/>
-      <c r="T17" s="74"/>
-      <c r="U17" s="74"/>
-      <c r="V17" s="74"/>
-      <c r="W17" s="74"/>
+      <c r="Q17" s="83"/>
+      <c r="R17" s="83"/>
+      <c r="S17" s="83"/>
+      <c r="T17" s="83"/>
+      <c r="U17" s="83"/>
+      <c r="V17" s="83"/>
+      <c r="W17" s="83"/>
       <c r="X17" s="26" t="s">
         <v>76</v>
       </c>
@@ -2645,45 +2645,45 @@
       <c r="D18" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="66"/>
-      <c r="F18" s="66"/>
-      <c r="G18" s="66"/>
-      <c r="H18" s="66"/>
+      <c r="E18" s="78"/>
+      <c r="F18" s="78"/>
+      <c r="G18" s="78"/>
+      <c r="H18" s="78"/>
       <c r="I18" s="16" t="s">
         <v>58</v>
       </c>
       <c r="K18" s="5"/>
       <c r="M18" s="4"/>
       <c r="O18" s="27"/>
-      <c r="P18" s="75"/>
-      <c r="Q18" s="75"/>
-      <c r="R18" s="75"/>
-      <c r="S18" s="75"/>
-      <c r="T18" s="75"/>
-      <c r="U18" s="75"/>
-      <c r="V18" s="75"/>
-      <c r="W18" s="75"/>
+      <c r="P18" s="84"/>
+      <c r="Q18" s="84"/>
+      <c r="R18" s="84"/>
+      <c r="S18" s="84"/>
+      <c r="T18" s="84"/>
+      <c r="U18" s="84"/>
+      <c r="V18" s="84"/>
+      <c r="W18" s="84"/>
       <c r="X18" s="28"/>
       <c r="Z18" s="5"/>
-      <c r="AB18" s="68" t="s">
+      <c r="AB18" s="80" t="s">
         <v>98</v>
       </c>
-      <c r="AC18" s="69"/>
-      <c r="AD18" s="69"/>
-      <c r="AE18" s="69"/>
-      <c r="AF18" s="69"/>
-      <c r="AG18" s="69"/>
-      <c r="AH18" s="69"/>
-      <c r="AI18" s="69"/>
-      <c r="AJ18" s="70"/>
+      <c r="AC18" s="81"/>
+      <c r="AD18" s="81"/>
+      <c r="AE18" s="81"/>
+      <c r="AF18" s="81"/>
+      <c r="AG18" s="81"/>
+      <c r="AH18" s="81"/>
+      <c r="AI18" s="81"/>
+      <c r="AJ18" s="82"/>
     </row>
     <row r="19" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="4"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="66"/>
-      <c r="F19" s="66"/>
-      <c r="G19" s="66"/>
-      <c r="H19" s="66"/>
+      <c r="E19" s="78"/>
+      <c r="F19" s="78"/>
+      <c r="G19" s="78"/>
+      <c r="H19" s="78"/>
       <c r="I19" s="5"/>
       <c r="K19" s="5"/>
       <c r="M19" s="4"/>
@@ -2693,14 +2693,14 @@
       <c r="O19" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P19" s="76"/>
-      <c r="Q19" s="76"/>
-      <c r="R19" s="76"/>
-      <c r="S19" s="76"/>
-      <c r="T19" s="76"/>
-      <c r="U19" s="76"/>
-      <c r="V19" s="76"/>
-      <c r="W19" s="76"/>
+      <c r="P19" s="85"/>
+      <c r="Q19" s="85"/>
+      <c r="R19" s="85"/>
+      <c r="S19" s="85"/>
+      <c r="T19" s="85"/>
+      <c r="U19" s="85"/>
+      <c r="V19" s="85"/>
+      <c r="W19" s="85"/>
       <c r="X19" s="30" t="s">
         <v>77</v>
       </c>
@@ -2726,10 +2726,10 @@
       <c r="D20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="66"/>
-      <c r="F20" s="66"/>
-      <c r="G20" s="66"/>
-      <c r="H20" s="66"/>
+      <c r="E20" s="78"/>
+      <c r="F20" s="78"/>
+      <c r="G20" s="78"/>
+      <c r="H20" s="78"/>
       <c r="I20" s="17" t="s">
         <v>59</v>
       </c>
@@ -2746,11 +2746,11 @@
       <c r="AD20" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AE20" s="71" t="s">
+      <c r="AE20" s="74" t="s">
         <v>95</v>
       </c>
-      <c r="AF20" s="71"/>
-      <c r="AG20" s="71"/>
+      <c r="AF20" s="74"/>
+      <c r="AG20" s="74"/>
       <c r="AH20" s="3"/>
       <c r="AJ20" s="5"/>
     </row>
@@ -2762,10 +2762,10 @@
       <c r="D21" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="67"/>
-      <c r="F21" s="67"/>
-      <c r="G21" s="67"/>
-      <c r="H21" s="67"/>
+      <c r="E21" s="79"/>
+      <c r="F21" s="79"/>
+      <c r="G21" s="79"/>
+      <c r="H21" s="79"/>
       <c r="I21" s="18" t="s">
         <v>60</v>
       </c>
@@ -2778,14 +2778,14 @@
       <c r="AB21" s="4"/>
       <c r="AC21" s="42"/>
       <c r="AD21" s="36"/>
-      <c r="AE21" s="72"/>
-      <c r="AF21" s="72"/>
-      <c r="AG21" s="72"/>
+      <c r="AE21" s="75"/>
+      <c r="AF21" s="75"/>
+      <c r="AG21" s="75"/>
       <c r="AH21" s="44" t="s">
         <v>96</v>
       </c>
       <c r="AI21" s="40" t="s">
-        <v>97</v>
+        <v>1</v>
       </c>
       <c r="AJ21" s="5"/>
     </row>
@@ -2801,9 +2801,9 @@
       <c r="AD22" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="AE22" s="73"/>
-      <c r="AF22" s="73"/>
-      <c r="AG22" s="73"/>
+      <c r="AE22" s="76"/>
+      <c r="AF22" s="76"/>
+      <c r="AG22" s="76"/>
       <c r="AH22" s="8"/>
       <c r="AJ22" s="5"/>
     </row>
@@ -2815,12 +2815,12 @@
       <c r="D23" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="65" t="s">
+      <c r="E23" s="77" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="65"/>
-      <c r="G23" s="65"/>
-      <c r="H23" s="65"/>
+      <c r="F23" s="77"/>
+      <c r="G23" s="77"/>
+      <c r="H23" s="77"/>
       <c r="I23" s="15" t="s">
         <v>57</v>
       </c>
@@ -2838,10 +2838,10 @@
       <c r="D24" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="66"/>
-      <c r="F24" s="66"/>
-      <c r="G24" s="66"/>
-      <c r="H24" s="66"/>
+      <c r="E24" s="78"/>
+      <c r="F24" s="78"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
       <c r="I24" s="16" t="s">
         <v>58</v>
       </c>
@@ -2855,21 +2855,21 @@
       <c r="AD24" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AE24" s="71" t="s">
+      <c r="AE24" s="74" t="s">
         <v>115</v>
       </c>
-      <c r="AF24" s="71"/>
-      <c r="AG24" s="71"/>
+      <c r="AF24" s="74"/>
+      <c r="AG24" s="74"/>
       <c r="AH24" s="3"/>
       <c r="AJ24" s="5"/>
     </row>
     <row r="25" spans="2:36" ht="19.5" x14ac:dyDescent="0.6">
       <c r="B25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="66"/>
-      <c r="F25" s="66"/>
-      <c r="G25" s="66"/>
-      <c r="H25" s="66"/>
+      <c r="E25" s="78"/>
+      <c r="F25" s="78"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="78"/>
       <c r="I25" s="5"/>
       <c r="K25" s="5"/>
       <c r="M25" s="4"/>
@@ -2877,14 +2877,14 @@
       <c r="AB25" s="4"/>
       <c r="AC25" s="42"/>
       <c r="AD25" s="36"/>
-      <c r="AE25" s="72"/>
-      <c r="AF25" s="72"/>
-      <c r="AG25" s="72"/>
+      <c r="AE25" s="75"/>
+      <c r="AF25" s="75"/>
+      <c r="AG25" s="75"/>
       <c r="AH25" s="44" t="s">
         <v>96</v>
       </c>
       <c r="AI25" s="40" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="AJ25" s="5"/>
     </row>
@@ -2896,10 +2896,10 @@
       <c r="D26" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="66"/>
-      <c r="F26" s="66"/>
-      <c r="G26" s="66"/>
-      <c r="H26" s="66"/>
+      <c r="E26" s="78"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
       <c r="I26" s="17" t="s">
         <v>59</v>
       </c>
@@ -2916,9 +2916,9 @@
       <c r="AD26" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="AE26" s="73"/>
-      <c r="AF26" s="73"/>
-      <c r="AG26" s="73"/>
+      <c r="AE26" s="76"/>
+      <c r="AF26" s="76"/>
+      <c r="AG26" s="76"/>
       <c r="AH26" s="8"/>
       <c r="AJ26" s="5"/>
     </row>
@@ -2930,10 +2930,10 @@
       <c r="D27" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E27" s="67"/>
-      <c r="F27" s="67"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="67"/>
+      <c r="E27" s="79"/>
+      <c r="F27" s="79"/>
+      <c r="G27" s="79"/>
+      <c r="H27" s="79"/>
       <c r="I27" s="18" t="s">
         <v>60</v>
       </c>
@@ -2948,14 +2948,14 @@
     </row>
     <row r="28" spans="2:36" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B28" s="4"/>
-      <c r="C28" s="82"/>
-      <c r="D28" s="83"/>
+      <c r="C28" s="65"/>
+      <c r="D28" s="66"/>
       <c r="E28" s="60"/>
       <c r="F28" s="60"/>
       <c r="G28" s="60"/>
       <c r="H28" s="60"/>
-      <c r="I28" s="84"/>
-      <c r="J28" s="85"/>
+      <c r="I28" s="67"/>
+      <c r="J28" s="68"/>
       <c r="K28" s="5"/>
       <c r="M28" s="4"/>
       <c r="Z28" s="5"/>
@@ -2966,33 +2966,33 @@
       <c r="AD28" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AE28" s="71" t="s">
+      <c r="AE28" s="74" t="s">
         <v>114</v>
       </c>
-      <c r="AF28" s="71"/>
-      <c r="AG28" s="71"/>
+      <c r="AF28" s="74"/>
+      <c r="AG28" s="74"/>
       <c r="AH28" s="3"/>
       <c r="AJ28" s="5"/>
     </row>
     <row r="29" spans="2:36" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B29" s="4"/>
-      <c r="C29" s="82"/>
-      <c r="D29" s="83"/>
+      <c r="C29" s="65"/>
+      <c r="D29" s="66"/>
       <c r="E29" s="60"/>
       <c r="F29" s="60"/>
       <c r="G29" s="60"/>
       <c r="H29" s="60"/>
-      <c r="I29" s="84"/>
-      <c r="J29" s="85"/>
+      <c r="I29" s="67"/>
+      <c r="J29" s="68"/>
       <c r="K29" s="5"/>
       <c r="M29" s="4"/>
       <c r="Z29" s="5"/>
       <c r="AB29" s="4"/>
       <c r="AC29" s="42"/>
       <c r="AD29" s="36"/>
-      <c r="AE29" s="72"/>
-      <c r="AF29" s="72"/>
-      <c r="AG29" s="72"/>
+      <c r="AE29" s="75"/>
+      <c r="AF29" s="75"/>
+      <c r="AG29" s="75"/>
       <c r="AH29" s="44" t="s">
         <v>96</v>
       </c>
@@ -3003,14 +3003,14 @@
     </row>
     <row r="30" spans="2:36" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B30" s="4"/>
-      <c r="C30" s="82"/>
-      <c r="D30" s="83"/>
+      <c r="C30" s="65"/>
+      <c r="D30" s="66"/>
       <c r="E30" s="60"/>
       <c r="F30" s="60"/>
       <c r="G30" s="60"/>
       <c r="H30" s="60"/>
-      <c r="I30" s="84"/>
-      <c r="J30" s="85"/>
+      <c r="I30" s="67"/>
+      <c r="J30" s="68"/>
       <c r="K30" s="5"/>
       <c r="M30" s="4"/>
       <c r="Z30" s="5"/>
@@ -3021,9 +3021,9 @@
       <c r="AD30" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="AE30" s="73"/>
-      <c r="AF30" s="73"/>
-      <c r="AG30" s="73"/>
+      <c r="AE30" s="76"/>
+      <c r="AF30" s="76"/>
+      <c r="AG30" s="76"/>
       <c r="AH30" s="8"/>
       <c r="AJ30" s="5"/>
     </row>

</xml_diff>

<commit_message>
Implemented RHS Arm manual Control jog and calibration
</commit_message>
<xml_diff>
--- a/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
+++ b/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
@@ -1067,6 +1067,42 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1080,42 +1116,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1411,26 +1411,26 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:19" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="85" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="73"/>
-      <c r="Q2" s="73"/>
-      <c r="R2" s="73"/>
-      <c r="S2" s="73"/>
+      <c r="C2" s="85"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="85"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
+      <c r="N2" s="85"/>
+      <c r="O2" s="85"/>
+      <c r="P2" s="85"/>
+      <c r="Q2" s="85"/>
+      <c r="R2" s="85"/>
+      <c r="S2" s="85"/>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B3" s="1"/>
@@ -1524,20 +1524,20 @@
       <c r="D6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="69" t="s">
+      <c r="E6" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="69"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="69"/>
-      <c r="I6" s="69"/>
-      <c r="J6" s="69"/>
-      <c r="K6" s="69"/>
-      <c r="L6" s="69"/>
-      <c r="M6" s="69"/>
-      <c r="N6" s="69"/>
-      <c r="O6" s="69"/>
-      <c r="P6" s="69"/>
+      <c r="F6" s="81"/>
+      <c r="G6" s="81"/>
+      <c r="H6" s="81"/>
+      <c r="I6" s="81"/>
+      <c r="J6" s="81"/>
+      <c r="K6" s="81"/>
+      <c r="L6" s="81"/>
+      <c r="M6" s="81"/>
+      <c r="N6" s="81"/>
+      <c r="O6" s="81"/>
+      <c r="P6" s="81"/>
       <c r="Q6" s="10" t="s">
         <v>25</v>
       </c>
@@ -1551,18 +1551,18 @@
       <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="69"/>
-      <c r="F7" s="69"/>
-      <c r="G7" s="69"/>
-      <c r="H7" s="69"/>
-      <c r="I7" s="69"/>
-      <c r="J7" s="69"/>
-      <c r="K7" s="69"/>
-      <c r="L7" s="69"/>
-      <c r="M7" s="69"/>
-      <c r="N7" s="69"/>
-      <c r="O7" s="69"/>
-      <c r="P7" s="69"/>
+      <c r="E7" s="81"/>
+      <c r="F7" s="81"/>
+      <c r="G7" s="81"/>
+      <c r="H7" s="81"/>
+      <c r="I7" s="81"/>
+      <c r="J7" s="81"/>
+      <c r="K7" s="81"/>
+      <c r="L7" s="81"/>
+      <c r="M7" s="81"/>
+      <c r="N7" s="81"/>
+      <c r="O7" s="81"/>
+      <c r="P7" s="81"/>
       <c r="Q7" s="10" t="s">
         <v>26</v>
       </c>
@@ -1720,20 +1720,20 @@
       <c r="D13" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="70" t="s">
+      <c r="E13" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="70"/>
-      <c r="G13" s="70"/>
-      <c r="H13" s="70"/>
-      <c r="I13" s="70"/>
-      <c r="J13" s="70"/>
-      <c r="K13" s="70"/>
-      <c r="L13" s="70"/>
-      <c r="M13" s="70"/>
-      <c r="N13" s="70"/>
-      <c r="O13" s="70"/>
-      <c r="P13" s="70"/>
+      <c r="F13" s="82"/>
+      <c r="G13" s="82"/>
+      <c r="H13" s="82"/>
+      <c r="I13" s="82"/>
+      <c r="J13" s="82"/>
+      <c r="K13" s="82"/>
+      <c r="L13" s="82"/>
+      <c r="M13" s="82"/>
+      <c r="N13" s="82"/>
+      <c r="O13" s="82"/>
+      <c r="P13" s="82"/>
       <c r="Q13" s="11" t="s">
         <v>25</v>
       </c>
@@ -1747,18 +1747,18 @@
       <c r="D14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="70"/>
-      <c r="F14" s="70"/>
-      <c r="G14" s="70"/>
-      <c r="H14" s="70"/>
-      <c r="I14" s="70"/>
-      <c r="J14" s="70"/>
-      <c r="K14" s="70"/>
-      <c r="L14" s="70"/>
-      <c r="M14" s="70"/>
-      <c r="N14" s="70"/>
-      <c r="O14" s="70"/>
-      <c r="P14" s="70"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="82"/>
+      <c r="H14" s="82"/>
+      <c r="I14" s="82"/>
+      <c r="J14" s="82"/>
+      <c r="K14" s="82"/>
+      <c r="L14" s="82"/>
+      <c r="M14" s="82"/>
+      <c r="N14" s="82"/>
+      <c r="O14" s="82"/>
+      <c r="P14" s="82"/>
       <c r="Q14" s="11" t="s">
         <v>26</v>
       </c>
@@ -1916,20 +1916,20 @@
       <c r="D20" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="71" t="s">
+      <c r="E20" s="83" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="70"/>
-      <c r="G20" s="70"/>
-      <c r="H20" s="70"/>
-      <c r="I20" s="70"/>
-      <c r="J20" s="70"/>
-      <c r="K20" s="70"/>
-      <c r="L20" s="70"/>
-      <c r="M20" s="70"/>
-      <c r="N20" s="70"/>
-      <c r="O20" s="70"/>
-      <c r="P20" s="72"/>
+      <c r="F20" s="82"/>
+      <c r="G20" s="82"/>
+      <c r="H20" s="82"/>
+      <c r="I20" s="82"/>
+      <c r="J20" s="82"/>
+      <c r="K20" s="82"/>
+      <c r="L20" s="82"/>
+      <c r="M20" s="82"/>
+      <c r="N20" s="82"/>
+      <c r="O20" s="82"/>
+      <c r="P20" s="84"/>
       <c r="Q20" s="11" t="s">
         <v>25</v>
       </c>
@@ -1943,18 +1943,18 @@
       <c r="D21" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="71"/>
-      <c r="F21" s="70"/>
-      <c r="G21" s="70"/>
-      <c r="H21" s="70"/>
-      <c r="I21" s="70"/>
-      <c r="J21" s="70"/>
-      <c r="K21" s="70"/>
-      <c r="L21" s="70"/>
-      <c r="M21" s="70"/>
-      <c r="N21" s="70"/>
-      <c r="O21" s="70"/>
-      <c r="P21" s="72"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="82"/>
+      <c r="G21" s="82"/>
+      <c r="H21" s="82"/>
+      <c r="I21" s="82"/>
+      <c r="J21" s="82"/>
+      <c r="K21" s="82"/>
+      <c r="L21" s="82"/>
+      <c r="M21" s="82"/>
+      <c r="N21" s="82"/>
+      <c r="O21" s="82"/>
+      <c r="P21" s="84"/>
       <c r="Q21" s="11" t="s">
         <v>26</v>
       </c>
@@ -2083,45 +2083,45 @@
   <sheetData>
     <row r="2" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:42" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B3" s="80" t="s">
+      <c r="B3" s="75" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="81"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="82"/>
-      <c r="M3" s="80" t="s">
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="77"/>
+      <c r="M3" s="75" t="s">
         <v>74</v>
       </c>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="81"/>
-      <c r="R3" s="81"/>
-      <c r="S3" s="81"/>
-      <c r="T3" s="81"/>
-      <c r="U3" s="81"/>
-      <c r="V3" s="81"/>
-      <c r="W3" s="81"/>
-      <c r="X3" s="81"/>
-      <c r="Y3" s="81"/>
-      <c r="Z3" s="82"/>
-      <c r="AB3" s="80" t="s">
+      <c r="N3" s="76"/>
+      <c r="O3" s="76"/>
+      <c r="P3" s="76"/>
+      <c r="Q3" s="76"/>
+      <c r="R3" s="76"/>
+      <c r="S3" s="76"/>
+      <c r="T3" s="76"/>
+      <c r="U3" s="76"/>
+      <c r="V3" s="76"/>
+      <c r="W3" s="76"/>
+      <c r="X3" s="76"/>
+      <c r="Y3" s="76"/>
+      <c r="Z3" s="77"/>
+      <c r="AB3" s="75" t="s">
         <v>91</v>
       </c>
-      <c r="AC3" s="81"/>
-      <c r="AD3" s="81"/>
-      <c r="AE3" s="81"/>
-      <c r="AF3" s="81"/>
-      <c r="AG3" s="81"/>
-      <c r="AH3" s="81"/>
-      <c r="AI3" s="81"/>
-      <c r="AJ3" s="82"/>
+      <c r="AC3" s="76"/>
+      <c r="AD3" s="76"/>
+      <c r="AE3" s="76"/>
+      <c r="AF3" s="76"/>
+      <c r="AG3" s="76"/>
+      <c r="AH3" s="76"/>
+      <c r="AI3" s="76"/>
+      <c r="AJ3" s="77"/>
       <c r="AK3" s="33"/>
       <c r="AL3" s="33"/>
       <c r="AM3" s="33"/>
@@ -2172,12 +2172,12 @@
       <c r="D5" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="77" t="s">
+      <c r="E5" s="72" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="77"/>
-      <c r="G5" s="77"/>
-      <c r="H5" s="77"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="72"/>
+      <c r="H5" s="72"/>
       <c r="I5" s="15" t="s">
         <v>57</v>
       </c>
@@ -2189,16 +2189,16 @@
       <c r="O5" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P5" s="83" t="s">
+      <c r="P5" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="Q5" s="83"/>
-      <c r="R5" s="83"/>
-      <c r="S5" s="83"/>
-      <c r="T5" s="83"/>
-      <c r="U5" s="83"/>
-      <c r="V5" s="83"/>
-      <c r="W5" s="83"/>
+      <c r="Q5" s="78"/>
+      <c r="R5" s="78"/>
+      <c r="S5" s="78"/>
+      <c r="T5" s="78"/>
+      <c r="U5" s="78"/>
+      <c r="V5" s="78"/>
+      <c r="W5" s="78"/>
       <c r="X5" s="26" t="s">
         <v>76</v>
       </c>
@@ -2213,11 +2213,11 @@
       <c r="AD5" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AE5" s="74" t="s">
+      <c r="AE5" s="69" t="s">
         <v>91</v>
       </c>
-      <c r="AF5" s="74"/>
-      <c r="AG5" s="74"/>
+      <c r="AF5" s="69"/>
+      <c r="AG5" s="69"/>
       <c r="AH5" s="35" t="s">
         <v>93</v>
       </c>
@@ -2234,32 +2234,32 @@
       <c r="D6" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="78"/>
-      <c r="F6" s="78"/>
-      <c r="G6" s="78"/>
-      <c r="H6" s="78"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
+      <c r="G6" s="73"/>
+      <c r="H6" s="73"/>
       <c r="I6" s="16" t="s">
         <v>58</v>
       </c>
       <c r="K6" s="5"/>
       <c r="M6" s="4"/>
       <c r="O6" s="27"/>
-      <c r="P6" s="84"/>
-      <c r="Q6" s="84"/>
-      <c r="R6" s="84"/>
-      <c r="S6" s="84"/>
-      <c r="T6" s="84"/>
-      <c r="U6" s="84"/>
-      <c r="V6" s="84"/>
-      <c r="W6" s="84"/>
+      <c r="P6" s="79"/>
+      <c r="Q6" s="79"/>
+      <c r="R6" s="79"/>
+      <c r="S6" s="79"/>
+      <c r="T6" s="79"/>
+      <c r="U6" s="79"/>
+      <c r="V6" s="79"/>
+      <c r="W6" s="79"/>
       <c r="X6" s="28"/>
       <c r="Z6" s="5"/>
       <c r="AB6" s="4"/>
       <c r="AC6" s="42"/>
       <c r="AD6" s="36"/>
-      <c r="AE6" s="75"/>
-      <c r="AF6" s="75"/>
-      <c r="AG6" s="75"/>
+      <c r="AE6" s="70"/>
+      <c r="AF6" s="70"/>
+      <c r="AG6" s="70"/>
       <c r="AH6" s="37"/>
       <c r="AI6" s="41"/>
       <c r="AJ6" s="5"/>
@@ -2267,10 +2267,10 @@
     <row r="7" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="4"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="78"/>
-      <c r="F7" s="78"/>
-      <c r="G7" s="78"/>
-      <c r="H7" s="78"/>
+      <c r="E7" s="73"/>
+      <c r="F7" s="73"/>
+      <c r="G7" s="73"/>
+      <c r="H7" s="73"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
       <c r="M7" s="4"/>
@@ -2280,14 +2280,14 @@
       <c r="O7" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P7" s="85"/>
-      <c r="Q7" s="85"/>
-      <c r="R7" s="85"/>
-      <c r="S7" s="85"/>
-      <c r="T7" s="85"/>
-      <c r="U7" s="85"/>
-      <c r="V7" s="85"/>
-      <c r="W7" s="85"/>
+      <c r="P7" s="80"/>
+      <c r="Q7" s="80"/>
+      <c r="R7" s="80"/>
+      <c r="S7" s="80"/>
+      <c r="T7" s="80"/>
+      <c r="U7" s="80"/>
+      <c r="V7" s="80"/>
+      <c r="W7" s="80"/>
       <c r="X7" s="30" t="s">
         <v>77</v>
       </c>
@@ -2302,9 +2302,9 @@
       <c r="AD7" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="AE7" s="76"/>
-      <c r="AF7" s="76"/>
-      <c r="AG7" s="76"/>
+      <c r="AE7" s="71"/>
+      <c r="AF7" s="71"/>
+      <c r="AG7" s="71"/>
       <c r="AH7" s="39" t="s">
         <v>94</v>
       </c>
@@ -2321,10 +2321,10 @@
       <c r="D8" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="78"/>
-      <c r="F8" s="78"/>
-      <c r="G8" s="78"/>
-      <c r="H8" s="78"/>
+      <c r="E8" s="73"/>
+      <c r="F8" s="73"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="73"/>
       <c r="I8" s="17" t="s">
         <v>59</v>
       </c>
@@ -2345,10 +2345,10 @@
       <c r="D9" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="79"/>
-      <c r="F9" s="79"/>
-      <c r="G9" s="79"/>
-      <c r="H9" s="79"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="74"/>
       <c r="I9" s="18" t="s">
         <v>60</v>
       </c>
@@ -2363,16 +2363,16 @@
       <c r="O9" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P9" s="83" t="s">
+      <c r="P9" s="78" t="s">
         <v>81</v>
       </c>
-      <c r="Q9" s="83"/>
-      <c r="R9" s="83"/>
-      <c r="S9" s="83"/>
-      <c r="T9" s="83"/>
-      <c r="U9" s="83"/>
-      <c r="V9" s="83"/>
-      <c r="W9" s="83"/>
+      <c r="Q9" s="78"/>
+      <c r="R9" s="78"/>
+      <c r="S9" s="78"/>
+      <c r="T9" s="78"/>
+      <c r="U9" s="78"/>
+      <c r="V9" s="78"/>
+      <c r="W9" s="78"/>
       <c r="X9" s="26" t="s">
         <v>76</v>
       </c>
@@ -2388,14 +2388,14 @@
       <c r="K10" s="5"/>
       <c r="M10" s="4"/>
       <c r="O10" s="27"/>
-      <c r="P10" s="84"/>
-      <c r="Q10" s="84"/>
-      <c r="R10" s="84"/>
-      <c r="S10" s="84"/>
-      <c r="T10" s="84"/>
-      <c r="U10" s="84"/>
-      <c r="V10" s="84"/>
-      <c r="W10" s="84"/>
+      <c r="P10" s="79"/>
+      <c r="Q10" s="79"/>
+      <c r="R10" s="79"/>
+      <c r="S10" s="79"/>
+      <c r="T10" s="79"/>
+      <c r="U10" s="79"/>
+      <c r="V10" s="79"/>
+      <c r="W10" s="79"/>
       <c r="X10" s="28"/>
       <c r="Z10" s="5"/>
       <c r="AB10" s="4"/>
@@ -2409,12 +2409,12 @@
       <c r="D11" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="77" t="s">
+      <c r="E11" s="72" t="s">
         <v>65</v>
       </c>
-      <c r="F11" s="77"/>
-      <c r="G11" s="77"/>
-      <c r="H11" s="77"/>
+      <c r="F11" s="72"/>
+      <c r="G11" s="72"/>
+      <c r="H11" s="72"/>
       <c r="I11" s="15" t="s">
         <v>57</v>
       </c>
@@ -2426,14 +2426,14 @@
       <c r="O11" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P11" s="85"/>
-      <c r="Q11" s="85"/>
-      <c r="R11" s="85"/>
-      <c r="S11" s="85"/>
-      <c r="T11" s="85"/>
-      <c r="U11" s="85"/>
-      <c r="V11" s="85"/>
-      <c r="W11" s="85"/>
+      <c r="P11" s="80"/>
+      <c r="Q11" s="80"/>
+      <c r="R11" s="80"/>
+      <c r="S11" s="80"/>
+      <c r="T11" s="80"/>
+      <c r="U11" s="80"/>
+      <c r="V11" s="80"/>
+      <c r="W11" s="80"/>
       <c r="X11" s="30" t="s">
         <v>77</v>
       </c>
@@ -2452,10 +2452,10 @@
       <c r="D12" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
+      <c r="E12" s="73"/>
+      <c r="F12" s="73"/>
+      <c r="G12" s="73"/>
+      <c r="H12" s="73"/>
       <c r="I12" s="16" t="s">
         <v>58</v>
       </c>
@@ -2468,10 +2468,10 @@
     <row r="13" spans="2:42" x14ac:dyDescent="0.45">
       <c r="B13" s="4"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="78"/>
-      <c r="F13" s="78"/>
-      <c r="G13" s="78"/>
-      <c r="H13" s="78"/>
+      <c r="E13" s="73"/>
+      <c r="F13" s="73"/>
+      <c r="G13" s="73"/>
+      <c r="H13" s="73"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
       <c r="M13" s="4"/>
@@ -2481,16 +2481,16 @@
       <c r="O13" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P13" s="83" t="s">
+      <c r="P13" s="78" t="s">
         <v>84</v>
       </c>
-      <c r="Q13" s="83"/>
-      <c r="R13" s="83"/>
-      <c r="S13" s="83"/>
-      <c r="T13" s="83"/>
-      <c r="U13" s="83"/>
-      <c r="V13" s="83"/>
-      <c r="W13" s="83"/>
+      <c r="Q13" s="78"/>
+      <c r="R13" s="78"/>
+      <c r="S13" s="78"/>
+      <c r="T13" s="78"/>
+      <c r="U13" s="78"/>
+      <c r="V13" s="78"/>
+      <c r="W13" s="78"/>
       <c r="X13" s="26" t="s">
         <v>76</v>
       </c>
@@ -2509,10 +2509,10 @@
       <c r="D14" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="78"/>
-      <c r="F14" s="78"/>
-      <c r="G14" s="78"/>
-      <c r="H14" s="78"/>
+      <c r="E14" s="73"/>
+      <c r="F14" s="73"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="73"/>
       <c r="I14" s="17" t="s">
         <v>59</v>
       </c>
@@ -2522,14 +2522,14 @@
       <c r="K14" s="5"/>
       <c r="M14" s="4"/>
       <c r="O14" s="27"/>
-      <c r="P14" s="84"/>
-      <c r="Q14" s="84"/>
-      <c r="R14" s="84"/>
-      <c r="S14" s="84"/>
-      <c r="T14" s="84"/>
-      <c r="U14" s="84"/>
-      <c r="V14" s="84"/>
-      <c r="W14" s="84"/>
+      <c r="P14" s="79"/>
+      <c r="Q14" s="79"/>
+      <c r="R14" s="79"/>
+      <c r="S14" s="79"/>
+      <c r="T14" s="79"/>
+      <c r="U14" s="79"/>
+      <c r="V14" s="79"/>
+      <c r="W14" s="79"/>
       <c r="X14" s="28"/>
       <c r="Z14" s="5"/>
       <c r="AB14" s="4"/>
@@ -2543,10 +2543,10 @@
       <c r="D15" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="79"/>
-      <c r="F15" s="79"/>
-      <c r="G15" s="79"/>
-      <c r="H15" s="79"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="74"/>
       <c r="I15" s="18" t="s">
         <v>60</v>
       </c>
@@ -2561,14 +2561,14 @@
       <c r="O15" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P15" s="85"/>
-      <c r="Q15" s="85"/>
-      <c r="R15" s="85"/>
-      <c r="S15" s="85"/>
-      <c r="T15" s="85"/>
-      <c r="U15" s="85"/>
-      <c r="V15" s="85"/>
-      <c r="W15" s="85"/>
+      <c r="P15" s="80"/>
+      <c r="Q15" s="80"/>
+      <c r="R15" s="80"/>
+      <c r="S15" s="80"/>
+      <c r="T15" s="80"/>
+      <c r="U15" s="80"/>
+      <c r="V15" s="80"/>
+      <c r="W15" s="80"/>
       <c r="X15" s="30" t="s">
         <v>77</v>
       </c>
@@ -2602,12 +2602,12 @@
       <c r="D17" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="77" t="s">
+      <c r="E17" s="72" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="77"/>
-      <c r="G17" s="77"/>
-      <c r="H17" s="77"/>
+      <c r="F17" s="72"/>
+      <c r="G17" s="72"/>
+      <c r="H17" s="72"/>
       <c r="I17" s="15" t="s">
         <v>57</v>
       </c>
@@ -2619,16 +2619,16 @@
       <c r="O17" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P17" s="83" t="s">
+      <c r="P17" s="78" t="s">
         <v>85</v>
       </c>
-      <c r="Q17" s="83"/>
-      <c r="R17" s="83"/>
-      <c r="S17" s="83"/>
-      <c r="T17" s="83"/>
-      <c r="U17" s="83"/>
-      <c r="V17" s="83"/>
-      <c r="W17" s="83"/>
+      <c r="Q17" s="78"/>
+      <c r="R17" s="78"/>
+      <c r="S17" s="78"/>
+      <c r="T17" s="78"/>
+      <c r="U17" s="78"/>
+      <c r="V17" s="78"/>
+      <c r="W17" s="78"/>
       <c r="X17" s="26" t="s">
         <v>76</v>
       </c>
@@ -2645,45 +2645,45 @@
       <c r="D18" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="78"/>
-      <c r="F18" s="78"/>
-      <c r="G18" s="78"/>
-      <c r="H18" s="78"/>
+      <c r="E18" s="73"/>
+      <c r="F18" s="73"/>
+      <c r="G18" s="73"/>
+      <c r="H18" s="73"/>
       <c r="I18" s="16" t="s">
         <v>58</v>
       </c>
       <c r="K18" s="5"/>
       <c r="M18" s="4"/>
       <c r="O18" s="27"/>
-      <c r="P18" s="84"/>
-      <c r="Q18" s="84"/>
-      <c r="R18" s="84"/>
-      <c r="S18" s="84"/>
-      <c r="T18" s="84"/>
-      <c r="U18" s="84"/>
-      <c r="V18" s="84"/>
-      <c r="W18" s="84"/>
+      <c r="P18" s="79"/>
+      <c r="Q18" s="79"/>
+      <c r="R18" s="79"/>
+      <c r="S18" s="79"/>
+      <c r="T18" s="79"/>
+      <c r="U18" s="79"/>
+      <c r="V18" s="79"/>
+      <c r="W18" s="79"/>
       <c r="X18" s="28"/>
       <c r="Z18" s="5"/>
-      <c r="AB18" s="80" t="s">
+      <c r="AB18" s="75" t="s">
         <v>98</v>
       </c>
-      <c r="AC18" s="81"/>
-      <c r="AD18" s="81"/>
-      <c r="AE18" s="81"/>
-      <c r="AF18" s="81"/>
-      <c r="AG18" s="81"/>
-      <c r="AH18" s="81"/>
-      <c r="AI18" s="81"/>
-      <c r="AJ18" s="82"/>
+      <c r="AC18" s="76"/>
+      <c r="AD18" s="76"/>
+      <c r="AE18" s="76"/>
+      <c r="AF18" s="76"/>
+      <c r="AG18" s="76"/>
+      <c r="AH18" s="76"/>
+      <c r="AI18" s="76"/>
+      <c r="AJ18" s="77"/>
     </row>
     <row r="19" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="4"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="78"/>
-      <c r="F19" s="78"/>
-      <c r="G19" s="78"/>
-      <c r="H19" s="78"/>
+      <c r="E19" s="73"/>
+      <c r="F19" s="73"/>
+      <c r="G19" s="73"/>
+      <c r="H19" s="73"/>
       <c r="I19" s="5"/>
       <c r="K19" s="5"/>
       <c r="M19" s="4"/>
@@ -2693,14 +2693,14 @@
       <c r="O19" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P19" s="85"/>
-      <c r="Q19" s="85"/>
-      <c r="R19" s="85"/>
-      <c r="S19" s="85"/>
-      <c r="T19" s="85"/>
-      <c r="U19" s="85"/>
-      <c r="V19" s="85"/>
-      <c r="W19" s="85"/>
+      <c r="P19" s="80"/>
+      <c r="Q19" s="80"/>
+      <c r="R19" s="80"/>
+      <c r="S19" s="80"/>
+      <c r="T19" s="80"/>
+      <c r="U19" s="80"/>
+      <c r="V19" s="80"/>
+      <c r="W19" s="80"/>
       <c r="X19" s="30" t="s">
         <v>77</v>
       </c>
@@ -2726,10 +2726,10 @@
       <c r="D20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="78"/>
-      <c r="F20" s="78"/>
-      <c r="G20" s="78"/>
-      <c r="H20" s="78"/>
+      <c r="E20" s="73"/>
+      <c r="F20" s="73"/>
+      <c r="G20" s="73"/>
+      <c r="H20" s="73"/>
       <c r="I20" s="17" t="s">
         <v>59</v>
       </c>
@@ -2746,11 +2746,11 @@
       <c r="AD20" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AE20" s="74" t="s">
+      <c r="AE20" s="69" t="s">
         <v>95</v>
       </c>
-      <c r="AF20" s="74"/>
-      <c r="AG20" s="74"/>
+      <c r="AF20" s="69"/>
+      <c r="AG20" s="69"/>
       <c r="AH20" s="3"/>
       <c r="AJ20" s="5"/>
     </row>
@@ -2762,10 +2762,10 @@
       <c r="D21" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="79"/>
-      <c r="F21" s="79"/>
-      <c r="G21" s="79"/>
-      <c r="H21" s="79"/>
+      <c r="E21" s="74"/>
+      <c r="F21" s="74"/>
+      <c r="G21" s="74"/>
+      <c r="H21" s="74"/>
       <c r="I21" s="18" t="s">
         <v>60</v>
       </c>
@@ -2778,9 +2778,9 @@
       <c r="AB21" s="4"/>
       <c r="AC21" s="42"/>
       <c r="AD21" s="36"/>
-      <c r="AE21" s="75"/>
-      <c r="AF21" s="75"/>
-      <c r="AG21" s="75"/>
+      <c r="AE21" s="70"/>
+      <c r="AF21" s="70"/>
+      <c r="AG21" s="70"/>
       <c r="AH21" s="44" t="s">
         <v>96</v>
       </c>
@@ -2801,9 +2801,9 @@
       <c r="AD22" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="AE22" s="76"/>
-      <c r="AF22" s="76"/>
-      <c r="AG22" s="76"/>
+      <c r="AE22" s="71"/>
+      <c r="AF22" s="71"/>
+      <c r="AG22" s="71"/>
       <c r="AH22" s="8"/>
       <c r="AJ22" s="5"/>
     </row>
@@ -2815,12 +2815,12 @@
       <c r="D23" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="77" t="s">
+      <c r="E23" s="72" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="77"/>
-      <c r="G23" s="77"/>
-      <c r="H23" s="77"/>
+      <c r="F23" s="72"/>
+      <c r="G23" s="72"/>
+      <c r="H23" s="72"/>
       <c r="I23" s="15" t="s">
         <v>57</v>
       </c>
@@ -2838,10 +2838,10 @@
       <c r="D24" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="78"/>
-      <c r="F24" s="78"/>
-      <c r="G24" s="78"/>
-      <c r="H24" s="78"/>
+      <c r="E24" s="73"/>
+      <c r="F24" s="73"/>
+      <c r="G24" s="73"/>
+      <c r="H24" s="73"/>
       <c r="I24" s="16" t="s">
         <v>58</v>
       </c>
@@ -2855,21 +2855,21 @@
       <c r="AD24" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AE24" s="74" t="s">
+      <c r="AE24" s="69" t="s">
         <v>115</v>
       </c>
-      <c r="AF24" s="74"/>
-      <c r="AG24" s="74"/>
+      <c r="AF24" s="69"/>
+      <c r="AG24" s="69"/>
       <c r="AH24" s="3"/>
       <c r="AJ24" s="5"/>
     </row>
     <row r="25" spans="2:36" ht="19.5" x14ac:dyDescent="0.6">
       <c r="B25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="78"/>
-      <c r="F25" s="78"/>
-      <c r="G25" s="78"/>
-      <c r="H25" s="78"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
+      <c r="H25" s="73"/>
       <c r="I25" s="5"/>
       <c r="K25" s="5"/>
       <c r="M25" s="4"/>
@@ -2877,9 +2877,9 @@
       <c r="AB25" s="4"/>
       <c r="AC25" s="42"/>
       <c r="AD25" s="36"/>
-      <c r="AE25" s="75"/>
-      <c r="AF25" s="75"/>
-      <c r="AG25" s="75"/>
+      <c r="AE25" s="70"/>
+      <c r="AF25" s="70"/>
+      <c r="AG25" s="70"/>
       <c r="AH25" s="44" t="s">
         <v>96</v>
       </c>
@@ -2896,10 +2896,10 @@
       <c r="D26" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="78"/>
-      <c r="F26" s="78"/>
-      <c r="G26" s="78"/>
-      <c r="H26" s="78"/>
+      <c r="E26" s="73"/>
+      <c r="F26" s="73"/>
+      <c r="G26" s="73"/>
+      <c r="H26" s="73"/>
       <c r="I26" s="17" t="s">
         <v>59</v>
       </c>
@@ -2916,9 +2916,9 @@
       <c r="AD26" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="AE26" s="76"/>
-      <c r="AF26" s="76"/>
-      <c r="AG26" s="76"/>
+      <c r="AE26" s="71"/>
+      <c r="AF26" s="71"/>
+      <c r="AG26" s="71"/>
       <c r="AH26" s="8"/>
       <c r="AJ26" s="5"/>
     </row>
@@ -2930,10 +2930,10 @@
       <c r="D27" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E27" s="79"/>
-      <c r="F27" s="79"/>
-      <c r="G27" s="79"/>
-      <c r="H27" s="79"/>
+      <c r="E27" s="74"/>
+      <c r="F27" s="74"/>
+      <c r="G27" s="74"/>
+      <c r="H27" s="74"/>
       <c r="I27" s="18" t="s">
         <v>60</v>
       </c>
@@ -2966,11 +2966,11 @@
       <c r="AD28" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AE28" s="74" t="s">
+      <c r="AE28" s="69" t="s">
         <v>114</v>
       </c>
-      <c r="AF28" s="74"/>
-      <c r="AG28" s="74"/>
+      <c r="AF28" s="69"/>
+      <c r="AG28" s="69"/>
       <c r="AH28" s="3"/>
       <c r="AJ28" s="5"/>
     </row>
@@ -2990,9 +2990,9 @@
       <c r="AB29" s="4"/>
       <c r="AC29" s="42"/>
       <c r="AD29" s="36"/>
-      <c r="AE29" s="75"/>
-      <c r="AF29" s="75"/>
-      <c r="AG29" s="75"/>
+      <c r="AE29" s="70"/>
+      <c r="AF29" s="70"/>
+      <c r="AG29" s="70"/>
       <c r="AH29" s="44" t="s">
         <v>96</v>
       </c>
@@ -3021,9 +3021,9 @@
       <c r="AD30" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="AE30" s="76"/>
-      <c r="AF30" s="76"/>
-      <c r="AG30" s="76"/>
+      <c r="AE30" s="71"/>
+      <c r="AF30" s="71"/>
+      <c r="AG30" s="71"/>
       <c r="AH30" s="8"/>
       <c r="AJ30" s="5"/>
     </row>

</xml_diff>

<commit_message>
Added NEW CV MODEL
</commit_message>
<xml_diff>
--- a/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
+++ b/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_Software\electrical_hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20ECBA8-3ADF-47F8-A074-073F4E5230E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF016CA9-7DE9-48AF-AF30-7D18E8B444F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="114">
   <si>
     <t>12V Power Distribution Rail</t>
   </si>
@@ -337,12 +337,6 @@
     <t>5V- Aux PDB</t>
   </si>
   <si>
-    <t>Aux Rail Ground</t>
-  </si>
-  <si>
-    <t>Servo Rail Ground</t>
-  </si>
-  <si>
     <t>Arduino GND</t>
   </si>
   <si>
@@ -358,15 +352,9 @@
     <t>D8</t>
   </si>
   <si>
-    <t>LHS Sweeper Servo +</t>
-  </si>
-  <si>
     <t>RHS Sweeper Swervo -</t>
   </si>
   <si>
-    <t>LHS Sweeper Swervo -</t>
-  </si>
-  <si>
     <t>RHS Sweeper Servo +</t>
   </si>
   <si>
@@ -374,6 +362,12 @@
   </si>
   <si>
     <t>MG996R Servo - Sweeper LHS</t>
+  </si>
+  <si>
+    <t>LHS Sweeper Servo -</t>
+  </si>
+  <si>
+    <t>LHS Sweeper Swervo +</t>
   </si>
 </sst>
 </file>
@@ -426,7 +420,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -531,24 +525,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.499984740745262"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -859,34 +859,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
@@ -916,6 +892,19 @@
         <color indexed="64"/>
       </right>
       <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -925,7 +914,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -970,11 +959,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -985,15 +972,12 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
@@ -1007,10 +991,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1019,72 +1003,61 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1117,6 +1090,47 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1411,26 +1425,26 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:19" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="85" t="s">
+      <c r="B2" s="75" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
-      <c r="J2" s="85"/>
-      <c r="K2" s="85"/>
-      <c r="L2" s="85"/>
-      <c r="M2" s="85"/>
-      <c r="N2" s="85"/>
-      <c r="O2" s="85"/>
-      <c r="P2" s="85"/>
-      <c r="Q2" s="85"/>
-      <c r="R2" s="85"/>
-      <c r="S2" s="85"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="75"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="75"/>
+      <c r="P2" s="75"/>
+      <c r="Q2" s="75"/>
+      <c r="R2" s="75"/>
+      <c r="S2" s="75"/>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B3" s="1"/>
@@ -1454,63 +1468,63 @@
     </row>
     <row r="4" spans="2:19" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="4"/>
-      <c r="E4" s="53" t="s">
+      <c r="E4" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="F4" s="54" t="s">
+      <c r="F4" s="49" t="s">
         <v>100</v>
       </c>
-      <c r="G4" s="59"/>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="59"/>
-      <c r="L4" s="59"/>
-      <c r="M4" s="59"/>
-      <c r="N4" s="59"/>
-      <c r="O4" s="59"/>
-      <c r="P4" s="54" t="s">
-        <v>105</v>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="54"/>
+      <c r="M4" s="54"/>
+      <c r="N4" s="54"/>
+      <c r="O4" s="54"/>
+      <c r="P4" s="49" t="s">
+        <v>103</v>
       </c>
       <c r="S4" s="5"/>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B5" s="4"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="45" t="s">
+      <c r="E5" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="45" t="s">
+      <c r="F5" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="G5" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="45" t="s">
+      <c r="H5" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="45" t="s">
+      <c r="I5" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="45" t="s">
+      <c r="J5" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="K5" s="45" t="s">
+      <c r="K5" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="L5" s="45" t="s">
+      <c r="L5" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="M5" s="45" t="s">
+      <c r="M5" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="N5" s="45" t="s">
+      <c r="N5" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="O5" s="45" t="s">
+      <c r="O5" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="P5" s="45" t="s">
+      <c r="P5" s="40" t="s">
         <v>24</v>
       </c>
       <c r="Q5" s="3"/>
@@ -1524,20 +1538,20 @@
       <c r="D6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="81" t="s">
+      <c r="E6" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="81"/>
-      <c r="G6" s="81"/>
-      <c r="H6" s="81"/>
-      <c r="I6" s="81"/>
-      <c r="J6" s="81"/>
-      <c r="K6" s="81"/>
-      <c r="L6" s="81"/>
-      <c r="M6" s="81"/>
-      <c r="N6" s="81"/>
-      <c r="O6" s="81"/>
-      <c r="P6" s="81"/>
+      <c r="F6" s="71"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="71"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="71"/>
+      <c r="K6" s="71"/>
+      <c r="L6" s="71"/>
+      <c r="M6" s="71"/>
+      <c r="N6" s="71"/>
+      <c r="O6" s="71"/>
+      <c r="P6" s="71"/>
       <c r="Q6" s="10" t="s">
         <v>25</v>
       </c>
@@ -1551,18 +1565,18 @@
       <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="81"/>
-      <c r="F7" s="81"/>
-      <c r="G7" s="81"/>
-      <c r="H7" s="81"/>
-      <c r="I7" s="81"/>
-      <c r="J7" s="81"/>
-      <c r="K7" s="81"/>
-      <c r="L7" s="81"/>
-      <c r="M7" s="81"/>
-      <c r="N7" s="81"/>
-      <c r="O7" s="81"/>
-      <c r="P7" s="81"/>
+      <c r="E7" s="71"/>
+      <c r="F7" s="71"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="71"/>
+      <c r="I7" s="71"/>
+      <c r="J7" s="71"/>
+      <c r="K7" s="71"/>
+      <c r="L7" s="71"/>
+      <c r="M7" s="71"/>
+      <c r="N7" s="71"/>
+      <c r="O7" s="71"/>
+      <c r="P7" s="71"/>
       <c r="Q7" s="10" t="s">
         <v>26</v>
       </c>
@@ -1571,40 +1585,40 @@
     <row r="8" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="4"/>
       <c r="D8" s="6"/>
-      <c r="E8" s="46" t="s">
+      <c r="E8" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="F8" s="46" t="s">
+      <c r="F8" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="G8" s="46" t="s">
+      <c r="G8" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="H8" s="46" t="s">
+      <c r="H8" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="I8" s="46" t="s">
+      <c r="I8" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="J8" s="46" t="s">
+      <c r="J8" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="K8" s="46" t="s">
+      <c r="K8" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="L8" s="46" t="s">
+      <c r="L8" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="M8" s="46" t="s">
+      <c r="M8" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="N8" s="46" t="s">
+      <c r="N8" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="O8" s="46" t="s">
+      <c r="O8" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="P8" s="46" t="s">
+      <c r="P8" s="41" t="s">
         <v>12</v>
       </c>
       <c r="Q8" s="8"/>
@@ -1612,38 +1626,38 @@
     </row>
     <row r="9" spans="2:19" ht="38.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="4"/>
-      <c r="E9" s="55" t="s">
+      <c r="E9" s="50" t="s">
         <v>101</v>
       </c>
-      <c r="F9" s="56" t="s">
+      <c r="F9" s="51" t="s">
         <v>102</v>
       </c>
-      <c r="G9" s="47" t="s">
+      <c r="G9" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="48" t="s">
+      <c r="H9" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="I9" s="47" t="s">
+      <c r="I9" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="48" t="s">
+      <c r="J9" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="K9" s="47" t="s">
+      <c r="K9" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="L9" s="48" t="s">
+      <c r="L9" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="M9" s="47" t="s">
+      <c r="M9" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="N9" s="48" t="s">
+      <c r="N9" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="O9" s="57"/>
-      <c r="P9" s="57"/>
+      <c r="O9" s="52"/>
+      <c r="P9" s="52"/>
       <c r="S9" s="5"/>
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.45">
@@ -1652,62 +1666,62 @@
     </row>
     <row r="11" spans="2:19" ht="29.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="4"/>
-      <c r="E11" s="59"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="59"/>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="59"/>
-      <c r="L11" s="59"/>
-      <c r="M11" s="59"/>
-      <c r="N11" s="59"/>
-      <c r="O11" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="P11" s="48" t="s">
+      <c r="E11" s="54"/>
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="54"/>
+      <c r="I11" s="54"/>
+      <c r="J11" s="54"/>
+      <c r="K11" s="54"/>
+      <c r="L11" s="54"/>
+      <c r="M11" s="54"/>
+      <c r="N11" s="54"/>
+      <c r="O11" s="43" t="s">
         <v>112</v>
+      </c>
+      <c r="P11" s="42" t="s">
+        <v>113</v>
       </c>
       <c r="S11" s="5"/>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B12" s="4"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="49" t="s">
+      <c r="E12" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="J12" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="M12" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="N12" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="O12" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="P12" s="44" t="s">
         <v>13</v>
-      </c>
-      <c r="F12" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" s="49" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="49" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" s="49" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="K12" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="L12" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="M12" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="N12" s="49" t="s">
-        <v>22</v>
-      </c>
-      <c r="O12" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="P12" s="49" t="s">
-        <v>24</v>
       </c>
       <c r="Q12" s="3"/>
       <c r="S12" s="5"/>
@@ -1720,20 +1734,20 @@
       <c r="D13" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="82" t="s">
+      <c r="E13" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="82"/>
-      <c r="G13" s="82"/>
-      <c r="H13" s="82"/>
-      <c r="I13" s="82"/>
-      <c r="J13" s="82"/>
-      <c r="K13" s="82"/>
-      <c r="L13" s="82"/>
-      <c r="M13" s="82"/>
-      <c r="N13" s="82"/>
-      <c r="O13" s="82"/>
-      <c r="P13" s="82"/>
+      <c r="F13" s="72"/>
+      <c r="G13" s="72"/>
+      <c r="H13" s="72"/>
+      <c r="I13" s="72"/>
+      <c r="J13" s="72"/>
+      <c r="K13" s="72"/>
+      <c r="L13" s="72"/>
+      <c r="M13" s="72"/>
+      <c r="N13" s="72"/>
+      <c r="O13" s="72"/>
+      <c r="P13" s="72"/>
       <c r="Q13" s="11" t="s">
         <v>25</v>
       </c>
@@ -1747,18 +1761,18 @@
       <c r="D14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="82"/>
-      <c r="F14" s="82"/>
-      <c r="G14" s="82"/>
-      <c r="H14" s="82"/>
-      <c r="I14" s="82"/>
-      <c r="J14" s="82"/>
-      <c r="K14" s="82"/>
-      <c r="L14" s="82"/>
-      <c r="M14" s="82"/>
-      <c r="N14" s="82"/>
-      <c r="O14" s="82"/>
-      <c r="P14" s="82"/>
+      <c r="E14" s="72"/>
+      <c r="F14" s="72"/>
+      <c r="G14" s="72"/>
+      <c r="H14" s="72"/>
+      <c r="I14" s="72"/>
+      <c r="J14" s="72"/>
+      <c r="K14" s="72"/>
+      <c r="L14" s="72"/>
+      <c r="M14" s="72"/>
+      <c r="N14" s="72"/>
+      <c r="O14" s="72"/>
+      <c r="P14" s="72"/>
       <c r="Q14" s="11" t="s">
         <v>26</v>
       </c>
@@ -1767,40 +1781,40 @@
     <row r="15" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="4"/>
       <c r="D15" s="6"/>
-      <c r="E15" s="50" t="s">
+      <c r="E15" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="F15" s="50" t="s">
+      <c r="F15" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="G15" s="50" t="s">
+      <c r="G15" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="H15" s="50" t="s">
+      <c r="H15" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="I15" s="50" t="s">
+      <c r="I15" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="J15" s="50" t="s">
+      <c r="J15" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="K15" s="50" t="s">
+      <c r="K15" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="L15" s="50" t="s">
+      <c r="L15" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="M15" s="50" t="s">
+      <c r="M15" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="N15" s="50" t="s">
+      <c r="N15" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="O15" s="50" t="s">
+      <c r="O15" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="P15" s="50" t="s">
+      <c r="P15" s="45" t="s">
         <v>12</v>
       </c>
       <c r="Q15" s="8"/>
@@ -1808,28 +1822,26 @@
     </row>
     <row r="16" spans="2:19" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B16" s="4"/>
-      <c r="E16" s="47" t="s">
+      <c r="E16" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="48" t="s">
+      <c r="F16" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="G16" s="57"/>
-      <c r="H16" s="48" t="s">
-        <v>103</v>
-      </c>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="57"/>
-      <c r="L16" s="57"/>
-      <c r="M16" s="57"/>
-      <c r="N16" s="57"/>
-      <c r="O16" s="47" t="s">
-        <v>113</v>
-      </c>
-      <c r="P16" s="48" t="s">
-        <v>111</v>
-      </c>
+      <c r="G16" s="52"/>
+      <c r="H16" s="76"/>
+      <c r="I16" s="52"/>
+      <c r="J16" s="52"/>
+      <c r="K16" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="L16" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="M16" s="52"/>
+      <c r="N16" s="52"/>
+      <c r="O16" s="76"/>
+      <c r="P16" s="76"/>
       <c r="S16" s="5"/>
     </row>
     <row r="17" spans="2:19" x14ac:dyDescent="0.45">
@@ -1838,72 +1850,70 @@
     </row>
     <row r="18" spans="2:19" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B18" s="4"/>
-      <c r="E18" s="59"/>
-      <c r="F18" s="59"/>
-      <c r="G18" s="51" t="s">
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="47" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="H18" s="52" t="s">
-        <v>50</v>
-      </c>
-      <c r="I18" s="52" t="s">
+      <c r="I18" s="54"/>
+      <c r="J18" s="53"/>
+      <c r="K18" s="53"/>
+      <c r="L18" s="53"/>
+      <c r="M18" s="47" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="58"/>
-      <c r="K18" s="58"/>
-      <c r="L18" s="58"/>
-      <c r="M18" s="51" t="s">
-        <v>107</v>
-      </c>
-      <c r="N18" s="52" t="s">
-        <v>106</v>
-      </c>
-      <c r="O18" s="51" t="s">
+      <c r="N18" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="O18" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="P18" s="46" t="s">
         <v>45</v>
-      </c>
-      <c r="P18" s="52" t="s">
-        <v>46</v>
       </c>
       <c r="S18" s="5"/>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B19" s="4"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="61" t="s">
+      <c r="E19" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="G19" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="I19" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="K19" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="L19" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="M19" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="N19" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="O19" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="P19" s="56" t="s">
         <v>13</v>
-      </c>
-      <c r="F19" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="G19" s="49" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" s="49" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" s="49" t="s">
-        <v>17</v>
-      </c>
-      <c r="J19" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="K19" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="L19" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="M19" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="N19" s="49" t="s">
-        <v>22</v>
-      </c>
-      <c r="O19" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="P19" s="62" t="s">
-        <v>24</v>
       </c>
       <c r="Q19" s="3"/>
       <c r="S19" s="5"/>
@@ -1916,20 +1926,20 @@
       <c r="D20" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="83" t="s">
+      <c r="E20" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="82"/>
-      <c r="G20" s="82"/>
-      <c r="H20" s="82"/>
-      <c r="I20" s="82"/>
-      <c r="J20" s="82"/>
-      <c r="K20" s="82"/>
-      <c r="L20" s="82"/>
-      <c r="M20" s="82"/>
-      <c r="N20" s="82"/>
-      <c r="O20" s="82"/>
-      <c r="P20" s="84"/>
+      <c r="F20" s="77"/>
+      <c r="G20" s="77"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="77"/>
+      <c r="J20" s="77"/>
+      <c r="K20" s="77"/>
+      <c r="L20" s="77"/>
+      <c r="M20" s="77"/>
+      <c r="N20" s="77"/>
+      <c r="O20" s="77"/>
+      <c r="P20" s="74"/>
       <c r="Q20" s="11" t="s">
         <v>25</v>
       </c>
@@ -1943,18 +1953,18 @@
       <c r="D21" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="83"/>
-      <c r="F21" s="82"/>
-      <c r="G21" s="82"/>
-      <c r="H21" s="82"/>
-      <c r="I21" s="82"/>
-      <c r="J21" s="82"/>
-      <c r="K21" s="82"/>
-      <c r="L21" s="82"/>
-      <c r="M21" s="82"/>
-      <c r="N21" s="82"/>
-      <c r="O21" s="82"/>
-      <c r="P21" s="84"/>
+      <c r="E21" s="73"/>
+      <c r="F21" s="77"/>
+      <c r="G21" s="77"/>
+      <c r="H21" s="77"/>
+      <c r="I21" s="77"/>
+      <c r="J21" s="77"/>
+      <c r="K21" s="77"/>
+      <c r="L21" s="77"/>
+      <c r="M21" s="77"/>
+      <c r="N21" s="77"/>
+      <c r="O21" s="77"/>
+      <c r="P21" s="74"/>
       <c r="Q21" s="11" t="s">
         <v>26</v>
       </c>
@@ -1963,40 +1973,40 @@
     <row r="22" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B22" s="4"/>
       <c r="D22" s="6"/>
-      <c r="E22" s="63" t="s">
+      <c r="E22" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="F22" s="50" t="s">
+      <c r="F22" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="G22" s="50" t="s">
+      <c r="G22" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="H22" s="50" t="s">
+      <c r="H22" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="I22" s="50" t="s">
+      <c r="I22" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="J22" s="50" t="s">
+      <c r="J22" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="K22" s="50" t="s">
+      <c r="K22" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="L22" s="50" t="s">
+      <c r="L22" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="M22" s="50" t="s">
+      <c r="M22" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="N22" s="50" t="s">
+      <c r="N22" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="O22" s="50" t="s">
+      <c r="O22" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="P22" s="64" t="s">
+      <c r="P22" s="58" t="s">
         <v>12</v>
       </c>
       <c r="Q22" s="8"/>
@@ -2004,24 +2014,24 @@
     </row>
     <row r="23" spans="2:19" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B23" s="4"/>
-      <c r="E23" s="47" t="s">
+      <c r="E23" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="47" t="s">
+      <c r="F23" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="57"/>
-      <c r="K23" s="57"/>
-      <c r="L23" s="57"/>
-      <c r="M23" s="57"/>
-      <c r="N23" s="57"/>
-      <c r="O23" s="47" t="s">
+      <c r="G23" s="52"/>
+      <c r="H23" s="52"/>
+      <c r="I23" s="52"/>
+      <c r="J23" s="52"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="52"/>
+      <c r="M23" s="52"/>
+      <c r="N23" s="52"/>
+      <c r="O23" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="P23" s="48" t="s">
+      <c r="P23" s="43" t="s">
         <v>44</v>
       </c>
       <c r="S23" s="5"/>
@@ -2083,51 +2093,51 @@
   <sheetData>
     <row r="2" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:42" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B3" s="75" t="s">
+      <c r="B3" s="65" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="76"/>
-      <c r="K3" s="77"/>
-      <c r="M3" s="75" t="s">
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="66"/>
+      <c r="K3" s="67"/>
+      <c r="M3" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="N3" s="76"/>
-      <c r="O3" s="76"/>
-      <c r="P3" s="76"/>
-      <c r="Q3" s="76"/>
-      <c r="R3" s="76"/>
-      <c r="S3" s="76"/>
-      <c r="T3" s="76"/>
-      <c r="U3" s="76"/>
-      <c r="V3" s="76"/>
-      <c r="W3" s="76"/>
-      <c r="X3" s="76"/>
-      <c r="Y3" s="76"/>
-      <c r="Z3" s="77"/>
-      <c r="AB3" s="75" t="s">
+      <c r="N3" s="66"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="66"/>
+      <c r="R3" s="66"/>
+      <c r="S3" s="66"/>
+      <c r="T3" s="66"/>
+      <c r="U3" s="66"/>
+      <c r="V3" s="66"/>
+      <c r="W3" s="66"/>
+      <c r="X3" s="66"/>
+      <c r="Y3" s="66"/>
+      <c r="Z3" s="67"/>
+      <c r="AB3" s="65" t="s">
         <v>91</v>
       </c>
-      <c r="AC3" s="76"/>
-      <c r="AD3" s="76"/>
-      <c r="AE3" s="76"/>
-      <c r="AF3" s="76"/>
-      <c r="AG3" s="76"/>
-      <c r="AH3" s="76"/>
-      <c r="AI3" s="76"/>
-      <c r="AJ3" s="77"/>
-      <c r="AK3" s="33"/>
-      <c r="AL3" s="33"/>
-      <c r="AM3" s="33"/>
-      <c r="AN3" s="33"/>
-      <c r="AO3" s="33"/>
-      <c r="AP3" s="33"/>
+      <c r="AC3" s="66"/>
+      <c r="AD3" s="66"/>
+      <c r="AE3" s="66"/>
+      <c r="AF3" s="66"/>
+      <c r="AG3" s="66"/>
+      <c r="AH3" s="66"/>
+      <c r="AI3" s="66"/>
+      <c r="AJ3" s="67"/>
+      <c r="AK3" s="31"/>
+      <c r="AL3" s="31"/>
+      <c r="AM3" s="31"/>
+      <c r="AN3" s="31"/>
+      <c r="AO3" s="31"/>
+      <c r="AP3" s="31"/>
     </row>
     <row r="4" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="1"/>
@@ -2172,34 +2182,34 @@
       <c r="D5" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="72" t="s">
+      <c r="E5" s="62" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="72"/>
-      <c r="G5" s="72"/>
-      <c r="H5" s="72"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
       <c r="I5" s="15" t="s">
         <v>57</v>
       </c>
       <c r="K5" s="5"/>
       <c r="M5" s="4"/>
-      <c r="N5" s="31" t="s">
+      <c r="N5" s="29" t="s">
         <v>29</v>
       </c>
       <c r="O5" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P5" s="78" t="s">
+      <c r="P5" s="68" t="s">
         <v>78</v>
       </c>
-      <c r="Q5" s="78"/>
-      <c r="R5" s="78"/>
-      <c r="S5" s="78"/>
-      <c r="T5" s="78"/>
-      <c r="U5" s="78"/>
-      <c r="V5" s="78"/>
-      <c r="W5" s="78"/>
-      <c r="X5" s="26" t="s">
+      <c r="Q5" s="68"/>
+      <c r="R5" s="68"/>
+      <c r="S5" s="68"/>
+      <c r="T5" s="68"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="80" t="s">
         <v>76</v>
       </c>
       <c r="Y5" s="20" t="s">
@@ -2207,22 +2217,22 @@
       </c>
       <c r="Z5" s="5"/>
       <c r="AB5" s="4"/>
-      <c r="AC5" s="43" t="s">
+      <c r="AC5" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="AD5" s="34" t="s">
+      <c r="AD5" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="AE5" s="69" t="s">
+      <c r="AE5" s="86" t="s">
         <v>91</v>
       </c>
-      <c r="AF5" s="69"/>
-      <c r="AG5" s="69"/>
-      <c r="AH5" s="35" t="s">
+      <c r="AF5" s="59"/>
+      <c r="AG5" s="87"/>
+      <c r="AH5" s="84" t="s">
         <v>93</v>
       </c>
-      <c r="AI5" s="40" t="s">
-        <v>109</v>
+      <c r="AI5" s="35" t="s">
+        <v>107</v>
       </c>
       <c r="AJ5" s="5"/>
     </row>
@@ -2234,61 +2244,61 @@
       <c r="D6" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="73"/>
-      <c r="F6" s="73"/>
-      <c r="G6" s="73"/>
-      <c r="H6" s="73"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="63"/>
       <c r="I6" s="16" t="s">
         <v>58</v>
       </c>
       <c r="K6" s="5"/>
       <c r="M6" s="4"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="79"/>
-      <c r="Q6" s="79"/>
-      <c r="R6" s="79"/>
-      <c r="S6" s="79"/>
-      <c r="T6" s="79"/>
-      <c r="U6" s="79"/>
-      <c r="V6" s="79"/>
-      <c r="W6" s="79"/>
-      <c r="X6" s="28"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="69"/>
+      <c r="Q6" s="69"/>
+      <c r="R6" s="69"/>
+      <c r="S6" s="69"/>
+      <c r="T6" s="69"/>
+      <c r="U6" s="69"/>
+      <c r="V6" s="69"/>
+      <c r="W6" s="69"/>
+      <c r="X6" s="27"/>
       <c r="Z6" s="5"/>
       <c r="AB6" s="4"/>
-      <c r="AC6" s="42"/>
-      <c r="AD6" s="36"/>
-      <c r="AE6" s="70"/>
-      <c r="AF6" s="70"/>
-      <c r="AG6" s="70"/>
-      <c r="AH6" s="37"/>
-      <c r="AI6" s="41"/>
+      <c r="AC6" s="37"/>
+      <c r="AD6" s="82"/>
+      <c r="AE6" s="88"/>
+      <c r="AF6" s="89"/>
+      <c r="AG6" s="90"/>
+      <c r="AH6" s="5"/>
+      <c r="AI6" s="36"/>
       <c r="AJ6" s="5"/>
     </row>
     <row r="7" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="4"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="73"/>
-      <c r="F7" s="73"/>
-      <c r="G7" s="73"/>
-      <c r="H7" s="73"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
       <c r="M7" s="4"/>
-      <c r="N7" s="32" t="s">
+      <c r="N7" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="O7" s="29" t="s">
+      <c r="O7" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P7" s="80"/>
-      <c r="Q7" s="80"/>
-      <c r="R7" s="80"/>
-      <c r="S7" s="80"/>
-      <c r="T7" s="80"/>
-      <c r="U7" s="80"/>
-      <c r="V7" s="80"/>
-      <c r="W7" s="80"/>
-      <c r="X7" s="30" t="s">
+      <c r="P7" s="70"/>
+      <c r="Q7" s="70"/>
+      <c r="R7" s="70"/>
+      <c r="S7" s="70"/>
+      <c r="T7" s="70"/>
+      <c r="U7" s="70"/>
+      <c r="V7" s="70"/>
+      <c r="W7" s="70"/>
+      <c r="X7" s="18" t="s">
         <v>77</v>
       </c>
       <c r="Y7" s="20" t="s">
@@ -2296,20 +2306,20 @@
       </c>
       <c r="Z7" s="5"/>
       <c r="AB7" s="4"/>
-      <c r="AC7" s="43" t="s">
+      <c r="AC7" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="AD7" s="38" t="s">
+      <c r="AD7" s="83" t="s">
         <v>57</v>
       </c>
-      <c r="AE7" s="71"/>
-      <c r="AF7" s="71"/>
-      <c r="AG7" s="71"/>
-      <c r="AH7" s="39" t="s">
+      <c r="AE7" s="91"/>
+      <c r="AF7" s="61"/>
+      <c r="AG7" s="92"/>
+      <c r="AH7" s="85" t="s">
         <v>94</v>
       </c>
-      <c r="AI7" s="40" t="s">
-        <v>108</v>
+      <c r="AI7" s="35" t="s">
+        <v>106</v>
       </c>
       <c r="AJ7" s="5"/>
     </row>
@@ -2321,10 +2331,10 @@
       <c r="D8" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="73"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="63"/>
+      <c r="G8" s="63"/>
+      <c r="H8" s="63"/>
       <c r="I8" s="17" t="s">
         <v>59</v>
       </c>
@@ -2345,11 +2355,11 @@
       <c r="D9" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="74"/>
-      <c r="F9" s="74"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="74"/>
-      <c r="I9" s="18" t="s">
+      <c r="E9" s="64"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="64"/>
+      <c r="H9" s="64"/>
+      <c r="I9" s="78" t="s">
         <v>60</v>
       </c>
       <c r="J9" s="20" t="s">
@@ -2357,23 +2367,23 @@
       </c>
       <c r="K9" s="5"/>
       <c r="M9" s="4"/>
-      <c r="N9" s="31" t="s">
+      <c r="N9" s="29" t="s">
         <v>29</v>
       </c>
       <c r="O9" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P9" s="78" t="s">
+      <c r="P9" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="Q9" s="78"/>
-      <c r="R9" s="78"/>
-      <c r="S9" s="78"/>
-      <c r="T9" s="78"/>
-      <c r="U9" s="78"/>
-      <c r="V9" s="78"/>
-      <c r="W9" s="78"/>
-      <c r="X9" s="26" t="s">
+      <c r="Q9" s="68"/>
+      <c r="R9" s="68"/>
+      <c r="S9" s="68"/>
+      <c r="T9" s="68"/>
+      <c r="U9" s="68"/>
+      <c r="V9" s="68"/>
+      <c r="W9" s="68"/>
+      <c r="X9" s="80" t="s">
         <v>76</v>
       </c>
       <c r="Y9" s="20" t="s">
@@ -2387,16 +2397,16 @@
       <c r="B10" s="4"/>
       <c r="K10" s="5"/>
       <c r="M10" s="4"/>
-      <c r="O10" s="27"/>
-      <c r="P10" s="79"/>
-      <c r="Q10" s="79"/>
-      <c r="R10" s="79"/>
-      <c r="S10" s="79"/>
-      <c r="T10" s="79"/>
-      <c r="U10" s="79"/>
-      <c r="V10" s="79"/>
-      <c r="W10" s="79"/>
-      <c r="X10" s="28"/>
+      <c r="O10" s="26"/>
+      <c r="P10" s="69"/>
+      <c r="Q10" s="69"/>
+      <c r="R10" s="69"/>
+      <c r="S10" s="69"/>
+      <c r="T10" s="69"/>
+      <c r="U10" s="69"/>
+      <c r="V10" s="69"/>
+      <c r="W10" s="69"/>
+      <c r="X10" s="27"/>
       <c r="Z10" s="5"/>
       <c r="AB10" s="4"/>
       <c r="AJ10" s="5"/>
@@ -2409,32 +2419,32 @@
       <c r="D11" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="72" t="s">
+      <c r="E11" s="62" t="s">
         <v>65</v>
       </c>
-      <c r="F11" s="72"/>
-      <c r="G11" s="72"/>
-      <c r="H11" s="72"/>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="62"/>
       <c r="I11" s="15" t="s">
         <v>57</v>
       </c>
       <c r="K11" s="5"/>
       <c r="M11" s="4"/>
-      <c r="N11" s="32" t="s">
+      <c r="N11" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="O11" s="29" t="s">
+      <c r="O11" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P11" s="80"/>
-      <c r="Q11" s="80"/>
-      <c r="R11" s="80"/>
-      <c r="S11" s="80"/>
-      <c r="T11" s="80"/>
-      <c r="U11" s="80"/>
-      <c r="V11" s="80"/>
-      <c r="W11" s="80"/>
-      <c r="X11" s="30" t="s">
+      <c r="P11" s="70"/>
+      <c r="Q11" s="70"/>
+      <c r="R11" s="70"/>
+      <c r="S11" s="70"/>
+      <c r="T11" s="70"/>
+      <c r="U11" s="70"/>
+      <c r="V11" s="70"/>
+      <c r="W11" s="70"/>
+      <c r="X11" s="18" t="s">
         <v>77</v>
       </c>
       <c r="Y11" s="20" t="s">
@@ -2452,10 +2462,10 @@
       <c r="D12" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="73"/>
-      <c r="F12" s="73"/>
-      <c r="G12" s="73"/>
-      <c r="H12" s="73"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="63"/>
       <c r="I12" s="16" t="s">
         <v>58</v>
       </c>
@@ -2468,30 +2478,30 @@
     <row r="13" spans="2:42" x14ac:dyDescent="0.45">
       <c r="B13" s="4"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="73"/>
-      <c r="F13" s="73"/>
-      <c r="G13" s="73"/>
-      <c r="H13" s="73"/>
+      <c r="E13" s="63"/>
+      <c r="F13" s="63"/>
+      <c r="G13" s="63"/>
+      <c r="H13" s="63"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
       <c r="M13" s="4"/>
-      <c r="N13" s="31" t="s">
+      <c r="N13" s="29" t="s">
         <v>29</v>
       </c>
       <c r="O13" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P13" s="78" t="s">
+      <c r="P13" s="68" t="s">
         <v>84</v>
       </c>
-      <c r="Q13" s="78"/>
-      <c r="R13" s="78"/>
-      <c r="S13" s="78"/>
-      <c r="T13" s="78"/>
-      <c r="U13" s="78"/>
-      <c r="V13" s="78"/>
-      <c r="W13" s="78"/>
-      <c r="X13" s="26" t="s">
+      <c r="Q13" s="68"/>
+      <c r="R13" s="68"/>
+      <c r="S13" s="68"/>
+      <c r="T13" s="68"/>
+      <c r="U13" s="68"/>
+      <c r="V13" s="68"/>
+      <c r="W13" s="68"/>
+      <c r="X13" s="80" t="s">
         <v>76</v>
       </c>
       <c r="Y13" s="20" t="s">
@@ -2509,10 +2519,10 @@
       <c r="D14" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="73"/>
-      <c r="F14" s="73"/>
-      <c r="G14" s="73"/>
-      <c r="H14" s="73"/>
+      <c r="E14" s="63"/>
+      <c r="F14" s="63"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="63"/>
       <c r="I14" s="17" t="s">
         <v>59</v>
       </c>
@@ -2521,16 +2531,16 @@
       </c>
       <c r="K14" s="5"/>
       <c r="M14" s="4"/>
-      <c r="O14" s="27"/>
-      <c r="P14" s="79"/>
-      <c r="Q14" s="79"/>
-      <c r="R14" s="79"/>
-      <c r="S14" s="79"/>
-      <c r="T14" s="79"/>
-      <c r="U14" s="79"/>
-      <c r="V14" s="79"/>
-      <c r="W14" s="79"/>
-      <c r="X14" s="28"/>
+      <c r="O14" s="26"/>
+      <c r="P14" s="69"/>
+      <c r="Q14" s="69"/>
+      <c r="R14" s="69"/>
+      <c r="S14" s="69"/>
+      <c r="T14" s="69"/>
+      <c r="U14" s="69"/>
+      <c r="V14" s="69"/>
+      <c r="W14" s="69"/>
+      <c r="X14" s="27"/>
       <c r="Z14" s="5"/>
       <c r="AB14" s="4"/>
       <c r="AJ14" s="5"/>
@@ -2543,11 +2553,11 @@
       <c r="D15" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="74"/>
-      <c r="F15" s="74"/>
-      <c r="G15" s="74"/>
-      <c r="H15" s="74"/>
-      <c r="I15" s="18" t="s">
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="64"/>
+      <c r="I15" s="78" t="s">
         <v>60</v>
       </c>
       <c r="J15" s="20" t="s">
@@ -2555,21 +2565,21 @@
       </c>
       <c r="K15" s="5"/>
       <c r="M15" s="4"/>
-      <c r="N15" s="32" t="s">
+      <c r="N15" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="O15" s="29" t="s">
+      <c r="O15" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P15" s="80"/>
-      <c r="Q15" s="80"/>
-      <c r="R15" s="80"/>
-      <c r="S15" s="80"/>
-      <c r="T15" s="80"/>
-      <c r="U15" s="80"/>
-      <c r="V15" s="80"/>
-      <c r="W15" s="80"/>
-      <c r="X15" s="30" t="s">
+      <c r="P15" s="70"/>
+      <c r="Q15" s="70"/>
+      <c r="R15" s="70"/>
+      <c r="S15" s="70"/>
+      <c r="T15" s="70"/>
+      <c r="U15" s="70"/>
+      <c r="V15" s="70"/>
+      <c r="W15" s="70"/>
+      <c r="X15" s="79" t="s">
         <v>77</v>
       </c>
       <c r="Y15" s="20" t="s">
@@ -2602,34 +2612,34 @@
       <c r="D17" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="72" t="s">
+      <c r="E17" s="62" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="72"/>
-      <c r="G17" s="72"/>
-      <c r="H17" s="72"/>
+      <c r="F17" s="62"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
       <c r="I17" s="15" t="s">
         <v>57</v>
       </c>
       <c r="K17" s="5"/>
       <c r="M17" s="4"/>
-      <c r="N17" s="31" t="s">
+      <c r="N17" s="29" t="s">
         <v>29</v>
       </c>
       <c r="O17" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="P17" s="78" t="s">
+      <c r="P17" s="68" t="s">
         <v>85</v>
       </c>
-      <c r="Q17" s="78"/>
-      <c r="R17" s="78"/>
-      <c r="S17" s="78"/>
-      <c r="T17" s="78"/>
-      <c r="U17" s="78"/>
-      <c r="V17" s="78"/>
-      <c r="W17" s="78"/>
-      <c r="X17" s="26" t="s">
+      <c r="Q17" s="68"/>
+      <c r="R17" s="68"/>
+      <c r="S17" s="68"/>
+      <c r="T17" s="68"/>
+      <c r="U17" s="68"/>
+      <c r="V17" s="68"/>
+      <c r="W17" s="68"/>
+      <c r="X17" s="80" t="s">
         <v>76</v>
       </c>
       <c r="Y17" s="20" t="s">
@@ -2645,63 +2655,63 @@
       <c r="D18" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="73"/>
-      <c r="F18" s="73"/>
-      <c r="G18" s="73"/>
-      <c r="H18" s="73"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
       <c r="I18" s="16" t="s">
         <v>58</v>
       </c>
       <c r="K18" s="5"/>
       <c r="M18" s="4"/>
-      <c r="O18" s="27"/>
-      <c r="P18" s="79"/>
-      <c r="Q18" s="79"/>
-      <c r="R18" s="79"/>
-      <c r="S18" s="79"/>
-      <c r="T18" s="79"/>
-      <c r="U18" s="79"/>
-      <c r="V18" s="79"/>
-      <c r="W18" s="79"/>
-      <c r="X18" s="28"/>
+      <c r="O18" s="26"/>
+      <c r="P18" s="69"/>
+      <c r="Q18" s="69"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="69"/>
+      <c r="T18" s="69"/>
+      <c r="U18" s="69"/>
+      <c r="V18" s="69"/>
+      <c r="W18" s="69"/>
+      <c r="X18" s="27"/>
       <c r="Z18" s="5"/>
-      <c r="AB18" s="75" t="s">
+      <c r="AB18" s="65" t="s">
         <v>98</v>
       </c>
-      <c r="AC18" s="76"/>
-      <c r="AD18" s="76"/>
-      <c r="AE18" s="76"/>
-      <c r="AF18" s="76"/>
-      <c r="AG18" s="76"/>
-      <c r="AH18" s="76"/>
-      <c r="AI18" s="76"/>
-      <c r="AJ18" s="77"/>
+      <c r="AC18" s="66"/>
+      <c r="AD18" s="66"/>
+      <c r="AE18" s="66"/>
+      <c r="AF18" s="66"/>
+      <c r="AG18" s="66"/>
+      <c r="AH18" s="66"/>
+      <c r="AI18" s="66"/>
+      <c r="AJ18" s="67"/>
     </row>
     <row r="19" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="4"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="73"/>
-      <c r="F19" s="73"/>
-      <c r="G19" s="73"/>
-      <c r="H19" s="73"/>
+      <c r="E19" s="63"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="63"/>
       <c r="I19" s="5"/>
       <c r="K19" s="5"/>
       <c r="M19" s="4"/>
-      <c r="N19" s="32" t="s">
+      <c r="N19" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="O19" s="29" t="s">
+      <c r="O19" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P19" s="80"/>
-      <c r="Q19" s="80"/>
-      <c r="R19" s="80"/>
-      <c r="S19" s="80"/>
-      <c r="T19" s="80"/>
-      <c r="U19" s="80"/>
-      <c r="V19" s="80"/>
-      <c r="W19" s="80"/>
-      <c r="X19" s="30" t="s">
+      <c r="P19" s="70"/>
+      <c r="Q19" s="70"/>
+      <c r="R19" s="70"/>
+      <c r="S19" s="70"/>
+      <c r="T19" s="70"/>
+      <c r="U19" s="70"/>
+      <c r="V19" s="70"/>
+      <c r="W19" s="70"/>
+      <c r="X19" s="79" t="s">
         <v>77</v>
       </c>
       <c r="Y19" s="20" t="s">
@@ -2726,10 +2736,10 @@
       <c r="D20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="73"/>
-      <c r="F20" s="73"/>
-      <c r="G20" s="73"/>
-      <c r="H20" s="73"/>
+      <c r="E20" s="63"/>
+      <c r="F20" s="63"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="63"/>
       <c r="I20" s="17" t="s">
         <v>59</v>
       </c>
@@ -2740,17 +2750,17 @@
       <c r="M20" s="4"/>
       <c r="Z20" s="5"/>
       <c r="AB20" s="4"/>
-      <c r="AC20" s="43" t="s">
+      <c r="AC20" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="AD20" s="34" t="s">
+      <c r="AD20" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="AE20" s="69" t="s">
+      <c r="AE20" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="AF20" s="69"/>
-      <c r="AG20" s="69"/>
+      <c r="AF20" s="59"/>
+      <c r="AG20" s="59"/>
       <c r="AH20" s="3"/>
       <c r="AJ20" s="5"/>
     </row>
@@ -2762,11 +2772,11 @@
       <c r="D21" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="74"/>
-      <c r="H21" s="74"/>
-      <c r="I21" s="18" t="s">
+      <c r="E21" s="64"/>
+      <c r="F21" s="64"/>
+      <c r="G21" s="64"/>
+      <c r="H21" s="64"/>
+      <c r="I21" s="78" t="s">
         <v>60</v>
       </c>
       <c r="J21" s="20" t="s">
@@ -2776,15 +2786,15 @@
       <c r="M21" s="4"/>
       <c r="Z21" s="5"/>
       <c r="AB21" s="4"/>
-      <c r="AC21" s="42"/>
-      <c r="AD21" s="36"/>
-      <c r="AE21" s="70"/>
-      <c r="AF21" s="70"/>
-      <c r="AG21" s="70"/>
-      <c r="AH21" s="44" t="s">
+      <c r="AC21" s="37"/>
+      <c r="AD21" s="33"/>
+      <c r="AE21" s="60"/>
+      <c r="AF21" s="60"/>
+      <c r="AG21" s="60"/>
+      <c r="AH21" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="AI21" s="40" t="s">
+      <c r="AI21" s="35" t="s">
         <v>1</v>
       </c>
       <c r="AJ21" s="5"/>
@@ -2795,15 +2805,15 @@
       <c r="M22" s="4"/>
       <c r="Z22" s="5"/>
       <c r="AB22" s="4"/>
-      <c r="AC22" s="43" t="s">
+      <c r="AC22" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="AD22" s="38" t="s">
+      <c r="AD22" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="AE22" s="71"/>
-      <c r="AF22" s="71"/>
-      <c r="AG22" s="71"/>
+      <c r="AE22" s="61"/>
+      <c r="AF22" s="61"/>
+      <c r="AG22" s="61"/>
       <c r="AH22" s="8"/>
       <c r="AJ22" s="5"/>
     </row>
@@ -2815,12 +2825,12 @@
       <c r="D23" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="72" t="s">
+      <c r="E23" s="62" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="72"/>
-      <c r="G23" s="72"/>
-      <c r="H23" s="72"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
       <c r="I23" s="15" t="s">
         <v>57</v>
       </c>
@@ -2838,10 +2848,10 @@
       <c r="D24" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="73"/>
-      <c r="F24" s="73"/>
-      <c r="G24" s="73"/>
-      <c r="H24" s="73"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="63"/>
+      <c r="G24" s="63"/>
+      <c r="H24" s="63"/>
       <c r="I24" s="16" t="s">
         <v>58</v>
       </c>
@@ -2849,42 +2859,42 @@
       <c r="M24" s="4"/>
       <c r="Z24" s="5"/>
       <c r="AB24" s="4"/>
-      <c r="AC24" s="43" t="s">
+      <c r="AC24" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="AD24" s="34" t="s">
+      <c r="AD24" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="AE24" s="69" t="s">
-        <v>115</v>
-      </c>
-      <c r="AF24" s="69"/>
-      <c r="AG24" s="69"/>
+      <c r="AE24" s="59" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF24" s="59"/>
+      <c r="AG24" s="59"/>
       <c r="AH24" s="3"/>
       <c r="AJ24" s="5"/>
     </row>
     <row r="25" spans="2:36" ht="19.5" x14ac:dyDescent="0.6">
       <c r="B25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="73"/>
-      <c r="F25" s="73"/>
-      <c r="G25" s="73"/>
-      <c r="H25" s="73"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="63"/>
+      <c r="G25" s="63"/>
+      <c r="H25" s="63"/>
       <c r="I25" s="5"/>
       <c r="K25" s="5"/>
       <c r="M25" s="4"/>
       <c r="Z25" s="5"/>
       <c r="AB25" s="4"/>
-      <c r="AC25" s="42"/>
-      <c r="AD25" s="36"/>
-      <c r="AE25" s="70"/>
-      <c r="AF25" s="70"/>
-      <c r="AG25" s="70"/>
-      <c r="AH25" s="44" t="s">
+      <c r="AC25" s="37"/>
+      <c r="AD25" s="33"/>
+      <c r="AE25" s="60"/>
+      <c r="AF25" s="60"/>
+      <c r="AG25" s="60"/>
+      <c r="AH25" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="AI25" s="40" t="s">
-        <v>97</v>
+      <c r="AI25" s="35" t="s">
+        <v>3</v>
       </c>
       <c r="AJ25" s="5"/>
     </row>
@@ -2896,10 +2906,10 @@
       <c r="D26" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="73"/>
-      <c r="F26" s="73"/>
-      <c r="G26" s="73"/>
-      <c r="H26" s="73"/>
+      <c r="E26" s="63"/>
+      <c r="F26" s="63"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="63"/>
       <c r="I26" s="17" t="s">
         <v>59</v>
       </c>
@@ -2910,15 +2920,15 @@
       <c r="M26" s="4"/>
       <c r="Z26" s="5"/>
       <c r="AB26" s="4"/>
-      <c r="AC26" s="43" t="s">
+      <c r="AC26" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="AD26" s="38" t="s">
+      <c r="AD26" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="AE26" s="71"/>
-      <c r="AF26" s="71"/>
-      <c r="AG26" s="71"/>
+      <c r="AE26" s="61"/>
+      <c r="AF26" s="61"/>
+      <c r="AG26" s="61"/>
       <c r="AH26" s="8"/>
       <c r="AJ26" s="5"/>
     </row>
@@ -2930,11 +2940,11 @@
       <c r="D27" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E27" s="74"/>
-      <c r="F27" s="74"/>
-      <c r="G27" s="74"/>
-      <c r="H27" s="74"/>
-      <c r="I27" s="18" t="s">
+      <c r="E27" s="64"/>
+      <c r="F27" s="64"/>
+      <c r="G27" s="64"/>
+      <c r="H27" s="64"/>
+      <c r="I27" s="78" t="s">
         <v>60</v>
       </c>
       <c r="J27" s="20" t="s">
@@ -2946,84 +2956,60 @@
       <c r="AB27" s="4"/>
       <c r="AJ27" s="5"/>
     </row>
-    <row r="28" spans="2:36" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="28" spans="2:36" x14ac:dyDescent="0.45">
       <c r="B28" s="4"/>
-      <c r="C28" s="65"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="60"/>
-      <c r="H28" s="60"/>
-      <c r="I28" s="67"/>
-      <c r="J28" s="68"/>
       <c r="K28" s="5"/>
       <c r="M28" s="4"/>
       <c r="Z28" s="5"/>
       <c r="AB28" s="4"/>
-      <c r="AC28" s="43" t="s">
+      <c r="AC28" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="AD28" s="34" t="s">
+      <c r="AD28" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="AE28" s="69" t="s">
-        <v>114</v>
-      </c>
-      <c r="AF28" s="69"/>
-      <c r="AG28" s="69"/>
+      <c r="AE28" s="59" t="s">
+        <v>110</v>
+      </c>
+      <c r="AF28" s="59"/>
+      <c r="AG28" s="59"/>
       <c r="AH28" s="3"/>
       <c r="AJ28" s="5"/>
     </row>
-    <row r="29" spans="2:36" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
+    <row r="29" spans="2:36" ht="19.5" x14ac:dyDescent="0.6">
       <c r="B29" s="4"/>
-      <c r="C29" s="65"/>
-      <c r="D29" s="66"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="60"/>
-      <c r="G29" s="60"/>
-      <c r="H29" s="60"/>
-      <c r="I29" s="67"/>
-      <c r="J29" s="68"/>
       <c r="K29" s="5"/>
       <c r="M29" s="4"/>
       <c r="Z29" s="5"/>
       <c r="AB29" s="4"/>
-      <c r="AC29" s="42"/>
-      <c r="AD29" s="36"/>
-      <c r="AE29" s="70"/>
-      <c r="AF29" s="70"/>
-      <c r="AG29" s="70"/>
-      <c r="AH29" s="44" t="s">
+      <c r="AC29" s="37"/>
+      <c r="AD29" s="33"/>
+      <c r="AE29" s="60"/>
+      <c r="AF29" s="60"/>
+      <c r="AG29" s="60"/>
+      <c r="AH29" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="AI29" s="40" t="s">
-        <v>3</v>
+      <c r="AI29" s="35" t="s">
+        <v>97</v>
       </c>
       <c r="AJ29" s="5"/>
     </row>
-    <row r="30" spans="2:36" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="30" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B30" s="4"/>
-      <c r="C30" s="65"/>
-      <c r="D30" s="66"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="60"/>
-      <c r="G30" s="60"/>
-      <c r="H30" s="60"/>
-      <c r="I30" s="67"/>
-      <c r="J30" s="68"/>
       <c r="K30" s="5"/>
       <c r="M30" s="4"/>
       <c r="Z30" s="5"/>
       <c r="AB30" s="4"/>
-      <c r="AC30" s="43" t="s">
+      <c r="AC30" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="AD30" s="38" t="s">
+      <c r="AD30" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="AE30" s="71"/>
-      <c r="AF30" s="71"/>
-      <c r="AG30" s="71"/>
+      <c r="AE30" s="61"/>
+      <c r="AF30" s="61"/>
+      <c r="AG30" s="61"/>
       <c r="AH30" s="8"/>
       <c r="AJ30" s="5"/>
     </row>

</xml_diff>

<commit_message>
FIXED DC MOTOR ACTUATOR MAPPING FOR DRV8871!
</commit_message>
<xml_diff>
--- a/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
+++ b/electrical_hardware/APWCR_Electrical_Pin_Connections.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_Software\electrical_hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF016CA9-7DE9-48AF-AF30-7D18E8B444F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29F124FB-5455-443C-9F60-313EE5171528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -220,36 +220,24 @@
     <t>D9</t>
   </si>
   <si>
-    <t>D32</t>
-  </si>
-  <si>
     <t>DRV8871 Motor Driver - RHS Arm Motor</t>
   </si>
   <si>
     <t>D10</t>
   </si>
   <si>
-    <t>D33</t>
-  </si>
-  <si>
     <t>DRV8871 Motor Driver - LHS DRIVE Motor</t>
   </si>
   <si>
     <t>D5</t>
   </si>
   <si>
-    <t>D30</t>
-  </si>
-  <si>
     <t>DRV8871 Motor Driver - RHS DRIVE Motor</t>
   </si>
   <si>
     <t>D6</t>
   </si>
   <si>
-    <t>D31</t>
-  </si>
-  <si>
     <t>4X Quadrature Encoders</t>
   </si>
   <si>
@@ -368,6 +356,18 @@
   </si>
   <si>
     <t>LHS Sweeper Swervo +</t>
+  </si>
+  <si>
+    <t>D11</t>
+  </si>
+  <si>
+    <t>D12</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D13</t>
   </si>
 </sst>
 </file>
@@ -914,7 +914,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1040,63 +1040,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1111,6 +1054,33 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1120,9 +1090,6 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1131,6 +1098,30 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1425,26 +1416,26 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:19" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="75" t="s">
+      <c r="B2" s="89" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="75"/>
-      <c r="I2" s="75"/>
-      <c r="J2" s="75"/>
-      <c r="K2" s="75"/>
-      <c r="L2" s="75"/>
-      <c r="M2" s="75"/>
-      <c r="N2" s="75"/>
-      <c r="O2" s="75"/>
-      <c r="P2" s="75"/>
-      <c r="Q2" s="75"/>
-      <c r="R2" s="75"/>
-      <c r="S2" s="75"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
+      <c r="K2" s="89"/>
+      <c r="L2" s="89"/>
+      <c r="M2" s="89"/>
+      <c r="N2" s="89"/>
+      <c r="O2" s="89"/>
+      <c r="P2" s="89"/>
+      <c r="Q2" s="89"/>
+      <c r="R2" s="89"/>
+      <c r="S2" s="89"/>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B3" s="1"/>
@@ -1469,10 +1460,10 @@
     <row r="4" spans="2:19" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="4"/>
       <c r="E4" s="48" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F4" s="49" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G4" s="54"/>
       <c r="H4" s="54"/>
@@ -1484,7 +1475,7 @@
       <c r="N4" s="54"/>
       <c r="O4" s="54"/>
       <c r="P4" s="49" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="S4" s="5"/>
     </row>
@@ -1538,20 +1529,20 @@
       <c r="D6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="71" t="s">
+      <c r="E6" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="71"/>
-      <c r="I6" s="71"/>
-      <c r="J6" s="71"/>
-      <c r="K6" s="71"/>
-      <c r="L6" s="71"/>
-      <c r="M6" s="71"/>
-      <c r="N6" s="71"/>
-      <c r="O6" s="71"/>
-      <c r="P6" s="71"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="85"/>
+      <c r="H6" s="85"/>
+      <c r="I6" s="85"/>
+      <c r="J6" s="85"/>
+      <c r="K6" s="85"/>
+      <c r="L6" s="85"/>
+      <c r="M6" s="85"/>
+      <c r="N6" s="85"/>
+      <c r="O6" s="85"/>
+      <c r="P6" s="85"/>
       <c r="Q6" s="10" t="s">
         <v>25</v>
       </c>
@@ -1565,18 +1556,18 @@
       <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="71"/>
-      <c r="F7" s="71"/>
-      <c r="G7" s="71"/>
-      <c r="H7" s="71"/>
-      <c r="I7" s="71"/>
-      <c r="J7" s="71"/>
-      <c r="K7" s="71"/>
-      <c r="L7" s="71"/>
-      <c r="M7" s="71"/>
-      <c r="N7" s="71"/>
-      <c r="O7" s="71"/>
-      <c r="P7" s="71"/>
+      <c r="E7" s="85"/>
+      <c r="F7" s="85"/>
+      <c r="G7" s="85"/>
+      <c r="H7" s="85"/>
+      <c r="I7" s="85"/>
+      <c r="J7" s="85"/>
+      <c r="K7" s="85"/>
+      <c r="L7" s="85"/>
+      <c r="M7" s="85"/>
+      <c r="N7" s="85"/>
+      <c r="O7" s="85"/>
+      <c r="P7" s="85"/>
       <c r="Q7" s="10" t="s">
         <v>26</v>
       </c>
@@ -1627,10 +1618,10 @@
     <row r="9" spans="2:19" ht="38.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="4"/>
       <c r="E9" s="50" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F9" s="51" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="G9" s="42" t="s">
         <v>31</v>
@@ -1677,10 +1668,10 @@
       <c r="M11" s="54"/>
       <c r="N11" s="54"/>
       <c r="O11" s="43" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="P11" s="42" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="S11" s="5"/>
     </row>
@@ -1734,20 +1725,20 @@
       <c r="D13" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="72" t="s">
+      <c r="E13" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="72"/>
-      <c r="G13" s="72"/>
-      <c r="H13" s="72"/>
-      <c r="I13" s="72"/>
-      <c r="J13" s="72"/>
-      <c r="K13" s="72"/>
-      <c r="L13" s="72"/>
-      <c r="M13" s="72"/>
-      <c r="N13" s="72"/>
-      <c r="O13" s="72"/>
-      <c r="P13" s="72"/>
+      <c r="F13" s="86"/>
+      <c r="G13" s="86"/>
+      <c r="H13" s="86"/>
+      <c r="I13" s="86"/>
+      <c r="J13" s="86"/>
+      <c r="K13" s="86"/>
+      <c r="L13" s="86"/>
+      <c r="M13" s="86"/>
+      <c r="N13" s="86"/>
+      <c r="O13" s="86"/>
+      <c r="P13" s="86"/>
       <c r="Q13" s="11" t="s">
         <v>25</v>
       </c>
@@ -1761,18 +1752,18 @@
       <c r="D14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="72"/>
-      <c r="F14" s="72"/>
-      <c r="G14" s="72"/>
-      <c r="H14" s="72"/>
-      <c r="I14" s="72"/>
-      <c r="J14" s="72"/>
-      <c r="K14" s="72"/>
-      <c r="L14" s="72"/>
-      <c r="M14" s="72"/>
-      <c r="N14" s="72"/>
-      <c r="O14" s="72"/>
-      <c r="P14" s="72"/>
+      <c r="E14" s="86"/>
+      <c r="F14" s="86"/>
+      <c r="G14" s="86"/>
+      <c r="H14" s="86"/>
+      <c r="I14" s="86"/>
+      <c r="J14" s="86"/>
+      <c r="K14" s="86"/>
+      <c r="L14" s="86"/>
+      <c r="M14" s="86"/>
+      <c r="N14" s="86"/>
+      <c r="O14" s="86"/>
+      <c r="P14" s="86"/>
       <c r="Q14" s="11" t="s">
         <v>26</v>
       </c>
@@ -1829,19 +1820,19 @@
         <v>42</v>
       </c>
       <c r="G16" s="52"/>
-      <c r="H16" s="76"/>
+      <c r="H16" s="52"/>
       <c r="I16" s="52"/>
       <c r="J16" s="52"/>
       <c r="K16" s="42" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="L16" s="43" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="M16" s="52"/>
       <c r="N16" s="52"/>
-      <c r="O16" s="76"/>
-      <c r="P16" s="76"/>
+      <c r="O16" s="52"/>
+      <c r="P16" s="52"/>
       <c r="S16" s="5"/>
     </row>
     <row r="17" spans="2:19" x14ac:dyDescent="0.45">
@@ -1863,10 +1854,10 @@
       <c r="K18" s="53"/>
       <c r="L18" s="53"/>
       <c r="M18" s="47" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="N18" s="46" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="O18" s="47" t="s">
         <v>46</v>
@@ -1926,20 +1917,20 @@
       <c r="D20" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="73" t="s">
+      <c r="E20" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="77"/>
-      <c r="G20" s="77"/>
-      <c r="H20" s="77"/>
-      <c r="I20" s="77"/>
-      <c r="J20" s="77"/>
-      <c r="K20" s="77"/>
-      <c r="L20" s="77"/>
-      <c r="M20" s="77"/>
-      <c r="N20" s="77"/>
-      <c r="O20" s="77"/>
-      <c r="P20" s="74"/>
+      <c r="F20" s="86"/>
+      <c r="G20" s="86"/>
+      <c r="H20" s="86"/>
+      <c r="I20" s="86"/>
+      <c r="J20" s="86"/>
+      <c r="K20" s="86"/>
+      <c r="L20" s="86"/>
+      <c r="M20" s="86"/>
+      <c r="N20" s="86"/>
+      <c r="O20" s="86"/>
+      <c r="P20" s="88"/>
       <c r="Q20" s="11" t="s">
         <v>25</v>
       </c>
@@ -1953,18 +1944,18 @@
       <c r="D21" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="73"/>
-      <c r="F21" s="77"/>
-      <c r="G21" s="77"/>
-      <c r="H21" s="77"/>
-      <c r="I21" s="77"/>
-      <c r="J21" s="77"/>
-      <c r="K21" s="77"/>
-      <c r="L21" s="77"/>
-      <c r="M21" s="77"/>
-      <c r="N21" s="77"/>
-      <c r="O21" s="77"/>
-      <c r="P21" s="74"/>
+      <c r="E21" s="87"/>
+      <c r="F21" s="86"/>
+      <c r="G21" s="86"/>
+      <c r="H21" s="86"/>
+      <c r="I21" s="86"/>
+      <c r="J21" s="86"/>
+      <c r="K21" s="86"/>
+      <c r="L21" s="86"/>
+      <c r="M21" s="86"/>
+      <c r="N21" s="86"/>
+      <c r="O21" s="86"/>
+      <c r="P21" s="88"/>
       <c r="Q21" s="11" t="s">
         <v>26</v>
       </c>
@@ -2093,45 +2084,45 @@
   <sheetData>
     <row r="2" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:42" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B3" s="65" t="s">
-        <v>90</v>
-      </c>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="67"/>
-      <c r="M3" s="65" t="s">
-        <v>74</v>
-      </c>
-      <c r="N3" s="66"/>
-      <c r="O3" s="66"/>
-      <c r="P3" s="66"/>
-      <c r="Q3" s="66"/>
-      <c r="R3" s="66"/>
-      <c r="S3" s="66"/>
-      <c r="T3" s="66"/>
-      <c r="U3" s="66"/>
-      <c r="V3" s="66"/>
-      <c r="W3" s="66"/>
-      <c r="X3" s="66"/>
-      <c r="Y3" s="66"/>
-      <c r="Z3" s="67"/>
-      <c r="AB3" s="65" t="s">
-        <v>91</v>
-      </c>
-      <c r="AC3" s="66"/>
-      <c r="AD3" s="66"/>
-      <c r="AE3" s="66"/>
-      <c r="AF3" s="66"/>
-      <c r="AG3" s="66"/>
-      <c r="AH3" s="66"/>
-      <c r="AI3" s="66"/>
-      <c r="AJ3" s="67"/>
+      <c r="B3" s="73" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="74"/>
+      <c r="J3" s="74"/>
+      <c r="K3" s="75"/>
+      <c r="M3" s="73" t="s">
+        <v>70</v>
+      </c>
+      <c r="N3" s="74"/>
+      <c r="O3" s="74"/>
+      <c r="P3" s="74"/>
+      <c r="Q3" s="74"/>
+      <c r="R3" s="74"/>
+      <c r="S3" s="74"/>
+      <c r="T3" s="74"/>
+      <c r="U3" s="74"/>
+      <c r="V3" s="74"/>
+      <c r="W3" s="74"/>
+      <c r="X3" s="74"/>
+      <c r="Y3" s="74"/>
+      <c r="Z3" s="75"/>
+      <c r="AB3" s="73" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC3" s="74"/>
+      <c r="AD3" s="74"/>
+      <c r="AE3" s="74"/>
+      <c r="AF3" s="74"/>
+      <c r="AG3" s="74"/>
+      <c r="AH3" s="74"/>
+      <c r="AI3" s="74"/>
+      <c r="AJ3" s="75"/>
       <c r="AK3" s="31"/>
       <c r="AL3" s="31"/>
       <c r="AM3" s="31"/>
@@ -2182,12 +2173,12 @@
       <c r="D5" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="62" t="s">
+      <c r="E5" s="70" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
+      <c r="F5" s="70"/>
+      <c r="G5" s="70"/>
+      <c r="H5" s="70"/>
       <c r="I5" s="15" t="s">
         <v>57</v>
       </c>
@@ -2197,42 +2188,42 @@
         <v>29</v>
       </c>
       <c r="O5" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="P5" s="82" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q5" s="82"/>
+      <c r="R5" s="82"/>
+      <c r="S5" s="82"/>
+      <c r="T5" s="82"/>
+      <c r="U5" s="82"/>
+      <c r="V5" s="82"/>
+      <c r="W5" s="82"/>
+      <c r="X5" s="61" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y5" s="20" t="s">
         <v>75</v>
-      </c>
-      <c r="P5" s="68" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q5" s="68"/>
-      <c r="R5" s="68"/>
-      <c r="S5" s="68"/>
-      <c r="T5" s="68"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="68"/>
-      <c r="W5" s="68"/>
-      <c r="X5" s="80" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y5" s="20" t="s">
-        <v>79</v>
       </c>
       <c r="Z5" s="5"/>
       <c r="AB5" s="4"/>
       <c r="AC5" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="AD5" s="81" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE5" s="86" t="s">
-        <v>91</v>
-      </c>
-      <c r="AF5" s="59"/>
-      <c r="AG5" s="87"/>
-      <c r="AH5" s="84" t="s">
-        <v>93</v>
+      <c r="AD5" s="62" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE5" s="76" t="s">
+        <v>87</v>
+      </c>
+      <c r="AF5" s="67"/>
+      <c r="AG5" s="77"/>
+      <c r="AH5" s="65" t="s">
+        <v>89</v>
       </c>
       <c r="AI5" s="35" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="AJ5" s="5"/>
     </row>
@@ -2244,32 +2235,32 @@
       <c r="D6" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
+      <c r="E6" s="71"/>
+      <c r="F6" s="71"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="71"/>
       <c r="I6" s="16" t="s">
         <v>58</v>
       </c>
       <c r="K6" s="5"/>
       <c r="M6" s="4"/>
       <c r="O6" s="26"/>
-      <c r="P6" s="69"/>
-      <c r="Q6" s="69"/>
-      <c r="R6" s="69"/>
-      <c r="S6" s="69"/>
-      <c r="T6" s="69"/>
-      <c r="U6" s="69"/>
-      <c r="V6" s="69"/>
-      <c r="W6" s="69"/>
+      <c r="P6" s="83"/>
+      <c r="Q6" s="83"/>
+      <c r="R6" s="83"/>
+      <c r="S6" s="83"/>
+      <c r="T6" s="83"/>
+      <c r="U6" s="83"/>
+      <c r="V6" s="83"/>
+      <c r="W6" s="83"/>
       <c r="X6" s="27"/>
       <c r="Z6" s="5"/>
       <c r="AB6" s="4"/>
       <c r="AC6" s="37"/>
-      <c r="AD6" s="82"/>
-      <c r="AE6" s="88"/>
-      <c r="AF6" s="89"/>
-      <c r="AG6" s="90"/>
+      <c r="AD6" s="63"/>
+      <c r="AE6" s="78"/>
+      <c r="AF6" s="68"/>
+      <c r="AG6" s="79"/>
       <c r="AH6" s="5"/>
       <c r="AI6" s="36"/>
       <c r="AJ6" s="5"/>
@@ -2277,10 +2268,10 @@
     <row r="7" spans="2:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="4"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
+      <c r="E7" s="71"/>
+      <c r="F7" s="71"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="71"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
       <c r="M7" s="4"/>
@@ -2290,36 +2281,36 @@
       <c r="O7" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P7" s="70"/>
-      <c r="Q7" s="70"/>
-      <c r="R7" s="70"/>
-      <c r="S7" s="70"/>
-      <c r="T7" s="70"/>
-      <c r="U7" s="70"/>
-      <c r="V7" s="70"/>
-      <c r="W7" s="70"/>
+      <c r="P7" s="84"/>
+      <c r="Q7" s="84"/>
+      <c r="R7" s="84"/>
+      <c r="S7" s="84"/>
+      <c r="T7" s="84"/>
+      <c r="U7" s="84"/>
+      <c r="V7" s="84"/>
+      <c r="W7" s="84"/>
       <c r="X7" s="18" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="Y7" s="20" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="Z7" s="5"/>
       <c r="AB7" s="4"/>
       <c r="AC7" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="AD7" s="83" t="s">
+      <c r="AD7" s="64" t="s">
         <v>57</v>
       </c>
-      <c r="AE7" s="91"/>
-      <c r="AF7" s="61"/>
-      <c r="AG7" s="92"/>
-      <c r="AH7" s="85" t="s">
-        <v>94</v>
+      <c r="AE7" s="80"/>
+      <c r="AF7" s="69"/>
+      <c r="AG7" s="81"/>
+      <c r="AH7" s="66" t="s">
+        <v>90</v>
       </c>
       <c r="AI7" s="35" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="AJ7" s="5"/>
     </row>
@@ -2331,15 +2322,15 @@
       <c r="D8" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="63"/>
-      <c r="F8" s="63"/>
-      <c r="G8" s="63"/>
-      <c r="H8" s="63"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="71"/>
+      <c r="G8" s="71"/>
+      <c r="H8" s="71"/>
       <c r="I8" s="17" t="s">
         <v>59</v>
       </c>
       <c r="J8" s="20" t="s">
-        <v>64</v>
+        <v>110</v>
       </c>
       <c r="K8" s="5"/>
       <c r="M8" s="4"/>
@@ -2355,11 +2346,11 @@
       <c r="D9" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="64"/>
-      <c r="F9" s="64"/>
-      <c r="G9" s="64"/>
-      <c r="H9" s="64"/>
-      <c r="I9" s="78" t="s">
+      <c r="E9" s="72"/>
+      <c r="F9" s="72"/>
+      <c r="G9" s="72"/>
+      <c r="H9" s="72"/>
+      <c r="I9" s="59" t="s">
         <v>60</v>
       </c>
       <c r="J9" s="20" t="s">
@@ -2371,23 +2362,23 @@
         <v>29</v>
       </c>
       <c r="O9" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="P9" s="68" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q9" s="68"/>
-      <c r="R9" s="68"/>
-      <c r="S9" s="68"/>
-      <c r="T9" s="68"/>
-      <c r="U9" s="68"/>
-      <c r="V9" s="68"/>
-      <c r="W9" s="68"/>
-      <c r="X9" s="80" t="s">
-        <v>76</v>
+        <v>71</v>
+      </c>
+      <c r="P9" s="82" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q9" s="82"/>
+      <c r="R9" s="82"/>
+      <c r="S9" s="82"/>
+      <c r="T9" s="82"/>
+      <c r="U9" s="82"/>
+      <c r="V9" s="82"/>
+      <c r="W9" s="82"/>
+      <c r="X9" s="61" t="s">
+        <v>72</v>
       </c>
       <c r="Y9" s="20" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="Z9" s="5"/>
       <c r="AB9" s="4"/>
@@ -2398,14 +2389,14 @@
       <c r="K10" s="5"/>
       <c r="M10" s="4"/>
       <c r="O10" s="26"/>
-      <c r="P10" s="69"/>
-      <c r="Q10" s="69"/>
-      <c r="R10" s="69"/>
-      <c r="S10" s="69"/>
-      <c r="T10" s="69"/>
-      <c r="U10" s="69"/>
-      <c r="V10" s="69"/>
-      <c r="W10" s="69"/>
+      <c r="P10" s="83"/>
+      <c r="Q10" s="83"/>
+      <c r="R10" s="83"/>
+      <c r="S10" s="83"/>
+      <c r="T10" s="83"/>
+      <c r="U10" s="83"/>
+      <c r="V10" s="83"/>
+      <c r="W10" s="83"/>
       <c r="X10" s="27"/>
       <c r="Z10" s="5"/>
       <c r="AB10" s="4"/>
@@ -2419,12 +2410,12 @@
       <c r="D11" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="62" t="s">
-        <v>65</v>
-      </c>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62"/>
-      <c r="H11" s="62"/>
+      <c r="E11" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" s="70"/>
+      <c r="G11" s="70"/>
+      <c r="H11" s="70"/>
       <c r="I11" s="15" t="s">
         <v>57</v>
       </c>
@@ -2436,19 +2427,19 @@
       <c r="O11" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P11" s="70"/>
-      <c r="Q11" s="70"/>
-      <c r="R11" s="70"/>
-      <c r="S11" s="70"/>
-      <c r="T11" s="70"/>
-      <c r="U11" s="70"/>
-      <c r="V11" s="70"/>
-      <c r="W11" s="70"/>
+      <c r="P11" s="84"/>
+      <c r="Q11" s="84"/>
+      <c r="R11" s="84"/>
+      <c r="S11" s="84"/>
+      <c r="T11" s="84"/>
+      <c r="U11" s="84"/>
+      <c r="V11" s="84"/>
+      <c r="W11" s="84"/>
       <c r="X11" s="18" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="Y11" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="Z11" s="5"/>
       <c r="AB11" s="4"/>
@@ -2462,10 +2453,10 @@
       <c r="D12" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
-      <c r="G12" s="63"/>
-      <c r="H12" s="63"/>
+      <c r="E12" s="71"/>
+      <c r="F12" s="71"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="71"/>
       <c r="I12" s="16" t="s">
         <v>58</v>
       </c>
@@ -2478,10 +2469,10 @@
     <row r="13" spans="2:42" x14ac:dyDescent="0.45">
       <c r="B13" s="4"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="63"/>
+      <c r="E13" s="71"/>
+      <c r="F13" s="71"/>
+      <c r="G13" s="71"/>
+      <c r="H13" s="71"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
       <c r="M13" s="4"/>
@@ -2489,23 +2480,23 @@
         <v>29</v>
       </c>
       <c r="O13" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="P13" s="68" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q13" s="68"/>
-      <c r="R13" s="68"/>
-      <c r="S13" s="68"/>
-      <c r="T13" s="68"/>
-      <c r="U13" s="68"/>
-      <c r="V13" s="68"/>
-      <c r="W13" s="68"/>
-      <c r="X13" s="80" t="s">
-        <v>76</v>
+        <v>71</v>
+      </c>
+      <c r="P13" s="82" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q13" s="82"/>
+      <c r="R13" s="82"/>
+      <c r="S13" s="82"/>
+      <c r="T13" s="82"/>
+      <c r="U13" s="82"/>
+      <c r="V13" s="82"/>
+      <c r="W13" s="82"/>
+      <c r="X13" s="61" t="s">
+        <v>72</v>
       </c>
       <c r="Y13" s="20" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="Z13" s="5"/>
       <c r="AB13" s="4"/>
@@ -2519,27 +2510,27 @@
       <c r="D14" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
-      <c r="G14" s="63"/>
-      <c r="H14" s="63"/>
+      <c r="E14" s="71"/>
+      <c r="F14" s="71"/>
+      <c r="G14" s="71"/>
+      <c r="H14" s="71"/>
       <c r="I14" s="17" t="s">
         <v>59</v>
       </c>
       <c r="J14" s="20" t="s">
-        <v>67</v>
+        <v>111</v>
       </c>
       <c r="K14" s="5"/>
       <c r="M14" s="4"/>
       <c r="O14" s="26"/>
-      <c r="P14" s="69"/>
-      <c r="Q14" s="69"/>
-      <c r="R14" s="69"/>
-      <c r="S14" s="69"/>
-      <c r="T14" s="69"/>
-      <c r="U14" s="69"/>
-      <c r="V14" s="69"/>
-      <c r="W14" s="69"/>
+      <c r="P14" s="83"/>
+      <c r="Q14" s="83"/>
+      <c r="R14" s="83"/>
+      <c r="S14" s="83"/>
+      <c r="T14" s="83"/>
+      <c r="U14" s="83"/>
+      <c r="V14" s="83"/>
+      <c r="W14" s="83"/>
       <c r="X14" s="27"/>
       <c r="Z14" s="5"/>
       <c r="AB14" s="4"/>
@@ -2553,15 +2544,15 @@
       <c r="D15" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
-      <c r="H15" s="64"/>
-      <c r="I15" s="78" t="s">
+      <c r="E15" s="72"/>
+      <c r="F15" s="72"/>
+      <c r="G15" s="72"/>
+      <c r="H15" s="72"/>
+      <c r="I15" s="59" t="s">
         <v>60</v>
       </c>
       <c r="J15" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K15" s="5"/>
       <c r="M15" s="4"/>
@@ -2571,19 +2562,19 @@
       <c r="O15" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P15" s="70"/>
-      <c r="Q15" s="70"/>
-      <c r="R15" s="70"/>
-      <c r="S15" s="70"/>
-      <c r="T15" s="70"/>
-      <c r="U15" s="70"/>
-      <c r="V15" s="70"/>
-      <c r="W15" s="70"/>
-      <c r="X15" s="79" t="s">
-        <v>77</v>
+      <c r="P15" s="84"/>
+      <c r="Q15" s="84"/>
+      <c r="R15" s="84"/>
+      <c r="S15" s="84"/>
+      <c r="T15" s="84"/>
+      <c r="U15" s="84"/>
+      <c r="V15" s="84"/>
+      <c r="W15" s="84"/>
+      <c r="X15" s="60" t="s">
+        <v>73</v>
       </c>
       <c r="Y15" s="20" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="Z15" s="5"/>
       <c r="AB15" s="4"/>
@@ -2612,12 +2603,12 @@
       <c r="D17" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="62" t="s">
-        <v>68</v>
-      </c>
-      <c r="F17" s="62"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
+      <c r="E17" s="70" t="s">
+        <v>66</v>
+      </c>
+      <c r="F17" s="70"/>
+      <c r="G17" s="70"/>
+      <c r="H17" s="70"/>
       <c r="I17" s="15" t="s">
         <v>57</v>
       </c>
@@ -2627,23 +2618,23 @@
         <v>29</v>
       </c>
       <c r="O17" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="P17" s="68" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q17" s="68"/>
-      <c r="R17" s="68"/>
-      <c r="S17" s="68"/>
-      <c r="T17" s="68"/>
-      <c r="U17" s="68"/>
-      <c r="V17" s="68"/>
-      <c r="W17" s="68"/>
-      <c r="X17" s="80" t="s">
-        <v>76</v>
+        <v>71</v>
+      </c>
+      <c r="P17" s="82" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q17" s="82"/>
+      <c r="R17" s="82"/>
+      <c r="S17" s="82"/>
+      <c r="T17" s="82"/>
+      <c r="U17" s="82"/>
+      <c r="V17" s="82"/>
+      <c r="W17" s="82"/>
+      <c r="X17" s="61" t="s">
+        <v>72</v>
       </c>
       <c r="Y17" s="20" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Z17" s="5"/>
     </row>
@@ -2655,45 +2646,45 @@
       <c r="D18" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="63"/>
+      <c r="E18" s="71"/>
+      <c r="F18" s="71"/>
+      <c r="G18" s="71"/>
+      <c r="H18" s="71"/>
       <c r="I18" s="16" t="s">
         <v>58</v>
       </c>
       <c r="K18" s="5"/>
       <c r="M18" s="4"/>
       <c r="O18" s="26"/>
-      <c r="P18" s="69"/>
-      <c r="Q18" s="69"/>
-      <c r="R18" s="69"/>
-      <c r="S18" s="69"/>
-      <c r="T18" s="69"/>
-      <c r="U18" s="69"/>
-      <c r="V18" s="69"/>
-      <c r="W18" s="69"/>
+      <c r="P18" s="83"/>
+      <c r="Q18" s="83"/>
+      <c r="R18" s="83"/>
+      <c r="S18" s="83"/>
+      <c r="T18" s="83"/>
+      <c r="U18" s="83"/>
+      <c r="V18" s="83"/>
+      <c r="W18" s="83"/>
       <c r="X18" s="27"/>
       <c r="Z18" s="5"/>
-      <c r="AB18" s="65" t="s">
-        <v>98</v>
-      </c>
-      <c r="AC18" s="66"/>
-      <c r="AD18" s="66"/>
-      <c r="AE18" s="66"/>
-      <c r="AF18" s="66"/>
-      <c r="AG18" s="66"/>
-      <c r="AH18" s="66"/>
-      <c r="AI18" s="66"/>
-      <c r="AJ18" s="67"/>
+      <c r="AB18" s="73" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC18" s="74"/>
+      <c r="AD18" s="74"/>
+      <c r="AE18" s="74"/>
+      <c r="AF18" s="74"/>
+      <c r="AG18" s="74"/>
+      <c r="AH18" s="74"/>
+      <c r="AI18" s="74"/>
+      <c r="AJ18" s="75"/>
     </row>
     <row r="19" spans="2:36" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="4"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="63"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="63"/>
-      <c r="H19" s="63"/>
+      <c r="E19" s="71"/>
+      <c r="F19" s="71"/>
+      <c r="G19" s="71"/>
+      <c r="H19" s="71"/>
       <c r="I19" s="5"/>
       <c r="K19" s="5"/>
       <c r="M19" s="4"/>
@@ -2703,19 +2694,19 @@
       <c r="O19" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P19" s="70"/>
-      <c r="Q19" s="70"/>
-      <c r="R19" s="70"/>
-      <c r="S19" s="70"/>
-      <c r="T19" s="70"/>
-      <c r="U19" s="70"/>
-      <c r="V19" s="70"/>
-      <c r="W19" s="70"/>
-      <c r="X19" s="79" t="s">
-        <v>77</v>
+      <c r="P19" s="84"/>
+      <c r="Q19" s="84"/>
+      <c r="R19" s="84"/>
+      <c r="S19" s="84"/>
+      <c r="T19" s="84"/>
+      <c r="U19" s="84"/>
+      <c r="V19" s="84"/>
+      <c r="W19" s="84"/>
+      <c r="X19" s="60" t="s">
+        <v>73</v>
       </c>
       <c r="Y19" s="20" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="Z19" s="5"/>
       <c r="AB19" s="1"/>
@@ -2736,15 +2727,15 @@
       <c r="D20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="63"/>
-      <c r="F20" s="63"/>
-      <c r="G20" s="63"/>
-      <c r="H20" s="63"/>
+      <c r="E20" s="71"/>
+      <c r="F20" s="71"/>
+      <c r="G20" s="71"/>
+      <c r="H20" s="71"/>
       <c r="I20" s="17" t="s">
         <v>59</v>
       </c>
       <c r="J20" s="20" t="s">
-        <v>70</v>
+        <v>112</v>
       </c>
       <c r="K20" s="5"/>
       <c r="M20" s="4"/>
@@ -2754,13 +2745,13 @@
         <v>29</v>
       </c>
       <c r="AD20" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE20" s="59" t="s">
-        <v>95</v>
-      </c>
-      <c r="AF20" s="59"/>
-      <c r="AG20" s="59"/>
+        <v>88</v>
+      </c>
+      <c r="AE20" s="67" t="s">
+        <v>91</v>
+      </c>
+      <c r="AF20" s="67"/>
+      <c r="AG20" s="67"/>
       <c r="AH20" s="3"/>
       <c r="AJ20" s="5"/>
     </row>
@@ -2772,15 +2763,15 @@
       <c r="D21" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="64"/>
-      <c r="F21" s="64"/>
-      <c r="G21" s="64"/>
-      <c r="H21" s="64"/>
-      <c r="I21" s="78" t="s">
+      <c r="E21" s="72"/>
+      <c r="F21" s="72"/>
+      <c r="G21" s="72"/>
+      <c r="H21" s="72"/>
+      <c r="I21" s="59" t="s">
         <v>60</v>
       </c>
       <c r="J21" s="20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K21" s="5"/>
       <c r="M21" s="4"/>
@@ -2788,11 +2779,11 @@
       <c r="AB21" s="4"/>
       <c r="AC21" s="37"/>
       <c r="AD21" s="33"/>
-      <c r="AE21" s="60"/>
-      <c r="AF21" s="60"/>
-      <c r="AG21" s="60"/>
+      <c r="AE21" s="68"/>
+      <c r="AF21" s="68"/>
+      <c r="AG21" s="68"/>
       <c r="AH21" s="39" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="AI21" s="35" t="s">
         <v>1</v>
@@ -2811,9 +2802,9 @@
       <c r="AD22" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="AE22" s="61"/>
-      <c r="AF22" s="61"/>
-      <c r="AG22" s="61"/>
+      <c r="AE22" s="69"/>
+      <c r="AF22" s="69"/>
+      <c r="AG22" s="69"/>
       <c r="AH22" s="8"/>
       <c r="AJ22" s="5"/>
     </row>
@@ -2825,12 +2816,12 @@
       <c r="D23" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="62" t="s">
-        <v>71</v>
-      </c>
-      <c r="F23" s="62"/>
-      <c r="G23" s="62"/>
-      <c r="H23" s="62"/>
+      <c r="E23" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="F23" s="70"/>
+      <c r="G23" s="70"/>
+      <c r="H23" s="70"/>
       <c r="I23" s="15" t="s">
         <v>57</v>
       </c>
@@ -2848,10 +2839,10 @@
       <c r="D24" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="63"/>
-      <c r="F24" s="63"/>
-      <c r="G24" s="63"/>
-      <c r="H24" s="63"/>
+      <c r="E24" s="71"/>
+      <c r="F24" s="71"/>
+      <c r="G24" s="71"/>
+      <c r="H24" s="71"/>
       <c r="I24" s="16" t="s">
         <v>58</v>
       </c>
@@ -2863,23 +2854,23 @@
         <v>29</v>
       </c>
       <c r="AD24" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE24" s="59" t="s">
-        <v>111</v>
-      </c>
-      <c r="AF24" s="59"/>
-      <c r="AG24" s="59"/>
+        <v>88</v>
+      </c>
+      <c r="AE24" s="67" t="s">
+        <v>107</v>
+      </c>
+      <c r="AF24" s="67"/>
+      <c r="AG24" s="67"/>
       <c r="AH24" s="3"/>
       <c r="AJ24" s="5"/>
     </row>
     <row r="25" spans="2:36" ht="19.5" x14ac:dyDescent="0.6">
       <c r="B25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63"/>
-      <c r="G25" s="63"/>
-      <c r="H25" s="63"/>
+      <c r="E25" s="71"/>
+      <c r="F25" s="71"/>
+      <c r="G25" s="71"/>
+      <c r="H25" s="71"/>
       <c r="I25" s="5"/>
       <c r="K25" s="5"/>
       <c r="M25" s="4"/>
@@ -2887,11 +2878,11 @@
       <c r="AB25" s="4"/>
       <c r="AC25" s="37"/>
       <c r="AD25" s="33"/>
-      <c r="AE25" s="60"/>
-      <c r="AF25" s="60"/>
-      <c r="AG25" s="60"/>
+      <c r="AE25" s="68"/>
+      <c r="AF25" s="68"/>
+      <c r="AG25" s="68"/>
       <c r="AH25" s="39" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="AI25" s="35" t="s">
         <v>3</v>
@@ -2906,15 +2897,15 @@
       <c r="D26" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="63"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="63"/>
-      <c r="H26" s="63"/>
+      <c r="E26" s="71"/>
+      <c r="F26" s="71"/>
+      <c r="G26" s="71"/>
+      <c r="H26" s="71"/>
       <c r="I26" s="17" t="s">
         <v>59</v>
       </c>
       <c r="J26" s="20" t="s">
-        <v>73</v>
+        <v>113</v>
       </c>
       <c r="K26" s="5"/>
       <c r="M26" s="4"/>
@@ -2926,9 +2917,9 @@
       <c r="AD26" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="AE26" s="61"/>
-      <c r="AF26" s="61"/>
-      <c r="AG26" s="61"/>
+      <c r="AE26" s="69"/>
+      <c r="AF26" s="69"/>
+      <c r="AG26" s="69"/>
       <c r="AH26" s="8"/>
       <c r="AJ26" s="5"/>
     </row>
@@ -2940,15 +2931,15 @@
       <c r="D27" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="E27" s="64"/>
-      <c r="F27" s="64"/>
-      <c r="G27" s="64"/>
-      <c r="H27" s="64"/>
-      <c r="I27" s="78" t="s">
+      <c r="E27" s="72"/>
+      <c r="F27" s="72"/>
+      <c r="G27" s="72"/>
+      <c r="H27" s="72"/>
+      <c r="I27" s="59" t="s">
         <v>60</v>
       </c>
       <c r="J27" s="20" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="K27" s="5"/>
       <c r="M27" s="4"/>
@@ -2966,13 +2957,13 @@
         <v>29</v>
       </c>
       <c r="AD28" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE28" s="59" t="s">
-        <v>110</v>
-      </c>
-      <c r="AF28" s="59"/>
-      <c r="AG28" s="59"/>
+        <v>88</v>
+      </c>
+      <c r="AE28" s="67" t="s">
+        <v>106</v>
+      </c>
+      <c r="AF28" s="67"/>
+      <c r="AG28" s="67"/>
       <c r="AH28" s="3"/>
       <c r="AJ28" s="5"/>
     </row>
@@ -2984,14 +2975,14 @@
       <c r="AB29" s="4"/>
       <c r="AC29" s="37"/>
       <c r="AD29" s="33"/>
-      <c r="AE29" s="60"/>
-      <c r="AF29" s="60"/>
-      <c r="AG29" s="60"/>
+      <c r="AE29" s="68"/>
+      <c r="AF29" s="68"/>
+      <c r="AG29" s="68"/>
       <c r="AH29" s="39" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="AI29" s="35" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="AJ29" s="5"/>
     </row>
@@ -3007,9 +2998,9 @@
       <c r="AD30" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="AE30" s="61"/>
-      <c r="AF30" s="61"/>
-      <c r="AG30" s="61"/>
+      <c r="AE30" s="69"/>
+      <c r="AF30" s="69"/>
+      <c r="AG30" s="69"/>
       <c r="AH30" s="8"/>
       <c r="AJ30" s="5"/>
     </row>

</xml_diff>